<commit_message>
data: EEX curves refresh (latest trade date 2026-04-20)
</commit_message>
<xml_diff>
--- a/data/EEX_Gas_Curves.xlsx
+++ b/data/EEX_Gas_Curves.xlsx
@@ -526,7 +526,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 21 Apr 2026 08:28  ·  Source: EEX Market Data Hub (public)  ·  EUR/MWh</t>
+          <t>Generated: 21 Apr 2026 13:02  ·  Source: EEX Market Data Hub (public)  ·  EUR/MWh</t>
         </is>
       </c>
     </row>
@@ -587,7 +587,7 @@
         </is>
       </c>
       <c r="F5" s="4" t="n">
-        <v>1008</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="6">
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="F6" s="6" t="n">
-        <v>259</v>
+        <v>267</v>
       </c>
     </row>
     <row r="7">
@@ -643,7 +643,7 @@
         </is>
       </c>
       <c r="F7" s="4" t="n">
-        <v>1104</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="8">
@@ -671,7 +671,7 @@
         </is>
       </c>
       <c r="F8" s="6" t="n">
-        <v>309</v>
+        <v>325</v>
       </c>
     </row>
     <row r="9">
@@ -699,7 +699,7 @@
         </is>
       </c>
       <c r="F9" s="4" t="n">
-        <v>117</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -1554,13 +1554,25 @@
       <c r="P3" s="10" t="n"/>
       <c r="Q3" s="10" t="n"/>
       <c r="R3" s="10" t="n"/>
-      <c r="S3" s="10" t="n"/>
-      <c r="T3" s="10" t="n"/>
-      <c r="U3" s="10" t="n"/>
-      <c r="V3" s="10" t="n"/>
+      <c r="S3" s="10" t="n">
+        <v>33.516</v>
+      </c>
+      <c r="T3" s="10" t="n">
+        <v>33.412</v>
+      </c>
+      <c r="U3" s="10" t="n">
+        <v>33.514</v>
+      </c>
+      <c r="V3" s="10" t="n">
+        <v>33.705</v>
+      </c>
       <c r="W3" s="10" t="n"/>
-      <c r="X3" s="10" t="n"/>
-      <c r="Y3" s="10" t="n"/>
+      <c r="X3" s="10" t="n">
+        <v>34.335</v>
+      </c>
+      <c r="Y3" s="10" t="n">
+        <v>34.826</v>
+      </c>
       <c r="Z3" s="10" t="n"/>
       <c r="AA3" s="10" t="n">
         <v>26.914</v>
@@ -1604,7 +1616,9 @@
       <c r="AN3" s="10" t="n">
         <v>28.281</v>
       </c>
-      <c r="AO3" s="10" t="n"/>
+      <c r="AO3" s="10" t="n">
+        <v>25.326</v>
+      </c>
       <c r="AP3" s="10" t="n">
         <v>24.508</v>
       </c>
@@ -1618,17 +1632,33 @@
       <c r="AX3" s="10" t="n"/>
       <c r="AY3" s="10" t="n"/>
       <c r="AZ3" s="10" t="n"/>
-      <c r="BA3" s="10" t="n"/>
-      <c r="BB3" s="10" t="n"/>
-      <c r="BC3" s="10" t="n"/>
-      <c r="BD3" s="10" t="n"/>
+      <c r="BA3" s="10" t="n">
+        <v>24.414</v>
+      </c>
+      <c r="BB3" s="10" t="n">
+        <v>24.691</v>
+      </c>
+      <c r="BC3" s="10" t="n">
+        <v>24.905</v>
+      </c>
+      <c r="BD3" s="10" t="n">
+        <v>24.555</v>
+      </c>
       <c r="BE3" s="10" t="n"/>
       <c r="BF3" s="10" t="n"/>
       <c r="BG3" s="10" t="n"/>
-      <c r="BH3" s="10" t="n"/>
-      <c r="BI3" s="10" t="n"/>
-      <c r="BJ3" s="10" t="n"/>
-      <c r="BK3" s="10" t="n"/>
+      <c r="BH3" s="10" t="n">
+        <v>25.785</v>
+      </c>
+      <c r="BI3" s="10" t="n">
+        <v>25.373</v>
+      </c>
+      <c r="BJ3" s="10" t="n">
+        <v>25.551</v>
+      </c>
+      <c r="BK3" s="10" t="n">
+        <v>25.115</v>
+      </c>
       <c r="BL3" s="10" t="n">
         <v>24.834</v>
       </c>
@@ -1646,7 +1676,9 @@
       <c r="BR3" s="10" t="n">
         <v>24.663</v>
       </c>
-      <c r="BS3" s="10" t="n"/>
+      <c r="BS3" s="10" t="n">
+        <v>24.989</v>
+      </c>
       <c r="BT3" s="10" t="n"/>
       <c r="BU3" s="10" t="n"/>
       <c r="BV3" s="10" t="n">
@@ -1671,17 +1703,31 @@
       <c r="CE3" s="10" t="n"/>
       <c r="CF3" s="10" t="n"/>
       <c r="CG3" s="10" t="n"/>
-      <c r="CH3" s="10" t="n"/>
+      <c r="CH3" s="10" t="n">
+        <v>25.915</v>
+      </c>
       <c r="CI3" s="10" t="n"/>
       <c r="CJ3" s="10" t="n"/>
       <c r="CK3" s="10" t="n"/>
-      <c r="CL3" s="10" t="n"/>
-      <c r="CM3" s="10" t="n"/>
-      <c r="CN3" s="10" t="n"/>
-      <c r="CO3" s="10" t="n"/>
+      <c r="CL3" s="10" t="n">
+        <v>25.796</v>
+      </c>
+      <c r="CM3" s="10" t="n">
+        <v>25.316</v>
+      </c>
+      <c r="CN3" s="10" t="n">
+        <v>24.905</v>
+      </c>
+      <c r="CO3" s="10" t="n">
+        <v>24.286</v>
+      </c>
       <c r="CP3" s="10" t="n"/>
-      <c r="CQ3" s="10" t="n"/>
-      <c r="CR3" s="10" t="n"/>
+      <c r="CQ3" s="10" t="n">
+        <v>24.783</v>
+      </c>
+      <c r="CR3" s="10" t="n">
+        <v>24.753</v>
+      </c>
       <c r="CS3" s="10" t="n"/>
       <c r="CT3" s="10" t="n">
         <v>27.166</v>
@@ -1725,12 +1771,20 @@
       <c r="DK3" s="10" t="n"/>
       <c r="DL3" s="10" t="n"/>
       <c r="DM3" s="10" t="n"/>
-      <c r="DN3" s="10" t="n"/>
-      <c r="DO3" s="10" t="n"/>
+      <c r="DN3" s="10" t="n">
+        <v>25.166</v>
+      </c>
+      <c r="DO3" s="10" t="n">
+        <v>23.248</v>
+      </c>
       <c r="DP3" s="10" t="n"/>
       <c r="DQ3" s="10" t="n"/>
-      <c r="DR3" s="10" t="n"/>
-      <c r="DS3" s="10" t="n"/>
+      <c r="DR3" s="10" t="n">
+        <v>25.153</v>
+      </c>
+      <c r="DS3" s="10" t="n">
+        <v>24.838</v>
+      </c>
       <c r="DT3" s="10" t="n"/>
       <c r="DU3" s="10" t="n">
         <v>26.762</v>
@@ -5145,7 +5199,9 @@
           <t>20 Apr 2026</t>
         </is>
       </c>
-      <c r="B3" s="10" t="n"/>
+      <c r="B3" s="10" t="n">
+        <v>40.802</v>
+      </c>
       <c r="C3" s="10" t="n">
         <v>42.098</v>
       </c>
@@ -5174,7 +5230,9 @@
         <v>35.561</v>
       </c>
       <c r="L3" s="10" t="n"/>
-      <c r="M3" s="10" t="n"/>
+      <c r="M3" s="10" t="n">
+        <v>33.004</v>
+      </c>
       <c r="N3" s="10" t="n">
         <v>39.97</v>
       </c>
@@ -5225,15 +5283,27 @@
         <v>40.376</v>
       </c>
       <c r="AG3" s="10" t="n">
-        <v>34.731</v>
-      </c>
-      <c r="AH3" s="10" t="n"/>
+        <v>40.376</v>
+      </c>
+      <c r="AH3" s="10" t="n">
+        <v>33.842</v>
+      </c>
       <c r="AI3" s="10" t="n"/>
-      <c r="AJ3" s="10" t="n"/>
-      <c r="AK3" s="10" t="n"/>
-      <c r="AL3" s="10" t="n"/>
-      <c r="AM3" s="10" t="n"/>
-      <c r="AN3" s="10" t="n"/>
+      <c r="AJ3" s="10" t="n">
+        <v>32.612</v>
+      </c>
+      <c r="AK3" s="10" t="n">
+        <v>27.755</v>
+      </c>
+      <c r="AL3" s="10" t="n">
+        <v>26.442</v>
+      </c>
+      <c r="AM3" s="10" t="n">
+        <v>26.966</v>
+      </c>
+      <c r="AN3" s="10" t="n">
+        <v>28.43</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
@@ -6925,24 +6995,46 @@
           <t>20 Apr 2026</t>
         </is>
       </c>
-      <c r="B3" s="10" t="n"/>
+      <c r="B3" s="10" t="n">
+        <v>38.394</v>
+      </c>
       <c r="C3" s="10" t="n">
         <v>39.501</v>
       </c>
-      <c r="D3" s="10" t="n"/>
-      <c r="E3" s="10" t="n"/>
-      <c r="F3" s="10" t="n"/>
-      <c r="G3" s="10" t="n"/>
-      <c r="H3" s="10" t="n"/>
-      <c r="I3" s="10" t="n"/>
+      <c r="D3" s="10" t="n">
+        <v>39.556</v>
+      </c>
+      <c r="E3" s="10" t="n">
+        <v>39.586</v>
+      </c>
+      <c r="F3" s="10" t="n">
+        <v>39.517</v>
+      </c>
+      <c r="G3" s="10" t="n">
+        <v>39.397</v>
+      </c>
+      <c r="H3" s="10" t="n">
+        <v>38.758</v>
+      </c>
+      <c r="I3" s="10" t="n">
+        <v>38.576</v>
+      </c>
       <c r="J3" s="10" t="n"/>
       <c r="K3" s="10" t="n">
         <v>33.251</v>
       </c>
-      <c r="L3" s="10" t="n"/>
-      <c r="M3" s="10" t="n"/>
-      <c r="N3" s="10" t="n"/>
-      <c r="O3" s="10" t="n"/>
+      <c r="L3" s="10" t="n">
+        <v>31.788</v>
+      </c>
+      <c r="M3" s="10" t="n">
+        <v>30.792</v>
+      </c>
+      <c r="N3" s="10" t="n">
+        <v>38.296</v>
+      </c>
+      <c r="O3" s="10" t="n">
+        <v>38.35</v>
+      </c>
       <c r="P3" s="10" t="n">
         <v>37.895</v>
       </c>
@@ -6974,9 +7066,15 @@
       <c r="Z3" s="10" t="n">
         <v>26.223</v>
       </c>
-      <c r="AA3" s="10" t="n"/>
-      <c r="AB3" s="10" t="n"/>
-      <c r="AC3" s="10" t="n"/>
+      <c r="AA3" s="10" t="n">
+        <v>24.835</v>
+      </c>
+      <c r="AB3" s="10" t="n">
+        <v>25.347</v>
+      </c>
+      <c r="AC3" s="10" t="n">
+        <v>30.904</v>
+      </c>
       <c r="AD3" s="10" t="n">
         <v>30.142</v>
       </c>
@@ -6986,18 +7084,34 @@
       <c r="AF3" s="10" t="n">
         <v>26.026</v>
       </c>
-      <c r="AG3" s="10" t="n"/>
-      <c r="AH3" s="10" t="n"/>
-      <c r="AI3" s="10" t="n"/>
-      <c r="AJ3" s="10" t="n"/>
-      <c r="AK3" s="10" t="n"/>
-      <c r="AL3" s="10" t="n"/>
+      <c r="AG3" s="10" t="n">
+        <v>25.593</v>
+      </c>
+      <c r="AH3" s="10" t="n">
+        <v>24.944</v>
+      </c>
+      <c r="AI3" s="10" t="n">
+        <v>24.06</v>
+      </c>
+      <c r="AJ3" s="10" t="n">
+        <v>24.136</v>
+      </c>
+      <c r="AK3" s="10" t="n">
+        <v>24.274</v>
+      </c>
+      <c r="AL3" s="10" t="n">
+        <v>24.741</v>
+      </c>
       <c r="AM3" s="10" t="n"/>
-      <c r="AN3" s="10" t="n"/>
+      <c r="AN3" s="10" t="n">
+        <v>25.258</v>
+      </c>
       <c r="AO3" s="10" t="n">
         <v>23.166</v>
       </c>
-      <c r="AP3" s="10" t="n"/>
+      <c r="AP3" s="10" t="n">
+        <v>21.946</v>
+      </c>
       <c r="AQ3" s="10" t="n"/>
       <c r="AR3" s="10" t="n"/>
       <c r="AS3" s="10" t="n"/>
@@ -7051,18 +7165,30 @@
       <c r="BO3" s="10" t="n">
         <v>20.752</v>
       </c>
-      <c r="BP3" s="10" t="n"/>
-      <c r="BQ3" s="10" t="n"/>
-      <c r="BR3" s="10" t="n"/>
+      <c r="BP3" s="10" t="n">
+        <v>22.361</v>
+      </c>
+      <c r="BQ3" s="10" t="n">
+        <v>23.381</v>
+      </c>
+      <c r="BR3" s="10" t="n">
+        <v>23.486</v>
+      </c>
       <c r="BS3" s="10" t="n">
         <v>22.791</v>
       </c>
       <c r="BT3" s="10" t="n"/>
       <c r="BU3" s="10" t="n"/>
-      <c r="BV3" s="10" t="n"/>
-      <c r="BW3" s="10" t="n"/>
+      <c r="BV3" s="10" t="n">
+        <v>23.487</v>
+      </c>
+      <c r="BW3" s="10" t="n">
+        <v>22.913</v>
+      </c>
       <c r="BX3" s="10" t="n"/>
-      <c r="BY3" s="10" t="n"/>
+      <c r="BY3" s="10" t="n">
+        <v>22.712</v>
+      </c>
       <c r="BZ3" s="10" t="n"/>
       <c r="CA3" s="10" t="n"/>
       <c r="CB3" s="10" t="n"/>
@@ -7103,20 +7229,36 @@
       <c r="CS3" s="10" t="n">
         <v>23.254</v>
       </c>
-      <c r="CT3" s="10" t="n"/>
+      <c r="CT3" s="10" t="n">
+        <v>23.493</v>
+      </c>
       <c r="CU3" s="10" t="n">
         <v>23.676</v>
       </c>
       <c r="CV3" s="10" t="n">
         <v>25.864</v>
       </c>
-      <c r="CW3" s="10" t="n"/>
-      <c r="CX3" s="10" t="n"/>
-      <c r="CY3" s="10" t="n"/>
-      <c r="CZ3" s="10" t="n"/>
-      <c r="DA3" s="10" t="n"/>
-      <c r="DB3" s="10" t="n"/>
-      <c r="DC3" s="10" t="n"/>
+      <c r="CW3" s="10" t="n">
+        <v>25.741</v>
+      </c>
+      <c r="CX3" s="10" t="n">
+        <v>24.909</v>
+      </c>
+      <c r="CY3" s="10" t="n">
+        <v>39.501</v>
+      </c>
+      <c r="CZ3" s="10" t="n">
+        <v>38.608</v>
+      </c>
+      <c r="DA3" s="10" t="n">
+        <v>38.175</v>
+      </c>
+      <c r="DB3" s="10" t="n">
+        <v>32.283</v>
+      </c>
+      <c r="DC3" s="10" t="n">
+        <v>31.299</v>
+      </c>
       <c r="DD3" s="10" t="n"/>
       <c r="DE3" s="10" t="n"/>
       <c r="DF3" s="10" t="n"/>
@@ -7154,7 +7296,9 @@
       <c r="DT3" s="10" t="n">
         <v>23.615</v>
       </c>
-      <c r="DU3" s="10" t="n"/>
+      <c r="DU3" s="10" t="n">
+        <v>24.878</v>
+      </c>
       <c r="DV3" s="10" t="n">
         <v>23.608</v>
       </c>
@@ -7162,7 +7306,9 @@
         <v>23.707</v>
       </c>
       <c r="DX3" s="10" t="n"/>
-      <c r="DY3" s="10" t="n"/>
+      <c r="DY3" s="10" t="n">
+        <v>25.497</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
@@ -10491,7 +10637,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN12"/>
+  <dimension ref="A1:AO12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -10534,6 +10680,7 @@
     <col width="10" customWidth="1" min="38" max="38"/>
     <col width="10" customWidth="1" min="39" max="39"/>
     <col width="10" customWidth="1" min="40" max="40"/>
+    <col width="10" customWidth="1" min="41" max="41"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -10666,80 +10813,85 @@
       </c>
       <c r="Y2" s="3" t="inlineStr">
         <is>
+          <t>Sum-30</t>
+        </is>
+      </c>
+      <c r="Z2" s="3" t="inlineStr">
+        <is>
           <t>Win-30</t>
         </is>
       </c>
-      <c r="Z2" s="3" t="inlineStr">
+      <c r="AA2" s="3" t="inlineStr">
         <is>
           <t>Cal-31</t>
         </is>
       </c>
-      <c r="AA2" s="3" t="inlineStr">
+      <c r="AB2" s="3" t="inlineStr">
         <is>
           <t>Sum-31</t>
         </is>
       </c>
-      <c r="AB2" s="3" t="inlineStr">
+      <c r="AC2" s="3" t="inlineStr">
         <is>
           <t>Win-31</t>
         </is>
       </c>
-      <c r="AC2" s="3" t="inlineStr">
+      <c r="AD2" s="3" t="inlineStr">
         <is>
           <t>Cal-32</t>
         </is>
       </c>
-      <c r="AD2" s="3" t="inlineStr">
+      <c r="AE2" s="3" t="inlineStr">
         <is>
           <t>2026-03</t>
         </is>
       </c>
-      <c r="AE2" s="3" t="inlineStr">
+      <c r="AF2" s="3" t="inlineStr">
         <is>
           <t>2026-04</t>
         </is>
       </c>
-      <c r="AF2" s="3" t="inlineStr">
+      <c r="AG2" s="3" t="inlineStr">
         <is>
           <t>2027-01</t>
         </is>
       </c>
-      <c r="AG2" s="3" t="inlineStr">
+      <c r="AH2" s="3" t="inlineStr">
         <is>
           <t>2027-02</t>
         </is>
       </c>
-      <c r="AH2" s="3" t="inlineStr">
+      <c r="AI2" s="3" t="inlineStr">
         <is>
           <t>2027-03</t>
         </is>
       </c>
-      <c r="AI2" s="3" t="inlineStr">
+      <c r="AJ2" s="3" t="inlineStr">
         <is>
           <t>2027-04</t>
         </is>
       </c>
-      <c r="AJ2" s="3" t="inlineStr">
+      <c r="AK2" s="3" t="inlineStr">
         <is>
           <t>2028-01</t>
         </is>
       </c>
-      <c r="AK2" s="3" t="inlineStr">
+      <c r="AL2" s="3" t="inlineStr">
         <is>
           <t>2028-02</t>
         </is>
       </c>
-      <c r="AL2" s="3" t="inlineStr">
+      <c r="AM2" s="3" t="inlineStr">
         <is>
           <t>2028-03</t>
         </is>
       </c>
-      <c r="AM2" s="3" t="inlineStr">
+      <c r="AN2" s="3" t="inlineStr">
         <is>
           <t>2028-04</t>
         </is>
       </c>
-      <c r="AN2" s="3" t="inlineStr">
+      <c r="AO2" s="3" t="inlineStr">
         <is>
           <t>2029-01</t>
         </is>
@@ -10766,62 +10918,95 @@
       <c r="F3" s="10" t="n">
         <v>39.78</v>
       </c>
-      <c r="G3" s="10" t="n"/>
-      <c r="H3" s="10" t="n"/>
-      <c r="I3" s="10" t="n"/>
-      <c r="J3" s="10" t="n"/>
-      <c r="K3" s="10" t="n"/>
+      <c r="G3" s="10" t="n">
+        <v>39.623</v>
+      </c>
+      <c r="H3" s="10" t="n">
+        <v>38.782</v>
+      </c>
+      <c r="I3" s="10" t="n">
+        <v>38.863</v>
+      </c>
+      <c r="J3" s="10" t="n">
+        <v>40.241</v>
+      </c>
+      <c r="K3" s="10" t="n">
+        <v>33.16</v>
+      </c>
       <c r="L3" s="10" t="n"/>
       <c r="M3" s="10" t="n"/>
-      <c r="N3" s="10" t="n"/>
-      <c r="O3" s="10" t="n"/>
-      <c r="P3" s="10" t="n"/>
-      <c r="Q3" s="10" t="n"/>
-      <c r="R3" s="10" t="n"/>
+      <c r="N3" s="10" t="n">
+        <v>39.493</v>
+      </c>
+      <c r="O3" s="10" t="n">
+        <v>40.151</v>
+      </c>
+      <c r="P3" s="10" t="n">
+        <v>34.864</v>
+      </c>
+      <c r="Q3" s="10" t="n">
+        <v>33.425</v>
+      </c>
+      <c r="R3" s="10" t="n">
+        <v>26.31</v>
+      </c>
       <c r="S3" s="10" t="n"/>
       <c r="T3" s="10" t="n"/>
       <c r="U3" s="10" t="n"/>
-      <c r="V3" s="10" t="n"/>
+      <c r="V3" s="10" t="n">
+        <v>21.599</v>
+      </c>
       <c r="W3" s="10" t="n"/>
-      <c r="X3" s="10" t="n"/>
-      <c r="Y3" s="10" t="n"/>
+      <c r="X3" s="10" t="n">
+        <v>22.549</v>
+      </c>
+      <c r="Y3" s="10" t="n">
+        <v>20.723</v>
+      </c>
       <c r="Z3" s="10" t="n">
+        <v>22.309</v>
+      </c>
+      <c r="AA3" s="10" t="n">
         <v>23.235</v>
       </c>
-      <c r="AA3" s="10" t="n"/>
-      <c r="AB3" s="10" t="n"/>
+      <c r="AB3" s="10" t="n">
+        <v>21.331</v>
+      </c>
       <c r="AC3" s="10" t="n">
+        <v>24.349</v>
+      </c>
+      <c r="AD3" s="10" t="n">
         <v>24.315</v>
       </c>
-      <c r="AD3" s="10" t="n">
+      <c r="AE3" s="10" t="n">
         <v>39.832</v>
       </c>
-      <c r="AE3" s="10" t="n">
+      <c r="AF3" s="10" t="n">
         <v>39.3</v>
       </c>
-      <c r="AF3" s="10" t="n">
+      <c r="AG3" s="10" t="n">
         <v>38.103</v>
       </c>
-      <c r="AG3" s="10" t="n">
+      <c r="AH3" s="10" t="n">
         <v>31.665</v>
       </c>
-      <c r="AH3" s="10" t="n">
+      <c r="AI3" s="10" t="n">
         <v>31.929</v>
       </c>
-      <c r="AI3" s="10" t="n">
+      <c r="AJ3" s="10" t="n">
         <v>31.035</v>
       </c>
-      <c r="AJ3" s="10" t="n"/>
-      <c r="AK3" s="10" t="n">
+      <c r="AK3" s="10" t="n"/>
+      <c r="AL3" s="10" t="n">
         <v>24.05</v>
       </c>
-      <c r="AL3" s="10" t="n">
+      <c r="AM3" s="10" t="n">
         <v>25.812</v>
       </c>
-      <c r="AM3" s="10" t="n">
+      <c r="AN3" s="10" t="n">
         <v>25.777</v>
       </c>
-      <c r="AN3" s="10" t="n">
+      <c r="AO3" s="10" t="n">
         <v>24.937</v>
       </c>
     </row>
@@ -10887,45 +11072,46 @@
         <v>22.474</v>
       </c>
       <c r="Y4" s="12" t="n"/>
-      <c r="Z4" s="12" t="n">
+      <c r="Z4" s="12" t="n"/>
+      <c r="AA4" s="12" t="n">
         <v>23.36</v>
       </c>
-      <c r="AA4" s="12" t="n"/>
       <c r="AB4" s="12" t="n"/>
-      <c r="AC4" s="12" t="n">
+      <c r="AC4" s="12" t="n"/>
+      <c r="AD4" s="12" t="n">
         <v>24.4</v>
       </c>
-      <c r="AD4" s="12" t="n">
+      <c r="AE4" s="12" t="n">
         <v>38.24</v>
       </c>
-      <c r="AE4" s="12" t="n">
+      <c r="AF4" s="12" t="n">
         <v>38.055</v>
       </c>
-      <c r="AF4" s="12" t="n">
+      <c r="AG4" s="12" t="n">
         <v>37.163</v>
       </c>
-      <c r="AG4" s="12" t="n">
+      <c r="AH4" s="12" t="n">
         <v>30.898</v>
       </c>
-      <c r="AH4" s="12" t="n">
+      <c r="AI4" s="12" t="n">
         <v>31.457</v>
       </c>
-      <c r="AI4" s="12" t="n">
+      <c r="AJ4" s="12" t="n">
         <v>30.429</v>
       </c>
-      <c r="AJ4" s="12" t="n">
+      <c r="AK4" s="12" t="n">
         <v>28.948</v>
       </c>
-      <c r="AK4" s="12" t="n">
+      <c r="AL4" s="12" t="n">
         <v>23.615</v>
       </c>
-      <c r="AL4" s="12" t="n">
+      <c r="AM4" s="12" t="n">
         <v>25.387</v>
       </c>
-      <c r="AM4" s="12" t="n">
+      <c r="AN4" s="12" t="n">
         <v>25.341</v>
       </c>
-      <c r="AN4" s="12" t="n">
+      <c r="AO4" s="12" t="n">
         <v>24.425</v>
       </c>
     </row>
@@ -10995,45 +11181,46 @@
         <v>22.974</v>
       </c>
       <c r="Y5" s="10" t="n"/>
-      <c r="Z5" s="10" t="n">
+      <c r="Z5" s="10" t="n"/>
+      <c r="AA5" s="10" t="n">
         <v>23.36</v>
       </c>
-      <c r="AA5" s="10" t="n"/>
       <c r="AB5" s="10" t="n"/>
-      <c r="AC5" s="10" t="n">
+      <c r="AC5" s="10" t="n"/>
+      <c r="AD5" s="10" t="n">
         <v>24.4</v>
       </c>
-      <c r="AD5" s="10" t="n">
+      <c r="AE5" s="10" t="n">
         <v>41.975</v>
       </c>
-      <c r="AE5" s="10" t="n">
+      <c r="AF5" s="10" t="n">
         <v>41.17</v>
       </c>
-      <c r="AF5" s="10" t="n">
+      <c r="AG5" s="10" t="n">
         <v>39.953</v>
       </c>
-      <c r="AG5" s="10" t="n">
+      <c r="AH5" s="10" t="n">
         <v>32.857</v>
       </c>
-      <c r="AH5" s="10" t="n">
+      <c r="AI5" s="10" t="n">
         <v>32.849</v>
       </c>
-      <c r="AI5" s="10" t="n">
+      <c r="AJ5" s="10" t="n">
         <v>31.81</v>
       </c>
-      <c r="AJ5" s="10" t="n">
+      <c r="AK5" s="10" t="n">
         <v>30.228</v>
       </c>
-      <c r="AK5" s="10" t="n">
+      <c r="AL5" s="10" t="n">
         <v>24.093</v>
       </c>
-      <c r="AL5" s="10" t="n">
+      <c r="AM5" s="10" t="n">
         <v>26.169</v>
       </c>
-      <c r="AM5" s="10" t="n">
+      <c r="AN5" s="10" t="n">
         <v>26.105</v>
       </c>
-      <c r="AN5" s="10" t="n">
+      <c r="AO5" s="10" t="n">
         <v>25.407</v>
       </c>
     </row>
@@ -11106,52 +11293,53 @@
       <c r="X6" s="12" t="n">
         <v>22.724</v>
       </c>
-      <c r="Y6" s="12" t="n">
+      <c r="Y6" s="12" t="n"/>
+      <c r="Z6" s="12" t="n">
         <v>22.467</v>
       </c>
-      <c r="Z6" s="12" t="n">
+      <c r="AA6" s="12" t="n">
         <v>23.61</v>
       </c>
-      <c r="AA6" s="12" t="n">
+      <c r="AB6" s="12" t="n">
         <v>21.797</v>
       </c>
-      <c r="AB6" s="12" t="n">
+      <c r="AC6" s="12" t="n">
         <v>24.609</v>
       </c>
-      <c r="AC6" s="12" t="n">
+      <c r="AD6" s="12" t="n">
         <v>24.4</v>
       </c>
-      <c r="AD6" s="12" t="n">
+      <c r="AE6" s="12" t="n">
         <v>40.793</v>
       </c>
-      <c r="AE6" s="12" t="n">
+      <c r="AF6" s="12" t="n">
         <v>40.037</v>
       </c>
-      <c r="AF6" s="12" t="n">
+      <c r="AG6" s="12" t="n">
         <v>38.896</v>
       </c>
-      <c r="AG6" s="12" t="n">
+      <c r="AH6" s="12" t="n">
         <v>31.781</v>
       </c>
-      <c r="AH6" s="12" t="n">
+      <c r="AI6" s="12" t="n">
         <v>31.873</v>
       </c>
-      <c r="AI6" s="12" t="n">
+      <c r="AJ6" s="12" t="n">
         <v>30.578</v>
       </c>
-      <c r="AJ6" s="12" t="n">
+      <c r="AK6" s="12" t="n">
         <v>28.997</v>
       </c>
-      <c r="AK6" s="12" t="n">
+      <c r="AL6" s="12" t="n">
         <v>23.844</v>
       </c>
-      <c r="AL6" s="12" t="n">
+      <c r="AM6" s="12" t="n">
         <v>25.924</v>
       </c>
-      <c r="AM6" s="12" t="n">
+      <c r="AN6" s="12" t="n">
         <v>25.894</v>
       </c>
-      <c r="AN6" s="12" t="n">
+      <c r="AO6" s="12" t="n">
         <v>24.754</v>
       </c>
     </row>
@@ -11226,52 +11414,53 @@
       <c r="X7" s="10" t="n">
         <v>22.724</v>
       </c>
-      <c r="Y7" s="10" t="n">
+      <c r="Y7" s="10" t="n"/>
+      <c r="Z7" s="10" t="n">
         <v>22.286</v>
       </c>
-      <c r="Z7" s="10" t="n">
+      <c r="AA7" s="10" t="n">
         <v>23.36</v>
       </c>
-      <c r="AA7" s="10" t="n">
+      <c r="AB7" s="10" t="n">
         <v>21.467</v>
       </c>
-      <c r="AB7" s="10" t="n">
+      <c r="AC7" s="10" t="n">
         <v>24.513</v>
       </c>
-      <c r="AC7" s="10" t="n">
+      <c r="AD7" s="10" t="n">
         <v>24.4</v>
       </c>
-      <c r="AD7" s="10" t="n">
+      <c r="AE7" s="10" t="n">
         <v>42.542</v>
       </c>
-      <c r="AE7" s="10" t="n">
+      <c r="AF7" s="10" t="n">
         <v>41.813</v>
       </c>
-      <c r="AF7" s="10" t="n">
+      <c r="AG7" s="10" t="n">
         <v>39.948</v>
       </c>
-      <c r="AG7" s="10" t="n">
+      <c r="AH7" s="10" t="n">
         <v>32.22</v>
       </c>
-      <c r="AH7" s="10" t="n">
+      <c r="AI7" s="10" t="n">
         <v>32.237</v>
       </c>
-      <c r="AI7" s="10" t="n">
+      <c r="AJ7" s="10" t="n">
         <v>31.455</v>
       </c>
-      <c r="AJ7" s="10" t="n">
+      <c r="AK7" s="10" t="n">
         <v>29.474</v>
       </c>
-      <c r="AK7" s="10" t="n">
+      <c r="AL7" s="10" t="n">
         <v>23.697</v>
       </c>
-      <c r="AL7" s="10" t="n">
+      <c r="AM7" s="10" t="n">
         <v>25.779</v>
       </c>
-      <c r="AM7" s="10" t="n">
+      <c r="AN7" s="10" t="n">
         <v>25.861</v>
       </c>
-      <c r="AN7" s="10" t="n">
+      <c r="AO7" s="10" t="n">
         <v>24.615</v>
       </c>
     </row>
@@ -11350,52 +11539,53 @@
       <c r="X8" s="12" t="n">
         <v>22.974</v>
       </c>
-      <c r="Y8" s="12" t="n">
+      <c r="Y8" s="12" t="n"/>
+      <c r="Z8" s="12" t="n">
         <v>22.928</v>
       </c>
-      <c r="Z8" s="12" t="n">
+      <c r="AA8" s="12" t="n">
         <v>23.11</v>
       </c>
-      <c r="AA8" s="12" t="n">
+      <c r="AB8" s="12" t="n">
         <v>21.131</v>
       </c>
-      <c r="AB8" s="12" t="n">
+      <c r="AC8" s="12" t="n">
         <v>24.232</v>
       </c>
-      <c r="AC8" s="12" t="n">
+      <c r="AD8" s="12" t="n">
         <v>24.3</v>
       </c>
-      <c r="AD8" s="12" t="n">
+      <c r="AE8" s="12" t="n">
         <v>45.351</v>
       </c>
-      <c r="AE8" s="12" t="n">
+      <c r="AF8" s="12" t="n">
         <v>44.898</v>
       </c>
-      <c r="AF8" s="12" t="n">
+      <c r="AG8" s="12" t="n">
         <v>42.498</v>
       </c>
-      <c r="AG8" s="12" t="n">
+      <c r="AH8" s="12" t="n">
         <v>33.856</v>
       </c>
-      <c r="AH8" s="12" t="n">
+      <c r="AI8" s="12" t="n">
         <v>33.89</v>
       </c>
-      <c r="AI8" s="12" t="n">
+      <c r="AJ8" s="12" t="n">
         <v>33.025</v>
       </c>
-      <c r="AJ8" s="12" t="n">
+      <c r="AK8" s="12" t="n">
         <v>30.71</v>
       </c>
-      <c r="AK8" s="12" t="n">
+      <c r="AL8" s="12" t="n">
         <v>24.181</v>
       </c>
-      <c r="AL8" s="12" t="n">
+      <c r="AM8" s="12" t="n">
         <v>26.259</v>
       </c>
-      <c r="AM8" s="12" t="n">
+      <c r="AN8" s="12" t="n">
         <v>26.264</v>
       </c>
-      <c r="AN8" s="12" t="n">
+      <c r="AO8" s="12" t="n">
         <v>24.94</v>
       </c>
     </row>
@@ -11463,45 +11653,46 @@
         <v>22.819</v>
       </c>
       <c r="Y9" s="10" t="n"/>
-      <c r="Z9" s="10" t="n">
+      <c r="Z9" s="10" t="n"/>
+      <c r="AA9" s="10" t="n">
         <v>23.11</v>
       </c>
-      <c r="AA9" s="10" t="n"/>
       <c r="AB9" s="10" t="n"/>
-      <c r="AC9" s="10" t="n">
+      <c r="AC9" s="10" t="n"/>
+      <c r="AD9" s="10" t="n">
         <v>24.3</v>
       </c>
-      <c r="AD9" s="10" t="n">
+      <c r="AE9" s="10" t="n">
         <v>43.051</v>
       </c>
-      <c r="AE9" s="10" t="n">
+      <c r="AF9" s="10" t="n">
         <v>42.82</v>
       </c>
-      <c r="AF9" s="10" t="n">
+      <c r="AG9" s="10" t="n">
         <v>40.705</v>
       </c>
-      <c r="AG9" s="10" t="n">
+      <c r="AH9" s="10" t="n">
         <v>32.478</v>
       </c>
-      <c r="AH9" s="10" t="n">
+      <c r="AI9" s="10" t="n">
         <v>33.379</v>
       </c>
-      <c r="AI9" s="10" t="n">
+      <c r="AJ9" s="10" t="n">
         <v>31.434</v>
       </c>
-      <c r="AJ9" s="10" t="n">
+      <c r="AK9" s="10" t="n">
         <v>30.32</v>
       </c>
-      <c r="AK9" s="10" t="n">
+      <c r="AL9" s="10" t="n">
         <v>23.847</v>
       </c>
-      <c r="AL9" s="10" t="n">
+      <c r="AM9" s="10" t="n">
         <v>25.928</v>
       </c>
-      <c r="AM9" s="10" t="n">
+      <c r="AN9" s="10" t="n">
         <v>25.259</v>
       </c>
-      <c r="AN9" s="10" t="n">
+      <c r="AO9" s="10" t="n">
         <v>25.475</v>
       </c>
     </row>
@@ -11569,45 +11760,46 @@
         <v>22.724</v>
       </c>
       <c r="Y10" s="12" t="n"/>
-      <c r="Z10" s="12" t="n">
+      <c r="Z10" s="12" t="n"/>
+      <c r="AA10" s="12" t="n">
         <v>23.431</v>
       </c>
-      <c r="AA10" s="12" t="n"/>
       <c r="AB10" s="12" t="n"/>
-      <c r="AC10" s="12" t="n">
+      <c r="AC10" s="12" t="n"/>
+      <c r="AD10" s="12" t="n">
         <v>23.834</v>
       </c>
-      <c r="AD10" s="12" t="n">
+      <c r="AE10" s="12" t="n">
         <v>45.853</v>
       </c>
-      <c r="AE10" s="12" t="n">
+      <c r="AF10" s="12" t="n">
         <v>45.695</v>
       </c>
-      <c r="AF10" s="12" t="n">
+      <c r="AG10" s="12" t="n">
         <v>43.503</v>
       </c>
-      <c r="AG10" s="12" t="n">
+      <c r="AH10" s="12" t="n">
         <v>35.124</v>
       </c>
-      <c r="AH10" s="12" t="n">
+      <c r="AI10" s="12" t="n">
         <v>34.599</v>
       </c>
-      <c r="AI10" s="12" t="n">
+      <c r="AJ10" s="12" t="n">
         <v>32.926</v>
       </c>
-      <c r="AJ10" s="12" t="n">
+      <c r="AK10" s="12" t="n">
         <v>32.212</v>
       </c>
-      <c r="AK10" s="12" t="n">
+      <c r="AL10" s="12" t="n">
         <v>24.348</v>
       </c>
-      <c r="AL10" s="12" t="n">
+      <c r="AM10" s="12" t="n">
         <v>26.424</v>
       </c>
-      <c r="AM10" s="12" t="n">
+      <c r="AN10" s="12" t="n">
         <v>25.046</v>
       </c>
-      <c r="AN10" s="12" t="n">
+      <c r="AO10" s="12" t="n">
         <v>26.209</v>
       </c>
     </row>
@@ -11675,45 +11867,46 @@
         <v>22.819</v>
       </c>
       <c r="Y11" s="10" t="n"/>
-      <c r="Z11" s="10" t="n">
+      <c r="Z11" s="10" t="n"/>
+      <c r="AA11" s="10" t="n">
         <v>23.256</v>
       </c>
-      <c r="AA11" s="10" t="n"/>
       <c r="AB11" s="10" t="n"/>
-      <c r="AC11" s="10" t="n">
+      <c r="AC11" s="10" t="n"/>
+      <c r="AD11" s="10" t="n">
         <v>24.012</v>
       </c>
-      <c r="AD11" s="10" t="n">
+      <c r="AE11" s="10" t="n">
         <v>45.048</v>
       </c>
-      <c r="AE11" s="10" t="n">
+      <c r="AF11" s="10" t="n">
         <v>44.939</v>
       </c>
-      <c r="AF11" s="10" t="n">
+      <c r="AG11" s="10" t="n">
         <v>42.925</v>
       </c>
-      <c r="AG11" s="10" t="n">
+      <c r="AH11" s="10" t="n">
         <v>34.361</v>
       </c>
-      <c r="AH11" s="10" t="n">
+      <c r="AI11" s="10" t="n">
         <v>35.246</v>
       </c>
-      <c r="AI11" s="10" t="n">
+      <c r="AJ11" s="10" t="n">
         <v>33.424</v>
       </c>
-      <c r="AJ11" s="10" t="n">
+      <c r="AK11" s="10" t="n">
         <v>31.277</v>
       </c>
-      <c r="AK11" s="10" t="n">
+      <c r="AL11" s="10" t="n">
         <v>24.496</v>
       </c>
-      <c r="AL11" s="10" t="n">
+      <c r="AM11" s="10" t="n">
         <v>26.571</v>
       </c>
-      <c r="AM11" s="10" t="n">
+      <c r="AN11" s="10" t="n">
         <v>26.186</v>
       </c>
-      <c r="AN11" s="10" t="n">
+      <c r="AO11" s="10" t="n">
         <v>25.94</v>
       </c>
     </row>
@@ -11781,45 +11974,46 @@
         <v>23.324</v>
       </c>
       <c r="Y12" s="12" t="n"/>
-      <c r="Z12" s="12" t="n">
+      <c r="Z12" s="12" t="n"/>
+      <c r="AA12" s="12" t="n">
         <v>23.65</v>
       </c>
-      <c r="AA12" s="12" t="n"/>
       <c r="AB12" s="12" t="n"/>
-      <c r="AC12" s="12" t="n">
+      <c r="AC12" s="12" t="n"/>
+      <c r="AD12" s="12" t="n">
         <v>20.587</v>
       </c>
-      <c r="AD12" s="12" t="n">
+      <c r="AE12" s="12" t="n">
         <v>52.736</v>
       </c>
-      <c r="AE12" s="12" t="n">
+      <c r="AF12" s="12" t="n">
         <v>52.189</v>
       </c>
-      <c r="AF12" s="12" t="n">
+      <c r="AG12" s="12" t="n">
         <v>49.898</v>
       </c>
-      <c r="AG12" s="12" t="n">
+      <c r="AH12" s="12" t="n">
         <v>38.256</v>
       </c>
-      <c r="AH12" s="12" t="n">
+      <c r="AI12" s="12" t="n">
         <v>39.103</v>
       </c>
-      <c r="AI12" s="12" t="n">
+      <c r="AJ12" s="12" t="n">
         <v>36.84</v>
       </c>
-      <c r="AJ12" s="12" t="n">
+      <c r="AK12" s="12" t="n">
         <v>35.122</v>
       </c>
-      <c r="AK12" s="12" t="n">
+      <c r="AL12" s="12" t="n">
         <v>25.801</v>
       </c>
-      <c r="AL12" s="12" t="n">
+      <c r="AM12" s="12" t="n">
         <v>27.861</v>
       </c>
-      <c r="AM12" s="12" t="n">
+      <c r="AN12" s="12" t="n">
         <v>27.222</v>
       </c>
-      <c r="AN12" s="12" t="n">
+      <c r="AO12" s="12" t="n">
         <v>26.693</v>
       </c>
     </row>
@@ -11837,7 +12031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y8"/>
+  <dimension ref="A1:Z8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -11865,6 +12059,7 @@
     <col width="10" customWidth="1" min="23" max="23"/>
     <col width="10" customWidth="1" min="24" max="24"/>
     <col width="10" customWidth="1" min="25" max="25"/>
+    <col width="10" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -11882,120 +12077,125 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
+          <t>Win-26</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
           <t>May-26</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>Jun-26</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>Jul-26</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>Aug-26</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Sep-26</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>Oct-26</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>Cal-27</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>Sum-27</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="K2" s="3" t="inlineStr">
         <is>
           <t>Win-27</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="L2" s="3" t="inlineStr">
         <is>
           <t>Cal-28</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="M2" s="3" t="inlineStr">
         <is>
           <t>Sum-28</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="N2" s="3" t="inlineStr">
         <is>
           <t>Win-28</t>
         </is>
       </c>
-      <c r="N2" s="3" t="inlineStr">
+      <c r="O2" s="3" t="inlineStr">
         <is>
           <t>Cal-29</t>
         </is>
       </c>
-      <c r="O2" s="3" t="inlineStr">
+      <c r="P2" s="3" t="inlineStr">
         <is>
           <t>Sum-29</t>
         </is>
       </c>
-      <c r="P2" s="3" t="inlineStr">
+      <c r="Q2" s="3" t="inlineStr">
         <is>
           <t>Cal-30</t>
         </is>
       </c>
-      <c r="Q2" s="3" t="inlineStr">
+      <c r="R2" s="3" t="inlineStr">
         <is>
           <t>Cal-31</t>
         </is>
       </c>
-      <c r="R2" s="3" t="inlineStr">
+      <c r="S2" s="3" t="inlineStr">
         <is>
           <t>Cal-32</t>
         </is>
       </c>
-      <c r="S2" s="3" t="inlineStr">
+      <c r="T2" s="3" t="inlineStr">
         <is>
           <t>2026-03</t>
         </is>
       </c>
-      <c r="T2" s="3" t="inlineStr">
+      <c r="U2" s="3" t="inlineStr">
         <is>
           <t>2026-04</t>
         </is>
       </c>
-      <c r="U2" s="3" t="inlineStr">
+      <c r="V2" s="3" t="inlineStr">
         <is>
           <t>2027-01</t>
         </is>
       </c>
-      <c r="V2" s="3" t="inlineStr">
+      <c r="W2" s="3" t="inlineStr">
         <is>
           <t>2027-02</t>
         </is>
       </c>
-      <c r="W2" s="3" t="inlineStr">
+      <c r="X2" s="3" t="inlineStr">
         <is>
           <t>2027-03</t>
         </is>
       </c>
-      <c r="X2" s="3" t="inlineStr">
+      <c r="Y2" s="3" t="inlineStr">
         <is>
           <t>2027-04</t>
         </is>
       </c>
-      <c r="Y2" s="3" t="inlineStr">
+      <c r="Z2" s="3" t="inlineStr">
         <is>
           <t>2028-01</t>
         </is>
@@ -12008,63 +12208,76 @@
         </is>
       </c>
       <c r="B3" s="10" t="n">
+        <v>39.276</v>
+      </c>
+      <c r="C3" s="10" t="n">
         <v>40.122</v>
       </c>
-      <c r="C3" s="10" t="n">
+      <c r="D3" s="10" t="n">
         <v>39.863</v>
       </c>
-      <c r="D3" s="10" t="n">
+      <c r="E3" s="10" t="n">
         <v>39.144</v>
       </c>
-      <c r="E3" s="10" t="n">
+      <c r="F3" s="10" t="n">
         <v>39.417</v>
       </c>
-      <c r="F3" s="10" t="n">
+      <c r="G3" s="10" t="n">
         <v>40.37</v>
       </c>
-      <c r="G3" s="10" t="n">
+      <c r="H3" s="10" t="n">
         <v>38.949</v>
       </c>
-      <c r="H3" s="10" t="n">
+      <c r="I3" s="10" t="n">
         <v>33.452</v>
       </c>
-      <c r="I3" s="10" t="n">
+      <c r="J3" s="10" t="n">
         <v>31.756</v>
       </c>
-      <c r="J3" s="10" t="n">
+      <c r="K3" s="10" t="n">
         <v>31.127</v>
       </c>
-      <c r="K3" s="10" t="n">
+      <c r="L3" s="10" t="n">
         <v>26.583</v>
       </c>
-      <c r="L3" s="10" t="n">
+      <c r="M3" s="10" t="n">
         <v>25.065</v>
       </c>
-      <c r="M3" s="10" t="n">
+      <c r="N3" s="10" t="n">
         <v>25.845</v>
       </c>
-      <c r="N3" s="10" t="n">
+      <c r="O3" s="10" t="n">
         <v>23.316</v>
       </c>
-      <c r="O3" s="10" t="n">
+      <c r="P3" s="10" t="n">
         <v>23.349</v>
       </c>
-      <c r="P3" s="10" t="n">
+      <c r="Q3" s="10" t="n">
         <v>23.18</v>
       </c>
-      <c r="Q3" s="10" t="n">
+      <c r="R3" s="10" t="n">
         <v>23.488</v>
       </c>
-      <c r="R3" s="10" t="n">
+      <c r="S3" s="10" t="n">
         <v>24.515</v>
       </c>
-      <c r="S3" s="10" t="n"/>
       <c r="T3" s="10" t="n"/>
       <c r="U3" s="10" t="n"/>
-      <c r="V3" s="10" t="n"/>
-      <c r="W3" s="10" t="n"/>
-      <c r="X3" s="10" t="n"/>
-      <c r="Y3" s="10" t="n"/>
+      <c r="V3" s="10" t="n">
+        <v>38.996</v>
+      </c>
+      <c r="W3" s="10" t="n">
+        <v>32.755</v>
+      </c>
+      <c r="X3" s="10" t="n">
+        <v>30.767</v>
+      </c>
+      <c r="Y3" s="10" t="n">
+        <v>31.407</v>
+      </c>
+      <c r="Z3" s="10" t="n">
+        <v>30.844</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
@@ -12072,68 +12285,69 @@
           <t>17 Apr 2026</t>
         </is>
       </c>
-      <c r="B4" s="12" t="n">
+      <c r="B4" s="12" t="n"/>
+      <c r="C4" s="12" t="n">
         <v>38.353</v>
       </c>
-      <c r="C4" s="12" t="n">
+      <c r="D4" s="12" t="n">
         <v>38.229</v>
       </c>
-      <c r="D4" s="12" t="n">
+      <c r="E4" s="12" t="n">
         <v>37.648</v>
       </c>
-      <c r="E4" s="12" t="n">
+      <c r="F4" s="12" t="n">
         <v>37.991</v>
       </c>
-      <c r="F4" s="12" t="n">
+      <c r="G4" s="12" t="n">
         <v>39.084</v>
       </c>
-      <c r="G4" s="12" t="n"/>
-      <c r="H4" s="12" t="n">
+      <c r="H4" s="12" t="n"/>
+      <c r="I4" s="12" t="n">
         <v>32.647</v>
       </c>
-      <c r="I4" s="12" t="n"/>
       <c r="J4" s="12" t="n"/>
-      <c r="K4" s="12" t="n">
+      <c r="K4" s="12" t="n"/>
+      <c r="L4" s="12" t="n">
         <v>26.072</v>
       </c>
-      <c r="L4" s="12" t="n"/>
-      <c r="M4" s="12" t="n">
+      <c r="M4" s="12" t="n"/>
+      <c r="N4" s="12" t="n">
         <v>25.372</v>
       </c>
-      <c r="N4" s="12" t="n">
+      <c r="O4" s="12" t="n">
         <v>23.266</v>
       </c>
-      <c r="O4" s="12" t="n">
+      <c r="P4" s="12" t="n">
         <v>23.434</v>
       </c>
-      <c r="P4" s="12" t="n">
+      <c r="Q4" s="12" t="n">
         <v>23.105</v>
       </c>
-      <c r="Q4" s="12" t="n">
+      <c r="R4" s="12" t="n">
         <v>23.613</v>
       </c>
-      <c r="R4" s="12" t="n">
+      <c r="S4" s="12" t="n">
         <v>24.6</v>
       </c>
-      <c r="S4" s="12" t="n">
+      <c r="T4" s="12" t="n">
         <v>38.232</v>
       </c>
-      <c r="T4" s="12" t="n">
+      <c r="U4" s="12" t="n">
         <v>38.182</v>
       </c>
-      <c r="U4" s="12" t="n">
+      <c r="V4" s="12" t="n">
         <v>37.953</v>
       </c>
-      <c r="V4" s="12" t="n">
+      <c r="W4" s="12" t="n">
         <v>31.879</v>
       </c>
-      <c r="W4" s="12" t="n">
+      <c r="X4" s="12" t="n">
         <v>30.186</v>
       </c>
-      <c r="X4" s="12" t="n">
+      <c r="Y4" s="12" t="n">
         <v>30.681</v>
       </c>
-      <c r="Y4" s="12" t="n">
+      <c r="Z4" s="12" t="n">
         <v>30.124</v>
       </c>
     </row>
@@ -12143,68 +12357,69 @@
           <t>16 Apr 2026</t>
         </is>
       </c>
-      <c r="B5" s="10" t="n">
+      <c r="B5" s="10" t="n"/>
+      <c r="C5" s="10" t="n">
         <v>42.273</v>
       </c>
-      <c r="C5" s="10" t="n">
+      <c r="D5" s="10" t="n">
         <v>42.018</v>
       </c>
-      <c r="D5" s="10" t="n">
+      <c r="E5" s="10" t="n">
         <v>41.32</v>
       </c>
-      <c r="E5" s="10" t="n">
+      <c r="F5" s="10" t="n">
         <v>41.534</v>
       </c>
-      <c r="F5" s="10" t="n">
+      <c r="G5" s="10" t="n">
         <v>42.647</v>
       </c>
-      <c r="G5" s="10" t="n"/>
-      <c r="H5" s="10" t="n">
+      <c r="H5" s="10" t="n"/>
+      <c r="I5" s="10" t="n">
         <v>34.669</v>
       </c>
-      <c r="I5" s="10" t="n"/>
       <c r="J5" s="10" t="n"/>
-      <c r="K5" s="10" t="n">
+      <c r="K5" s="10" t="n"/>
+      <c r="L5" s="10" t="n">
         <v>26.952</v>
       </c>
-      <c r="L5" s="10" t="n"/>
-      <c r="M5" s="10" t="n">
+      <c r="M5" s="10" t="n"/>
+      <c r="N5" s="10" t="n">
         <v>26.243</v>
       </c>
-      <c r="N5" s="10" t="n">
+      <c r="O5" s="10" t="n">
         <v>23.886</v>
       </c>
-      <c r="O5" s="10" t="n">
+      <c r="P5" s="10" t="n">
         <v>23.894</v>
       </c>
-      <c r="P5" s="10" t="n">
+      <c r="Q5" s="10" t="n">
         <v>23.605</v>
       </c>
-      <c r="Q5" s="10" t="n">
+      <c r="R5" s="10" t="n">
         <v>23.613</v>
       </c>
-      <c r="R5" s="10" t="n">
+      <c r="S5" s="10" t="n">
         <v>24.6</v>
       </c>
-      <c r="S5" s="10" t="n">
+      <c r="T5" s="10" t="n">
         <v>41.825</v>
       </c>
-      <c r="T5" s="10" t="n">
+      <c r="U5" s="10" t="n">
         <v>41.617</v>
       </c>
-      <c r="U5" s="10" t="n">
+      <c r="V5" s="10" t="n">
         <v>40.943</v>
       </c>
-      <c r="V5" s="10" t="n">
+      <c r="W5" s="10" t="n">
         <v>33.951</v>
       </c>
-      <c r="W5" s="10" t="n">
+      <c r="X5" s="10" t="n">
         <v>31.691</v>
       </c>
-      <c r="X5" s="10" t="n">
+      <c r="Y5" s="10" t="n">
         <v>32.222</v>
       </c>
-      <c r="Y5" s="10" t="n">
+      <c r="Z5" s="10" t="n">
         <v>31.5</v>
       </c>
     </row>
@@ -12214,68 +12429,69 @@
           <t>15 Apr 2026</t>
         </is>
       </c>
-      <c r="B6" s="12" t="n">
+      <c r="B6" s="12" t="n"/>
+      <c r="C6" s="12" t="n">
         <v>41.178</v>
       </c>
-      <c r="C6" s="12" t="n">
+      <c r="D6" s="12" t="n">
         <v>41.047</v>
       </c>
-      <c r="D6" s="12" t="n">
+      <c r="E6" s="12" t="n">
         <v>40.324</v>
       </c>
-      <c r="E6" s="12" t="n">
+      <c r="F6" s="12" t="n">
         <v>40.492</v>
       </c>
-      <c r="F6" s="12" t="n">
+      <c r="G6" s="12" t="n">
         <v>41.599</v>
       </c>
-      <c r="G6" s="12" t="n"/>
-      <c r="H6" s="12" t="n">
+      <c r="H6" s="12" t="n"/>
+      <c r="I6" s="12" t="n">
         <v>33.519</v>
       </c>
-      <c r="I6" s="12" t="n"/>
       <c r="J6" s="12" t="n"/>
-      <c r="K6" s="12" t="n">
+      <c r="K6" s="12" t="n"/>
+      <c r="L6" s="12" t="n">
         <v>26.419</v>
       </c>
-      <c r="L6" s="12" t="n"/>
-      <c r="M6" s="12" t="n">
+      <c r="M6" s="12" t="n"/>
+      <c r="N6" s="12" t="n">
         <v>25.814</v>
       </c>
-      <c r="N6" s="12" t="n">
+      <c r="O6" s="12" t="n">
         <v>23.594</v>
       </c>
-      <c r="O6" s="12" t="n">
+      <c r="P6" s="12" t="n">
         <v>23.733</v>
       </c>
-      <c r="P6" s="12" t="n">
+      <c r="Q6" s="12" t="n">
         <v>23.355</v>
       </c>
-      <c r="Q6" s="12" t="n">
+      <c r="R6" s="12" t="n">
         <v>23.863</v>
       </c>
-      <c r="R6" s="12" t="n">
+      <c r="S6" s="12" t="n">
         <v>24.6</v>
       </c>
-      <c r="S6" s="12" t="n">
+      <c r="T6" s="12" t="n">
         <v>40.796</v>
       </c>
-      <c r="T6" s="12" t="n">
+      <c r="U6" s="12" t="n">
         <v>40.343</v>
       </c>
-      <c r="U6" s="12" t="n">
+      <c r="V6" s="12" t="n">
         <v>39.614</v>
       </c>
-      <c r="V6" s="12" t="n">
+      <c r="W6" s="12" t="n">
         <v>32.904</v>
       </c>
-      <c r="W6" s="12" t="n">
+      <c r="X6" s="12" t="n">
         <v>30.744</v>
       </c>
-      <c r="X6" s="12" t="n">
+      <c r="Y6" s="12" t="n">
         <v>30.945</v>
       </c>
-      <c r="Y6" s="12" t="n">
+      <c r="Z6" s="12" t="n">
         <v>30.313</v>
       </c>
     </row>
@@ -12285,68 +12501,69 @@
           <t>14 Apr 2026</t>
         </is>
       </c>
-      <c r="B7" s="10" t="n">
+      <c r="B7" s="10" t="n"/>
+      <c r="C7" s="10" t="n">
         <v>43.21</v>
       </c>
-      <c r="C7" s="10" t="n">
+      <c r="D7" s="10" t="n">
         <v>42.964</v>
       </c>
-      <c r="D7" s="10" t="n">
+      <c r="E7" s="10" t="n">
         <v>42.154</v>
       </c>
-      <c r="E7" s="10" t="n">
+      <c r="F7" s="10" t="n">
         <v>42.18</v>
       </c>
-      <c r="F7" s="10" t="n">
+      <c r="G7" s="10" t="n">
         <v>43.297</v>
       </c>
-      <c r="G7" s="10" t="n"/>
-      <c r="H7" s="10" t="n">
+      <c r="H7" s="10" t="n"/>
+      <c r="I7" s="10" t="n">
         <v>34.257</v>
       </c>
-      <c r="I7" s="10" t="n"/>
       <c r="J7" s="10" t="n"/>
-      <c r="K7" s="10" t="n">
+      <c r="K7" s="10" t="n"/>
+      <c r="L7" s="10" t="n">
         <v>26.455</v>
       </c>
-      <c r="L7" s="10" t="n"/>
-      <c r="M7" s="10" t="n">
+      <c r="M7" s="10" t="n"/>
+      <c r="N7" s="10" t="n">
         <v>25.728</v>
       </c>
-      <c r="N7" s="10" t="n">
+      <c r="O7" s="10" t="n">
         <v>23.641</v>
       </c>
-      <c r="O7" s="10" t="n">
+      <c r="P7" s="10" t="n">
         <v>23.878</v>
       </c>
-      <c r="P7" s="10" t="n">
+      <c r="Q7" s="10" t="n">
         <v>23.355</v>
       </c>
-      <c r="Q7" s="10" t="n">
+      <c r="R7" s="10" t="n">
         <v>23.613</v>
       </c>
-      <c r="R7" s="10" t="n">
+      <c r="S7" s="10" t="n">
         <v>24.6</v>
       </c>
-      <c r="S7" s="10" t="n">
+      <c r="T7" s="10" t="n">
         <v>42.535</v>
       </c>
-      <c r="T7" s="10" t="n">
+      <c r="U7" s="10" t="n">
         <v>42.053</v>
       </c>
-      <c r="U7" s="10" t="n">
+      <c r="V7" s="10" t="n">
         <v>40.908</v>
       </c>
-      <c r="V7" s="10" t="n">
+      <c r="W7" s="10" t="n">
         <v>33.266</v>
       </c>
-      <c r="W7" s="10" t="n">
+      <c r="X7" s="10" t="n">
         <v>31.031</v>
       </c>
-      <c r="X7" s="10" t="n">
+      <c r="Y7" s="10" t="n">
         <v>31.961</v>
       </c>
-      <c r="Y7" s="10" t="n">
+      <c r="Z7" s="10" t="n">
         <v>30.716</v>
       </c>
     </row>
@@ -12356,68 +12573,69 @@
           <t>13 Apr 2026</t>
         </is>
       </c>
-      <c r="B8" s="12" t="n">
+      <c r="B8" s="12" t="n"/>
+      <c r="C8" s="12" t="n">
         <v>46.222</v>
       </c>
-      <c r="C8" s="12" t="n">
+      <c r="D8" s="12" t="n">
         <v>45.909</v>
       </c>
-      <c r="D8" s="12" t="n">
+      <c r="E8" s="12" t="n">
         <v>45.068</v>
       </c>
-      <c r="E8" s="12" t="n">
+      <c r="F8" s="12" t="n">
         <v>44.953</v>
       </c>
-      <c r="F8" s="12" t="n">
+      <c r="G8" s="12" t="n">
         <v>46.087</v>
       </c>
-      <c r="G8" s="12" t="n"/>
-      <c r="H8" s="12" t="n">
+      <c r="H8" s="12" t="n"/>
+      <c r="I8" s="12" t="n">
         <v>36.132</v>
       </c>
-      <c r="I8" s="12" t="n"/>
       <c r="J8" s="12" t="n"/>
-      <c r="K8" s="12" t="n">
+      <c r="K8" s="12" t="n"/>
+      <c r="L8" s="12" t="n">
         <v>27.106</v>
       </c>
-      <c r="L8" s="12" t="n"/>
-      <c r="M8" s="12" t="n">
+      <c r="M8" s="12" t="n"/>
+      <c r="N8" s="12" t="n">
         <v>26.093</v>
       </c>
-      <c r="N8" s="12" t="n">
+      <c r="O8" s="12" t="n">
         <v>23.898</v>
       </c>
-      <c r="O8" s="12" t="n">
+      <c r="P8" s="12" t="n">
         <v>24.168</v>
       </c>
-      <c r="P8" s="12" t="n">
+      <c r="Q8" s="12" t="n">
         <v>23.605</v>
       </c>
-      <c r="Q8" s="12" t="n">
+      <c r="R8" s="12" t="n">
         <v>23.363</v>
       </c>
-      <c r="R8" s="12" t="n">
+      <c r="S8" s="12" t="n">
         <v>24.5</v>
       </c>
-      <c r="S8" s="12" t="n">
+      <c r="T8" s="12" t="n">
         <v>45.362</v>
       </c>
-      <c r="T8" s="12" t="n">
+      <c r="U8" s="12" t="n">
         <v>44.953</v>
       </c>
-      <c r="U8" s="12" t="n">
+      <c r="V8" s="12" t="n">
         <v>43.66</v>
       </c>
-      <c r="V8" s="12" t="n">
+      <c r="W8" s="12" t="n">
         <v>34.855</v>
       </c>
-      <c r="W8" s="12" t="n">
+      <c r="X8" s="12" t="n">
         <v>32.637</v>
       </c>
-      <c r="X8" s="12" t="n">
+      <c r="Y8" s="12" t="n">
         <v>33.529</v>
       </c>
-      <c r="Y8" s="12" t="n">
+      <c r="Z8" s="12" t="n">
         <v>31.911</v>
       </c>
     </row>

</xml_diff>

<commit_message>
data: EEX curves refresh (latest trade date 2026-04-22)
</commit_message>
<xml_diff>
--- a/data/EEX_Gas_Curves.xlsx
+++ b/data/EEX_Gas_Curves.xlsx
@@ -526,7 +526,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 23 Apr 2026 08:18  ·  Source: EEX Market Data Hub (public)  ·  EUR/MWh</t>
+          <t>Generated: 23 Apr 2026 17:33  ·  Source: EEX Market Data Hub (public)  ·  EUR/MWh</t>
         </is>
       </c>
     </row>
@@ -587,7 +587,7 @@
         </is>
       </c>
       <c r="F5" s="4" t="n">
-        <v>1164</v>
+        <v>1167</v>
       </c>
     </row>
     <row r="6">
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="F6" s="6" t="n">
-        <v>318</v>
+        <v>319</v>
       </c>
     </row>
     <row r="7">
@@ -643,7 +643,7 @@
         </is>
       </c>
       <c r="F7" s="4" t="n">
-        <v>1326</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="8">
@@ -671,7 +671,7 @@
         </is>
       </c>
       <c r="F8" s="6" t="n">
-        <v>393</v>
+        <v>397</v>
       </c>
     </row>
     <row r="9">
@@ -699,7 +699,7 @@
         </is>
       </c>
       <c r="F9" s="4" t="n">
-        <v>165</v>
+        <v>170</v>
       </c>
     </row>
   </sheetData>
@@ -1562,7 +1562,9 @@
       <c r="X3" s="10" t="n"/>
       <c r="Y3" s="10" t="n"/>
       <c r="Z3" s="10" t="n"/>
-      <c r="AA3" s="10" t="n"/>
+      <c r="AA3" s="10" t="n">
+        <v>27.278</v>
+      </c>
       <c r="AB3" s="10" t="n"/>
       <c r="AC3" s="10" t="n">
         <v>36.237</v>
@@ -1660,7 +1662,9 @@
       <c r="BX3" s="10" t="n">
         <v>24.657</v>
       </c>
-      <c r="BY3" s="10" t="n"/>
+      <c r="BY3" s="10" t="n">
+        <v>25.372</v>
+      </c>
       <c r="BZ3" s="10" t="n"/>
       <c r="CA3" s="10" t="n"/>
       <c r="CB3" s="10" t="n"/>
@@ -1711,7 +1715,9 @@
       <c r="DA3" s="10" t="n">
         <v>44.226</v>
       </c>
-      <c r="DB3" s="10" t="n"/>
+      <c r="DB3" s="10" t="n">
+        <v>36.854</v>
+      </c>
       <c r="DC3" s="10" t="n"/>
       <c r="DD3" s="10" t="n"/>
       <c r="DE3" s="10" t="n"/>
@@ -5777,7 +5783,9 @@
         <v>28.268</v>
       </c>
       <c r="U3" s="10" t="n"/>
-      <c r="V3" s="10" t="n"/>
+      <c r="V3" s="10" t="n">
+        <v>24.508</v>
+      </c>
       <c r="W3" s="10" t="n"/>
       <c r="X3" s="10" t="n"/>
       <c r="Y3" s="10" t="n"/>
@@ -7772,12 +7780,18 @@
       <c r="T3" s="10" t="n">
         <v>32.746</v>
       </c>
-      <c r="U3" s="10" t="n"/>
-      <c r="V3" s="10" t="n"/>
+      <c r="U3" s="10" t="n">
+        <v>32.846</v>
+      </c>
+      <c r="V3" s="10" t="n">
+        <v>33.038</v>
+      </c>
       <c r="W3" s="10" t="n"/>
       <c r="X3" s="10" t="n"/>
       <c r="Y3" s="10" t="n"/>
-      <c r="Z3" s="10" t="n"/>
+      <c r="Z3" s="10" t="n">
+        <v>27.049</v>
+      </c>
       <c r="AA3" s="10" t="n">
         <v>25.373</v>
       </c>
@@ -7798,7 +7812,9 @@
       <c r="AN3" s="10" t="n">
         <v>25.736</v>
       </c>
-      <c r="AO3" s="10" t="n"/>
+      <c r="AO3" s="10" t="n">
+        <v>23.272</v>
+      </c>
       <c r="AP3" s="10" t="n">
         <v>22.15</v>
       </c>
@@ -7838,15 +7854,21 @@
       <c r="BB3" s="10" t="n">
         <v>22.853</v>
       </c>
-      <c r="BC3" s="10" t="n"/>
-      <c r="BD3" s="10" t="n"/>
+      <c r="BC3" s="10" t="n">
+        <v>23.06</v>
+      </c>
+      <c r="BD3" s="10" t="n">
+        <v>22.319</v>
+      </c>
       <c r="BE3" s="10" t="n">
         <v>21.316</v>
       </c>
       <c r="BF3" s="10" t="n">
         <v>22.7</v>
       </c>
-      <c r="BG3" s="10" t="n"/>
+      <c r="BG3" s="10" t="n">
+        <v>24.104</v>
+      </c>
       <c r="BH3" s="10" t="n"/>
       <c r="BI3" s="10" t="n"/>
       <c r="BJ3" s="10" t="n"/>
@@ -7908,8 +7930,12 @@
       <c r="CL3" s="10" t="n">
         <v>24.045</v>
       </c>
-      <c r="CM3" s="10" t="n"/>
-      <c r="CN3" s="10" t="n"/>
+      <c r="CM3" s="10" t="n">
+        <v>24.059</v>
+      </c>
+      <c r="CN3" s="10" t="n">
+        <v>23.674</v>
+      </c>
       <c r="CO3" s="10" t="n"/>
       <c r="CP3" s="10" t="n"/>
       <c r="CQ3" s="10" t="n"/>
@@ -7958,9 +7984,15 @@
       <c r="DL3" s="10" t="n">
         <v>22.832</v>
       </c>
-      <c r="DM3" s="10" t="n"/>
-      <c r="DN3" s="10" t="n"/>
-      <c r="DO3" s="10" t="n"/>
+      <c r="DM3" s="10" t="n">
+        <v>23.988</v>
+      </c>
+      <c r="DN3" s="10" t="n">
+        <v>22.315</v>
+      </c>
+      <c r="DO3" s="10" t="n">
+        <v>20.327</v>
+      </c>
       <c r="DP3" s="10" t="n"/>
       <c r="DQ3" s="10" t="n"/>
       <c r="DR3" s="10" t="n"/>
@@ -12263,7 +12295,9 @@
           <t>22 Apr 2026</t>
         </is>
       </c>
-      <c r="B3" s="10" t="n"/>
+      <c r="B3" s="10" t="n">
+        <v>41.679</v>
+      </c>
       <c r="C3" s="10" t="n">
         <v>42.655</v>
       </c>
@@ -12289,12 +12323,16 @@
         <v>43.326</v>
       </c>
       <c r="K3" s="10" t="n"/>
-      <c r="L3" s="10" t="n"/>
+      <c r="L3" s="10" t="n">
+        <v>33.791</v>
+      </c>
       <c r="M3" s="10" t="n"/>
       <c r="N3" s="10" t="n">
         <v>42.39</v>
       </c>
-      <c r="O3" s="10" t="n"/>
+      <c r="O3" s="10" t="n">
+        <v>43.008</v>
+      </c>
       <c r="P3" s="10" t="n"/>
       <c r="Q3" s="10" t="n">
         <v>35.691</v>
@@ -12352,7 +12390,9 @@
       <c r="AN3" s="10" t="n">
         <v>26.376</v>
       </c>
-      <c r="AO3" s="10" t="n"/>
+      <c r="AO3" s="10" t="n">
+        <v>25.494</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
@@ -13815,7 +13855,9 @@
       <c r="G3" s="10" t="n">
         <v>43.609</v>
       </c>
-      <c r="H3" s="10" t="n"/>
+      <c r="H3" s="10" t="n">
+        <v>42.06</v>
+      </c>
       <c r="I3" s="10" t="n">
         <v>35.558</v>
       </c>
@@ -13843,10 +13885,18 @@
       <c r="Q3" s="10" t="n">
         <v>22.995</v>
       </c>
-      <c r="R3" s="10" t="n"/>
-      <c r="S3" s="10" t="n"/>
-      <c r="T3" s="10" t="n"/>
-      <c r="U3" s="10" t="n"/>
+      <c r="R3" s="10" t="n">
+        <v>23.501</v>
+      </c>
+      <c r="S3" s="10" t="n">
+        <v>24.515</v>
+      </c>
+      <c r="T3" s="10" t="n">
+        <v>43.03</v>
+      </c>
+      <c r="U3" s="10" t="n">
+        <v>42.592</v>
+      </c>
       <c r="V3" s="10" t="n"/>
       <c r="W3" s="10" t="n"/>
       <c r="X3" s="10" t="n"/>

</xml_diff>

<commit_message>
data: EEX curves refresh (latest trade date 2026-04-23)
</commit_message>
<xml_diff>
--- a/data/EEX_Gas_Curves.xlsx
+++ b/data/EEX_Gas_Curves.xlsx
@@ -526,7 +526,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 24 Apr 2026 10:12  ·  Source: EEX Market Data Hub (public)  ·  EUR/MWh</t>
+          <t>Generated: 24 Apr 2026 14:05  ·  Source: EEX Market Data Hub (public)  ·  EUR/MWh</t>
         </is>
       </c>
     </row>
@@ -699,7 +699,7 @@
         </is>
       </c>
       <c r="F9" s="4" t="n">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
   </sheetData>
@@ -14681,7 +14681,9 @@
       <c r="G3" s="10" t="n">
         <v>44.41</v>
       </c>
-      <c r="H3" s="10" t="n"/>
+      <c r="H3" s="10" t="n">
+        <v>42.699</v>
+      </c>
       <c r="I3" s="10" t="n">
         <v>35.973</v>
       </c>

</xml_diff>

<commit_message>
data: EEX curves refresh (latest trade date 2026-04-24)
</commit_message>
<xml_diff>
--- a/data/EEX_Gas_Curves.xlsx
+++ b/data/EEX_Gas_Curves.xlsx
@@ -526,7 +526,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 25 Apr 2026 09:03  ·  Source: EEX Market Data Hub (public)  ·  EUR/MWh</t>
+          <t>Generated: 27 Apr 2026 17:35  ·  Source: EEX Market Data Hub (public)  ·  EUR/MWh</t>
         </is>
       </c>
     </row>
@@ -587,7 +587,7 @@
         </is>
       </c>
       <c r="F5" s="4" t="n">
-        <v>1426</v>
+        <v>1445</v>
       </c>
     </row>
     <row r="6">
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="F6" s="6" t="n">
-        <v>404</v>
+        <v>422</v>
       </c>
     </row>
     <row r="7">
@@ -643,7 +643,7 @@
         </is>
       </c>
       <c r="F7" s="4" t="n">
-        <v>1573</v>
+        <v>1643</v>
       </c>
     </row>
     <row r="8">
@@ -671,7 +671,7 @@
         </is>
       </c>
       <c r="F8" s="6" t="n">
-        <v>447</v>
+        <v>454</v>
       </c>
     </row>
     <row r="9">
@@ -699,7 +699,7 @@
         </is>
       </c>
       <c r="F9" s="4" t="n">
-        <v>211</v>
+        <v>222</v>
       </c>
     </row>
   </sheetData>
@@ -1511,7 +1511,9 @@
           <t>24 Apr 2026</t>
         </is>
       </c>
-      <c r="B3" s="10" t="n"/>
+      <c r="B3" s="10" t="n">
+        <v>46.091</v>
+      </c>
       <c r="C3" s="10" t="n">
         <v>45.315</v>
       </c>
@@ -1539,8 +1541,12 @@
       <c r="K3" s="10" t="n">
         <v>39.301</v>
       </c>
-      <c r="L3" s="10" t="n"/>
-      <c r="M3" s="10" t="n"/>
+      <c r="L3" s="10" t="n">
+        <v>37.101</v>
+      </c>
+      <c r="M3" s="10" t="n">
+        <v>36.992</v>
+      </c>
       <c r="N3" s="10" t="n">
         <v>46.505</v>
       </c>
@@ -1562,7 +1568,9 @@
       <c r="Z3" s="10" t="n">
         <v>30.667</v>
       </c>
-      <c r="AA3" s="10" t="n"/>
+      <c r="AA3" s="10" t="n">
+        <v>28.122</v>
+      </c>
       <c r="AB3" s="10" t="n"/>
       <c r="AC3" s="10" t="n">
         <v>37.418</v>
@@ -1597,7 +1605,9 @@
       <c r="AM3" s="10" t="n">
         <v>29.871</v>
       </c>
-      <c r="AN3" s="10" t="n"/>
+      <c r="AN3" s="10" t="n">
+        <v>30.17</v>
+      </c>
       <c r="AO3" s="10" t="n">
         <v>26.148</v>
       </c>
@@ -1651,15 +1661,23 @@
       <c r="BO3" s="10" t="n">
         <v>23.712</v>
       </c>
-      <c r="BP3" s="10" t="n"/>
-      <c r="BQ3" s="10" t="n"/>
-      <c r="BR3" s="10" t="n"/>
+      <c r="BP3" s="10" t="n">
+        <v>22.96</v>
+      </c>
+      <c r="BQ3" s="10" t="n">
+        <v>24.011</v>
+      </c>
+      <c r="BR3" s="10" t="n">
+        <v>24.141</v>
+      </c>
       <c r="BS3" s="10" t="n">
         <v>24.764</v>
       </c>
       <c r="BT3" s="10" t="n"/>
       <c r="BU3" s="10" t="n"/>
-      <c r="BV3" s="10" t="n"/>
+      <c r="BV3" s="10" t="n">
+        <v>25.52</v>
+      </c>
       <c r="BW3" s="10" t="n">
         <v>24.965</v>
       </c>
@@ -1733,13 +1751,27 @@
       <c r="CU3" s="10" t="n">
         <v>27.455</v>
       </c>
-      <c r="CV3" s="10" t="n"/>
-      <c r="CW3" s="10" t="n"/>
-      <c r="CX3" s="10" t="n"/>
-      <c r="CY3" s="10" t="n"/>
-      <c r="CZ3" s="10" t="n"/>
-      <c r="DA3" s="10" t="n"/>
-      <c r="DB3" s="10" t="n"/>
+      <c r="CV3" s="10" t="n">
+        <v>27.974</v>
+      </c>
+      <c r="CW3" s="10" t="n">
+        <v>27.816</v>
+      </c>
+      <c r="CX3" s="10" t="n">
+        <v>26.914</v>
+      </c>
+      <c r="CY3" s="10" t="n">
+        <v>45.878</v>
+      </c>
+      <c r="CZ3" s="10" t="n">
+        <v>46.414</v>
+      </c>
+      <c r="DA3" s="10" t="n">
+        <v>45.761</v>
+      </c>
+      <c r="DB3" s="10" t="n">
+        <v>37.906</v>
+      </c>
       <c r="DC3" s="10" t="n"/>
       <c r="DD3" s="10" t="n"/>
       <c r="DE3" s="10" t="n"/>
@@ -1784,9 +1816,15 @@
       <c r="DV3" s="10" t="n">
         <v>24.871</v>
       </c>
-      <c r="DW3" s="10" t="n"/>
-      <c r="DX3" s="10" t="n"/>
-      <c r="DY3" s="10" t="n"/>
+      <c r="DW3" s="10" t="n">
+        <v>24.953</v>
+      </c>
+      <c r="DX3" s="10" t="n">
+        <v>27.189</v>
+      </c>
+      <c r="DY3" s="10" t="n">
+        <v>27.56</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
@@ -6527,7 +6565,9 @@
           <t>24 Apr 2026</t>
         </is>
       </c>
-      <c r="B3" s="10" t="n"/>
+      <c r="B3" s="10" t="n">
+        <v>45.472</v>
+      </c>
       <c r="C3" s="10" t="n">
         <v>46.008</v>
       </c>
@@ -6540,22 +6580,44 @@
       <c r="F3" s="10" t="n">
         <v>46.633</v>
       </c>
-      <c r="G3" s="10" t="n"/>
-      <c r="H3" s="10" t="n"/>
-      <c r="I3" s="10" t="n"/>
-      <c r="J3" s="10" t="n"/>
+      <c r="G3" s="10" t="n">
+        <v>48.569</v>
+      </c>
+      <c r="H3" s="10" t="n">
+        <v>46.136</v>
+      </c>
+      <c r="I3" s="10" t="n">
+        <v>45.624</v>
+      </c>
+      <c r="J3" s="10" t="n">
+        <v>46.032</v>
+      </c>
       <c r="K3" s="10" t="n"/>
-      <c r="L3" s="10" t="n"/>
-      <c r="M3" s="10" t="n"/>
-      <c r="N3" s="10" t="n"/>
-      <c r="O3" s="10" t="n"/>
+      <c r="L3" s="10" t="n">
+        <v>37.448</v>
+      </c>
+      <c r="M3" s="10" t="n">
+        <v>35.971</v>
+      </c>
+      <c r="N3" s="10" t="n">
+        <v>44.663</v>
+      </c>
+      <c r="O3" s="10" t="n">
+        <v>44.976</v>
+      </c>
       <c r="P3" s="10" t="n"/>
       <c r="Q3" s="10" t="n"/>
       <c r="R3" s="10" t="n"/>
-      <c r="S3" s="10" t="n"/>
-      <c r="T3" s="10" t="n"/>
+      <c r="S3" s="10" t="n">
+        <v>28.77</v>
+      </c>
+      <c r="T3" s="10" t="n">
+        <v>29.031</v>
+      </c>
       <c r="U3" s="10" t="n"/>
-      <c r="V3" s="10" t="n"/>
+      <c r="V3" s="10" t="n">
+        <v>24.902</v>
+      </c>
       <c r="W3" s="10" t="n"/>
       <c r="X3" s="10" t="n">
         <v>24.447</v>
@@ -6610,7 +6672,9 @@
           <t>23 Apr 2026</t>
         </is>
       </c>
-      <c r="B4" s="12" t="n"/>
+      <c r="B4" s="12" t="n">
+        <v>44.631</v>
+      </c>
       <c r="C4" s="12" t="n">
         <v>45.819</v>
       </c>
@@ -6638,8 +6702,12 @@
       <c r="K4" s="12" t="n">
         <v>38.068</v>
       </c>
-      <c r="L4" s="12" t="n"/>
-      <c r="M4" s="12" t="n"/>
+      <c r="L4" s="12" t="n">
+        <v>36.458</v>
+      </c>
+      <c r="M4" s="12" t="n">
+        <v>35.02</v>
+      </c>
       <c r="N4" s="12" t="n">
         <v>43.674</v>
       </c>
@@ -6655,12 +6723,18 @@
       <c r="R4" s="12" t="n">
         <v>29.523</v>
       </c>
-      <c r="S4" s="12" t="n"/>
-      <c r="T4" s="12" t="n"/>
+      <c r="S4" s="12" t="n">
+        <v>27.96</v>
+      </c>
+      <c r="T4" s="12" t="n">
+        <v>28.292</v>
+      </c>
       <c r="U4" s="12" t="n">
         <v>25.54</v>
       </c>
-      <c r="V4" s="12" t="n"/>
+      <c r="V4" s="12" t="n">
+        <v>24.334</v>
+      </c>
       <c r="W4" s="12" t="n"/>
       <c r="X4" s="12" t="n">
         <v>24.352</v>
@@ -8819,19 +8893,41 @@
       <c r="I3" s="10" t="n">
         <v>42.938</v>
       </c>
-      <c r="J3" s="10" t="n"/>
-      <c r="K3" s="10" t="n"/>
+      <c r="J3" s="10" t="n">
+        <v>43.447</v>
+      </c>
+      <c r="K3" s="10" t="n">
+        <v>36.637</v>
+      </c>
       <c r="L3" s="10" t="n"/>
       <c r="M3" s="10" t="n"/>
-      <c r="N3" s="10" t="n"/>
-      <c r="O3" s="10" t="n"/>
-      <c r="P3" s="10" t="n"/>
-      <c r="Q3" s="10" t="n"/>
-      <c r="R3" s="10" t="n"/>
-      <c r="S3" s="10" t="n"/>
-      <c r="T3" s="10" t="n"/>
-      <c r="U3" s="10" t="n"/>
-      <c r="V3" s="10" t="n"/>
+      <c r="N3" s="10" t="n">
+        <v>42.796</v>
+      </c>
+      <c r="O3" s="10" t="n">
+        <v>42.784</v>
+      </c>
+      <c r="P3" s="10" t="n">
+        <v>42.253</v>
+      </c>
+      <c r="Q3" s="10" t="n">
+        <v>37.016</v>
+      </c>
+      <c r="R3" s="10" t="n">
+        <v>35.219</v>
+      </c>
+      <c r="S3" s="10" t="n">
+        <v>34.776</v>
+      </c>
+      <c r="T3" s="10" t="n">
+        <v>33.983</v>
+      </c>
+      <c r="U3" s="10" t="n">
+        <v>34.087</v>
+      </c>
+      <c r="V3" s="10" t="n">
+        <v>34.286</v>
+      </c>
       <c r="W3" s="10" t="n">
         <v>33.869</v>
       </c>
@@ -8841,7 +8937,9 @@
       <c r="Y3" s="10" t="n">
         <v>34.808</v>
       </c>
-      <c r="Z3" s="10" t="n"/>
+      <c r="Z3" s="10" t="n">
+        <v>28.139</v>
+      </c>
       <c r="AA3" s="10" t="n"/>
       <c r="AB3" s="10" t="n"/>
       <c r="AC3" s="10" t="n">
@@ -8874,26 +8972,60 @@
       <c r="AL3" s="10" t="n"/>
       <c r="AM3" s="10" t="n"/>
       <c r="AN3" s="10" t="n"/>
-      <c r="AO3" s="10" t="n"/>
+      <c r="AO3" s="10" t="n">
+        <v>23.886</v>
+      </c>
       <c r="AP3" s="10" t="n"/>
-      <c r="AQ3" s="10" t="n"/>
+      <c r="AQ3" s="10" t="n">
+        <v>23.887</v>
+      </c>
       <c r="AR3" s="10" t="n"/>
       <c r="AS3" s="10" t="n"/>
-      <c r="AT3" s="10" t="n"/>
-      <c r="AU3" s="10" t="n"/>
-      <c r="AV3" s="10" t="n"/>
-      <c r="AW3" s="10" t="n"/>
-      <c r="AX3" s="10" t="n"/>
-      <c r="AY3" s="10" t="n"/>
-      <c r="AZ3" s="10" t="n"/>
-      <c r="BA3" s="10" t="n"/>
-      <c r="BB3" s="10" t="n"/>
-      <c r="BC3" s="10" t="n"/>
-      <c r="BD3" s="10" t="n"/>
-      <c r="BE3" s="10" t="n"/>
-      <c r="BF3" s="10" t="n"/>
-      <c r="BG3" s="10" t="n"/>
-      <c r="BH3" s="10" t="n"/>
+      <c r="AT3" s="10" t="n">
+        <v>26.286</v>
+      </c>
+      <c r="AU3" s="10" t="n">
+        <v>23.304</v>
+      </c>
+      <c r="AV3" s="10" t="n">
+        <v>22.886</v>
+      </c>
+      <c r="AW3" s="10" t="n">
+        <v>22.262</v>
+      </c>
+      <c r="AX3" s="10" t="n">
+        <v>22.517</v>
+      </c>
+      <c r="AY3" s="10" t="n">
+        <v>22.593</v>
+      </c>
+      <c r="AZ3" s="10" t="n">
+        <v>22.732</v>
+      </c>
+      <c r="BA3" s="10" t="n">
+        <v>23.082</v>
+      </c>
+      <c r="BB3" s="10" t="n">
+        <v>23.36</v>
+      </c>
+      <c r="BC3" s="10" t="n">
+        <v>23.575</v>
+      </c>
+      <c r="BD3" s="10" t="n">
+        <v>22.574</v>
+      </c>
+      <c r="BE3" s="10" t="n">
+        <v>21.667</v>
+      </c>
+      <c r="BF3" s="10" t="n">
+        <v>22.695</v>
+      </c>
+      <c r="BG3" s="10" t="n">
+        <v>24.568</v>
+      </c>
+      <c r="BH3" s="10" t="n">
+        <v>24.613</v>
+      </c>
       <c r="BI3" s="10" t="n">
         <v>24.181</v>
       </c>
@@ -8927,8 +9059,12 @@
       <c r="BS3" s="10" t="n">
         <v>22.566</v>
       </c>
-      <c r="BT3" s="10" t="n"/>
-      <c r="BU3" s="10" t="n"/>
+      <c r="BT3" s="10" t="n">
+        <v>21.965</v>
+      </c>
+      <c r="BU3" s="10" t="n">
+        <v>24.065</v>
+      </c>
       <c r="BV3" s="10" t="n">
         <v>23.362</v>
       </c>
@@ -8940,21 +9076,45 @@
       <c r="BZ3" s="10" t="n"/>
       <c r="CA3" s="10" t="n"/>
       <c r="CB3" s="10" t="n"/>
-      <c r="CC3" s="10" t="n"/>
-      <c r="CD3" s="10" t="n"/>
-      <c r="CE3" s="10" t="n"/>
-      <c r="CF3" s="10" t="n"/>
-      <c r="CG3" s="10" t="n"/>
+      <c r="CC3" s="10" t="n">
+        <v>21.645</v>
+      </c>
+      <c r="CD3" s="10" t="n">
+        <v>22.543</v>
+      </c>
+      <c r="CE3" s="10" t="n">
+        <v>23.393</v>
+      </c>
+      <c r="CF3" s="10" t="n">
+        <v>23.419</v>
+      </c>
+      <c r="CG3" s="10" t="n">
+        <v>23.627</v>
+      </c>
       <c r="CH3" s="10" t="n">
         <v>23.915</v>
       </c>
-      <c r="CI3" s="10" t="n"/>
-      <c r="CJ3" s="10" t="n"/>
-      <c r="CK3" s="10" t="n"/>
-      <c r="CL3" s="10" t="n"/>
-      <c r="CM3" s="10" t="n"/>
-      <c r="CN3" s="10" t="n"/>
-      <c r="CO3" s="10" t="n"/>
+      <c r="CI3" s="10" t="n">
+        <v>23.497</v>
+      </c>
+      <c r="CJ3" s="10" t="n">
+        <v>25.156</v>
+      </c>
+      <c r="CK3" s="10" t="n">
+        <v>24.841</v>
+      </c>
+      <c r="CL3" s="10" t="n">
+        <v>23.991</v>
+      </c>
+      <c r="CM3" s="10" t="n">
+        <v>24.084</v>
+      </c>
+      <c r="CN3" s="10" t="n">
+        <v>23.699</v>
+      </c>
+      <c r="CO3" s="10" t="n">
+        <v>23.118</v>
+      </c>
       <c r="CP3" s="10" t="n">
         <v>23.661</v>
       </c>
@@ -8992,17 +9152,39 @@
       <c r="DB3" s="10" t="n"/>
       <c r="DC3" s="10" t="n"/>
       <c r="DD3" s="10" t="n"/>
-      <c r="DE3" s="10" t="n"/>
-      <c r="DF3" s="10" t="n"/>
-      <c r="DG3" s="10" t="n"/>
-      <c r="DH3" s="10" t="n"/>
-      <c r="DI3" s="10" t="n"/>
-      <c r="DJ3" s="10" t="n"/>
-      <c r="DK3" s="10" t="n"/>
-      <c r="DL3" s="10" t="n"/>
-      <c r="DM3" s="10" t="n"/>
-      <c r="DN3" s="10" t="n"/>
-      <c r="DO3" s="10" t="n"/>
+      <c r="DE3" s="10" t="n">
+        <v>33.192</v>
+      </c>
+      <c r="DF3" s="10" t="n">
+        <v>27.176</v>
+      </c>
+      <c r="DG3" s="10" t="n">
+        <v>25.769</v>
+      </c>
+      <c r="DH3" s="10" t="n">
+        <v>26.464</v>
+      </c>
+      <c r="DI3" s="10" t="n">
+        <v>26.826</v>
+      </c>
+      <c r="DJ3" s="10" t="n">
+        <v>22.818</v>
+      </c>
+      <c r="DK3" s="10" t="n">
+        <v>22.613</v>
+      </c>
+      <c r="DL3" s="10" t="n">
+        <v>23.339</v>
+      </c>
+      <c r="DM3" s="10" t="n">
+        <v>24.448</v>
+      </c>
+      <c r="DN3" s="10" t="n">
+        <v>22.701</v>
+      </c>
+      <c r="DO3" s="10" t="n">
+        <v>20.645</v>
+      </c>
       <c r="DP3" s="10" t="n">
         <v>22.539</v>
       </c>
@@ -9064,13 +9246,17 @@
       <c r="I4" s="12" t="n">
         <v>42.679</v>
       </c>
-      <c r="J4" s="12" t="n"/>
+      <c r="J4" s="12" t="n">
+        <v>42.589</v>
+      </c>
       <c r="K4" s="12" t="n">
         <v>35.681</v>
       </c>
       <c r="L4" s="12" t="n"/>
       <c r="M4" s="12" t="n"/>
-      <c r="N4" s="12" t="n"/>
+      <c r="N4" s="12" t="n">
+        <v>41.941</v>
+      </c>
       <c r="O4" s="12" t="n">
         <v>41.941</v>
       </c>
@@ -9143,12 +9329,20 @@
         <v>23.775</v>
       </c>
       <c r="AP4" s="12" t="n"/>
-      <c r="AQ4" s="12" t="n"/>
+      <c r="AQ4" s="12" t="n">
+        <v>23.749</v>
+      </c>
       <c r="AR4" s="12" t="n"/>
       <c r="AS4" s="12" t="n"/>
-      <c r="AT4" s="12" t="n"/>
-      <c r="AU4" s="12" t="n"/>
-      <c r="AV4" s="12" t="n"/>
+      <c r="AT4" s="12" t="n">
+        <v>26.082</v>
+      </c>
+      <c r="AU4" s="12" t="n">
+        <v>23.126</v>
+      </c>
+      <c r="AV4" s="12" t="n">
+        <v>22.723</v>
+      </c>
       <c r="AW4" s="12" t="n">
         <v>22.12</v>
       </c>
@@ -9173,8 +9367,12 @@
       <c r="BD4" s="12" t="n">
         <v>22.479</v>
       </c>
-      <c r="BE4" s="12" t="n"/>
-      <c r="BF4" s="12" t="n"/>
+      <c r="BE4" s="12" t="n">
+        <v>21.58</v>
+      </c>
+      <c r="BF4" s="12" t="n">
+        <v>22.822</v>
+      </c>
       <c r="BG4" s="12" t="n">
         <v>24.193</v>
       </c>
@@ -9214,7 +9412,9 @@
       <c r="BS4" s="12" t="n">
         <v>22.804</v>
       </c>
-      <c r="BT4" s="12" t="n"/>
+      <c r="BT4" s="12" t="n">
+        <v>22.292</v>
+      </c>
       <c r="BU4" s="12" t="n">
         <v>24.212</v>
       </c>
@@ -9229,9 +9429,15 @@
       <c r="BZ4" s="12" t="n"/>
       <c r="CA4" s="12" t="n"/>
       <c r="CB4" s="12" t="n"/>
-      <c r="CC4" s="12" t="n"/>
-      <c r="CD4" s="12" t="n"/>
-      <c r="CE4" s="12" t="n"/>
+      <c r="CC4" s="12" t="n">
+        <v>21.973</v>
+      </c>
+      <c r="CD4" s="12" t="n">
+        <v>22.869</v>
+      </c>
+      <c r="CE4" s="12" t="n">
+        <v>23.609</v>
+      </c>
       <c r="CF4" s="12" t="n">
         <v>23.618</v>
       </c>
@@ -9299,10 +9505,18 @@
       <c r="DB4" s="12" t="n"/>
       <c r="DC4" s="12" t="n"/>
       <c r="DD4" s="12" t="n"/>
-      <c r="DE4" s="12" t="n"/>
-      <c r="DF4" s="12" t="n"/>
-      <c r="DG4" s="12" t="n"/>
-      <c r="DH4" s="12" t="n"/>
+      <c r="DE4" s="12" t="n">
+        <v>32.161</v>
+      </c>
+      <c r="DF4" s="12" t="n">
+        <v>26.299</v>
+      </c>
+      <c r="DG4" s="12" t="n">
+        <v>24.912</v>
+      </c>
+      <c r="DH4" s="12" t="n">
+        <v>25.607</v>
+      </c>
       <c r="DI4" s="12" t="n">
         <v>26.606</v>
       </c>
@@ -14139,12 +14353,18 @@
       <c r="M3" s="10" t="n">
         <v>33.361</v>
       </c>
-      <c r="N3" s="10" t="n"/>
-      <c r="O3" s="10" t="n"/>
+      <c r="N3" s="10" t="n">
+        <v>44.146</v>
+      </c>
+      <c r="O3" s="10" t="n">
+        <v>44.74</v>
+      </c>
       <c r="P3" s="10" t="n"/>
       <c r="Q3" s="10" t="n"/>
       <c r="R3" s="10" t="n"/>
-      <c r="S3" s="10" t="n"/>
+      <c r="S3" s="10" t="n">
+        <v>26.545</v>
+      </c>
       <c r="T3" s="10" t="n"/>
       <c r="U3" s="10" t="n"/>
       <c r="V3" s="10" t="n"/>
@@ -14224,8 +14444,12 @@
       <c r="M4" s="12" t="n">
         <v>32.342</v>
       </c>
-      <c r="N4" s="12" t="n"/>
-      <c r="O4" s="12" t="n"/>
+      <c r="N4" s="12" t="n">
+        <v>43.291</v>
+      </c>
+      <c r="O4" s="12" t="n">
+        <v>43.897</v>
+      </c>
       <c r="P4" s="12" t="n">
         <v>38.548</v>
       </c>
@@ -14235,7 +14459,9 @@
       <c r="R4" s="12" t="n">
         <v>27.303</v>
       </c>
-      <c r="S4" s="12" t="n"/>
+      <c r="S4" s="12" t="n">
+        <v>25.636</v>
+      </c>
       <c r="T4" s="12" t="n"/>
       <c r="U4" s="12" t="n">
         <v>23.187</v>
@@ -14344,7 +14570,9 @@
       <c r="R5" s="10" t="n">
         <v>27.265</v>
       </c>
-      <c r="S5" s="10" t="n"/>
+      <c r="S5" s="10" t="n">
+        <v>25.6</v>
+      </c>
       <c r="T5" s="10" t="n"/>
       <c r="U5" s="10" t="n">
         <v>23.265</v>
@@ -15898,10 +16126,18 @@
       <c r="V3" s="10" t="n">
         <v>43.547</v>
       </c>
-      <c r="W3" s="10" t="n"/>
-      <c r="X3" s="10" t="n"/>
-      <c r="Y3" s="10" t="n"/>
-      <c r="Z3" s="10" t="n"/>
+      <c r="W3" s="10" t="n">
+        <v>36.145</v>
+      </c>
+      <c r="X3" s="10" t="n">
+        <v>33.64</v>
+      </c>
+      <c r="Y3" s="10" t="n">
+        <v>34.394</v>
+      </c>
+      <c r="Z3" s="10" t="n">
+        <v>33.812</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
@@ -15972,9 +16208,15 @@
       <c r="V4" s="12" t="n">
         <v>42.716</v>
       </c>
-      <c r="W4" s="12" t="n"/>
-      <c r="X4" s="12" t="n"/>
-      <c r="Y4" s="12" t="n"/>
+      <c r="W4" s="12" t="n">
+        <v>35.178</v>
+      </c>
+      <c r="X4" s="12" t="n">
+        <v>32.763</v>
+      </c>
+      <c r="Y4" s="12" t="n">
+        <v>33.376</v>
+      </c>
       <c r="Z4" s="12" t="n">
         <v>32.793</v>
       </c>
@@ -16048,9 +16290,15 @@
       <c r="V5" s="10" t="n">
         <v>41.824</v>
       </c>
-      <c r="W5" s="10" t="n"/>
-      <c r="X5" s="10" t="n"/>
-      <c r="Y5" s="10" t="n"/>
+      <c r="W5" s="10" t="n">
+        <v>34.93</v>
+      </c>
+      <c r="X5" s="10" t="n">
+        <v>32.509</v>
+      </c>
+      <c r="Y5" s="10" t="n">
+        <v>33.1</v>
+      </c>
       <c r="Z5" s="10" t="n">
         <v>32.718</v>
       </c>
@@ -16130,7 +16378,9 @@
       <c r="X6" s="12" t="n">
         <v>31.228</v>
       </c>
-      <c r="Y6" s="12" t="n"/>
+      <c r="Y6" s="12" t="n">
+        <v>31.836</v>
+      </c>
       <c r="Z6" s="12" t="n">
         <v>31.548</v>
       </c>

</xml_diff>

<commit_message>
data: EEX curves refresh (latest trade date 2026-04-27)
</commit_message>
<xml_diff>
--- a/data/EEX_Gas_Curves.xlsx
+++ b/data/EEX_Gas_Curves.xlsx
@@ -526,7 +526,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 28 Apr 2026 09:33  ·  Source: EEX Market Data Hub (public)  ·  EUR/MWh</t>
+          <t>Generated: 28 Apr 2026 10:00  ·  Source: EEX Market Data Hub (public)  ·  EUR/MWh</t>
         </is>
       </c>
     </row>
@@ -587,7 +587,7 @@
         </is>
       </c>
       <c r="F5" s="4" t="n">
-        <v>1518</v>
+        <v>1538</v>
       </c>
     </row>
     <row r="6">
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="F6" s="6" t="n">
-        <v>443</v>
+        <v>458</v>
       </c>
     </row>
     <row r="7">
@@ -643,7 +643,7 @@
         </is>
       </c>
       <c r="F7" s="4" t="n">
-        <v>1707</v>
+        <v>1721</v>
       </c>
     </row>
     <row r="8">
@@ -671,7 +671,7 @@
         </is>
       </c>
       <c r="F8" s="6" t="n">
-        <v>471</v>
+        <v>477</v>
       </c>
     </row>
     <row r="9">
@@ -699,7 +699,7 @@
         </is>
       </c>
       <c r="F9" s="4" t="n">
-        <v>237</v>
+        <v>243</v>
       </c>
     </row>
   </sheetData>
@@ -1599,15 +1599,33 @@
       <c r="AE3" s="10" t="n">
         <v>35.604</v>
       </c>
-      <c r="AF3" s="10" t="n"/>
-      <c r="AG3" s="10" t="n"/>
-      <c r="AH3" s="10" t="n"/>
-      <c r="AI3" s="10" t="n"/>
-      <c r="AJ3" s="10" t="n"/>
-      <c r="AK3" s="10" t="n"/>
-      <c r="AL3" s="10" t="n"/>
-      <c r="AM3" s="10" t="n"/>
-      <c r="AN3" s="10" t="n"/>
+      <c r="AF3" s="10" t="n">
+        <v>28.694</v>
+      </c>
+      <c r="AG3" s="10" t="n">
+        <v>28.2</v>
+      </c>
+      <c r="AH3" s="10" t="n">
+        <v>27.457</v>
+      </c>
+      <c r="AI3" s="10" t="n">
+        <v>26.883</v>
+      </c>
+      <c r="AJ3" s="10" t="n">
+        <v>26.972</v>
+      </c>
+      <c r="AK3" s="10" t="n">
+        <v>27.133</v>
+      </c>
+      <c r="AL3" s="10" t="n">
+        <v>29.078</v>
+      </c>
+      <c r="AM3" s="10" t="n">
+        <v>29.45</v>
+      </c>
+      <c r="AN3" s="10" t="n">
+        <v>29.745</v>
+      </c>
       <c r="AO3" s="10" t="n">
         <v>25.95</v>
       </c>
@@ -1617,7 +1635,9 @@
       <c r="AQ3" s="10" t="n">
         <v>25.459</v>
       </c>
-      <c r="AR3" s="10" t="n"/>
+      <c r="AR3" s="10" t="n">
+        <v>28.906</v>
+      </c>
       <c r="AS3" s="10" t="n">
         <v>28.557</v>
       </c>
@@ -1667,12 +1687,24 @@
       <c r="BI3" s="10" t="n"/>
       <c r="BJ3" s="10" t="n"/>
       <c r="BK3" s="10" t="n"/>
-      <c r="BL3" s="10" t="n"/>
-      <c r="BM3" s="10" t="n"/>
-      <c r="BN3" s="10" t="n"/>
-      <c r="BO3" s="10" t="n"/>
-      <c r="BP3" s="10" t="n"/>
-      <c r="BQ3" s="10" t="n"/>
+      <c r="BL3" s="10" t="n">
+        <v>25.195</v>
+      </c>
+      <c r="BM3" s="10" t="n">
+        <v>23.239</v>
+      </c>
+      <c r="BN3" s="10" t="n">
+        <v>23.548</v>
+      </c>
+      <c r="BO3" s="10" t="n">
+        <v>23.831</v>
+      </c>
+      <c r="BP3" s="10" t="n">
+        <v>22.861</v>
+      </c>
+      <c r="BQ3" s="10" t="n">
+        <v>23.909</v>
+      </c>
       <c r="BR3" s="10" t="n">
         <v>24.039</v>
       </c>
@@ -1681,13 +1713,21 @@
       </c>
       <c r="BT3" s="10" t="n"/>
       <c r="BU3" s="10" t="n"/>
-      <c r="BV3" s="10" t="n"/>
-      <c r="BW3" s="10" t="n"/>
-      <c r="BX3" s="10" t="n"/>
+      <c r="BV3" s="10" t="n">
+        <v>25.233</v>
+      </c>
+      <c r="BW3" s="10" t="n">
+        <v>24.68</v>
+      </c>
+      <c r="BX3" s="10" t="n">
+        <v>24.479</v>
+      </c>
       <c r="BY3" s="10" t="n">
         <v>24.488</v>
       </c>
-      <c r="BZ3" s="10" t="n"/>
+      <c r="BZ3" s="10" t="n">
+        <v>24.319</v>
+      </c>
       <c r="CA3" s="10" t="n">
         <v>23.411</v>
       </c>
@@ -6873,7 +6913,9 @@
       <c r="J3" s="10" t="n">
         <v>45.823</v>
       </c>
-      <c r="K3" s="10" t="n"/>
+      <c r="K3" s="10" t="n">
+        <v>38.757</v>
+      </c>
       <c r="L3" s="10" t="n">
         <v>37.093</v>
       </c>
@@ -6886,31 +6928,59 @@
       <c r="O3" s="10" t="n">
         <v>44.821</v>
       </c>
-      <c r="P3" s="10" t="n"/>
-      <c r="Q3" s="10" t="n"/>
-      <c r="R3" s="10" t="n"/>
+      <c r="P3" s="10" t="n">
+        <v>45.205</v>
+      </c>
+      <c r="Q3" s="10" t="n">
+        <v>39.438</v>
+      </c>
+      <c r="R3" s="10" t="n">
+        <v>30.008</v>
+      </c>
       <c r="S3" s="10" t="n">
         <v>28.344</v>
       </c>
       <c r="T3" s="10" t="n">
         <v>28.599</v>
       </c>
-      <c r="U3" s="10" t="n"/>
+      <c r="U3" s="10" t="n">
+        <v>25.84</v>
+      </c>
       <c r="V3" s="10" t="n">
         <v>24.704</v>
       </c>
       <c r="W3" s="10" t="n"/>
-      <c r="X3" s="10" t="n"/>
+      <c r="X3" s="10" t="n">
+        <v>24.482</v>
+      </c>
       <c r="Y3" s="10" t="n"/>
-      <c r="Z3" s="10" t="n"/>
-      <c r="AA3" s="10" t="n"/>
-      <c r="AB3" s="10" t="n"/>
-      <c r="AC3" s="10" t="n"/>
-      <c r="AD3" s="10" t="n"/>
-      <c r="AE3" s="10" t="n"/>
-      <c r="AF3" s="10" t="n"/>
-      <c r="AG3" s="10" t="n"/>
-      <c r="AH3" s="10" t="n"/>
+      <c r="Z3" s="10" t="n">
+        <v>24.716</v>
+      </c>
+      <c r="AA3" s="10" t="n">
+        <v>23.875</v>
+      </c>
+      <c r="AB3" s="10" t="n">
+        <v>23.484</v>
+      </c>
+      <c r="AC3" s="10" t="n">
+        <v>25.888</v>
+      </c>
+      <c r="AD3" s="10" t="n">
+        <v>25.615</v>
+      </c>
+      <c r="AE3" s="10" t="n">
+        <v>47.451</v>
+      </c>
+      <c r="AF3" s="10" t="n">
+        <v>45.727</v>
+      </c>
+      <c r="AG3" s="10" t="n">
+        <v>44.845</v>
+      </c>
+      <c r="AH3" s="10" t="n">
+        <v>37.747</v>
+      </c>
       <c r="AI3" s="10" t="n"/>
       <c r="AJ3" s="10" t="n"/>
       <c r="AK3" s="10" t="n">
@@ -9299,15 +9369,23 @@
       <c r="W3" s="10" t="n">
         <v>33.59</v>
       </c>
-      <c r="X3" s="10" t="n"/>
-      <c r="Y3" s="10" t="n"/>
+      <c r="X3" s="10" t="n">
+        <v>33.842</v>
+      </c>
+      <c r="Y3" s="10" t="n">
+        <v>34.478</v>
+      </c>
       <c r="Z3" s="10" t="n">
         <v>27.657</v>
       </c>
       <c r="AA3" s="10" t="n"/>
       <c r="AB3" s="10" t="n"/>
-      <c r="AC3" s="10" t="n"/>
-      <c r="AD3" s="10" t="n"/>
+      <c r="AC3" s="10" t="n">
+        <v>33.557</v>
+      </c>
+      <c r="AD3" s="10" t="n">
+        <v>32.715</v>
+      </c>
       <c r="AE3" s="10" t="n"/>
       <c r="AF3" s="10" t="n"/>
       <c r="AG3" s="10" t="n"/>
@@ -9369,9 +9447,15 @@
       <c r="BI3" s="10" t="n">
         <v>24.163</v>
       </c>
-      <c r="BJ3" s="10" t="n"/>
-      <c r="BK3" s="10" t="n"/>
-      <c r="BL3" s="10" t="n"/>
+      <c r="BJ3" s="10" t="n">
+        <v>23.171</v>
+      </c>
+      <c r="BK3" s="10" t="n">
+        <v>22.773</v>
+      </c>
+      <c r="BL3" s="10" t="n">
+        <v>22.566</v>
+      </c>
       <c r="BM3" s="10" t="n"/>
       <c r="BN3" s="10" t="n"/>
       <c r="BO3" s="10" t="n"/>
@@ -9437,9 +9521,15 @@
       <c r="CQ3" s="10" t="n">
         <v>23.292</v>
       </c>
-      <c r="CR3" s="10" t="n"/>
-      <c r="CS3" s="10" t="n"/>
-      <c r="CT3" s="10" t="n"/>
+      <c r="CR3" s="10" t="n">
+        <v>23.217</v>
+      </c>
+      <c r="CS3" s="10" t="n">
+        <v>23.797</v>
+      </c>
+      <c r="CT3" s="10" t="n">
+        <v>24.072</v>
+      </c>
       <c r="CU3" s="10" t="n"/>
       <c r="CV3" s="10" t="n"/>
       <c r="CW3" s="10" t="n"/>
@@ -9488,10 +9578,18 @@
       <c r="DR3" s="10" t="n">
         <v>21.535</v>
       </c>
-      <c r="DS3" s="10" t="n"/>
-      <c r="DT3" s="10" t="n"/>
-      <c r="DU3" s="10" t="n"/>
-      <c r="DV3" s="10" t="n"/>
+      <c r="DS3" s="10" t="n">
+        <v>21.437</v>
+      </c>
+      <c r="DT3" s="10" t="n">
+        <v>23.128</v>
+      </c>
+      <c r="DU3" s="10" t="n">
+        <v>24.555</v>
+      </c>
+      <c r="DV3" s="10" t="n">
+        <v>23.659</v>
+      </c>
       <c r="DW3" s="10" t="n"/>
       <c r="DX3" s="10" t="n"/>
       <c r="DY3" s="10" t="n"/>
@@ -14953,9 +15051,15 @@
         </is>
       </c>
       <c r="B3" s="10" t="n"/>
-      <c r="C3" s="10" t="n"/>
-      <c r="D3" s="10" t="n"/>
-      <c r="E3" s="10" t="n"/>
+      <c r="C3" s="10" t="n">
+        <v>43.935</v>
+      </c>
+      <c r="D3" s="10" t="n">
+        <v>44.184</v>
+      </c>
+      <c r="E3" s="10" t="n">
+        <v>44.634</v>
+      </c>
       <c r="F3" s="10" t="n"/>
       <c r="G3" s="10" t="n"/>
       <c r="H3" s="10" t="n"/>
@@ -15023,9 +15127,15 @@
       <c r="AL3" s="10" t="n">
         <v>25.16</v>
       </c>
-      <c r="AM3" s="10" t="n"/>
-      <c r="AN3" s="10" t="n"/>
-      <c r="AO3" s="10" t="n"/>
+      <c r="AM3" s="10" t="n">
+        <v>26.892</v>
+      </c>
+      <c r="AN3" s="10" t="n">
+        <v>26.81</v>
+      </c>
+      <c r="AO3" s="10" t="n">
+        <v>25.723</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
@@ -16798,8 +16908,12 @@
       <c r="F3" s="10" t="n">
         <v>43.663</v>
       </c>
-      <c r="G3" s="10" t="n"/>
-      <c r="H3" s="10" t="n"/>
+      <c r="G3" s="10" t="n">
+        <v>44.786</v>
+      </c>
+      <c r="H3" s="10" t="n">
+        <v>43.5</v>
+      </c>
       <c r="I3" s="10" t="n">
         <v>36.645</v>
       </c>
@@ -16824,10 +16938,18 @@
       <c r="P3" s="10" t="n">
         <v>23.995</v>
       </c>
-      <c r="Q3" s="10" t="n"/>
-      <c r="R3" s="10" t="n"/>
-      <c r="S3" s="10" t="n"/>
-      <c r="T3" s="10" t="n"/>
+      <c r="Q3" s="10" t="n">
+        <v>23.285</v>
+      </c>
+      <c r="R3" s="10" t="n">
+        <v>22.863</v>
+      </c>
+      <c r="S3" s="10" t="n">
+        <v>24.515</v>
+      </c>
+      <c r="T3" s="10" t="n">
+        <v>44.209</v>
+      </c>
       <c r="U3" s="10" t="n"/>
       <c r="V3" s="10" t="n"/>
       <c r="W3" s="10" t="n"/>

</xml_diff>

<commit_message>
data: EEX curves refresh (latest trade date 2026-04-28)
</commit_message>
<xml_diff>
--- a/data/EEX_Gas_Curves.xlsx
+++ b/data/EEX_Gas_Curves.xlsx
@@ -526,7 +526,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 29 Apr 2026 08:22  ·  Source: EEX Market Data Hub (public)  ·  EUR/MWh</t>
+          <t>Generated: 29 Apr 2026 17:36  ·  Source: EEX Market Data Hub (public)  ·  EUR/MWh</t>
         </is>
       </c>
     </row>
@@ -587,7 +587,7 @@
         </is>
       </c>
       <c r="F5" s="4" t="n">
-        <v>1596</v>
+        <v>1599</v>
       </c>
     </row>
     <row r="6">
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="F6" s="6" t="n">
-        <v>485</v>
+        <v>486</v>
       </c>
     </row>
     <row r="7">
@@ -643,7 +643,7 @@
         </is>
       </c>
       <c r="F7" s="4" t="n">
-        <v>1779</v>
+        <v>1784</v>
       </c>
     </row>
     <row r="8">
@@ -671,7 +671,7 @@
         </is>
       </c>
       <c r="F8" s="6" t="n">
-        <v>494</v>
+        <v>498</v>
       </c>
     </row>
     <row r="9">
@@ -699,7 +699,7 @@
         </is>
       </c>
       <c r="F9" s="4" t="n">
-        <v>258</v>
+        <v>260</v>
       </c>
     </row>
   </sheetData>
@@ -1586,9 +1586,11 @@
       <c r="AH3" s="10" t="n">
         <v>27.395</v>
       </c>
-      <c r="AI3" s="10" t="n"/>
+      <c r="AI3" s="10" t="n">
+        <v>26.82</v>
+      </c>
       <c r="AJ3" s="10" t="n">
-        <v>26.82</v>
+        <v>26.909</v>
       </c>
       <c r="AK3" s="10" t="n">
         <v>27.07</v>
@@ -1605,7 +1607,9 @@
       <c r="AO3" s="10" t="n"/>
       <c r="AP3" s="10" t="n"/>
       <c r="AQ3" s="10" t="n"/>
-      <c r="AR3" s="10" t="n"/>
+      <c r="AR3" s="10" t="n">
+        <v>28.328</v>
+      </c>
       <c r="AS3" s="10" t="n"/>
       <c r="AT3" s="10" t="n"/>
       <c r="AU3" s="10" t="n"/>
@@ -1663,7 +1667,9 @@
       <c r="BY3" s="10" t="n">
         <v>24.559</v>
       </c>
-      <c r="BZ3" s="10" t="n"/>
+      <c r="BZ3" s="10" t="n">
+        <v>24.388</v>
+      </c>
       <c r="CA3" s="10" t="n"/>
       <c r="CB3" s="10" t="n"/>
       <c r="CC3" s="10" t="n"/>
@@ -1857,7 +1863,7 @@
         <v>26.883</v>
       </c>
       <c r="AJ4" s="12" t="n">
-        <v>26.883</v>
+        <v>26.972</v>
       </c>
       <c r="AK4" s="12" t="n">
         <v>27.133</v>
@@ -7218,7 +7224,9 @@
       <c r="AF3" s="10" t="n">
         <v>44.702</v>
       </c>
-      <c r="AG3" s="10" t="n"/>
+      <c r="AG3" s="10" t="n">
+        <v>43.713</v>
+      </c>
       <c r="AH3" s="10" t="n"/>
       <c r="AI3" s="10" t="n"/>
       <c r="AJ3" s="10" t="n"/>
@@ -9780,7 +9788,9 @@
       <c r="BJ3" s="10" t="n">
         <v>22.982</v>
       </c>
-      <c r="BK3" s="10" t="n"/>
+      <c r="BK3" s="10" t="n">
+        <v>22.585</v>
+      </c>
       <c r="BL3" s="10" t="n"/>
       <c r="BM3" s="10" t="n"/>
       <c r="BN3" s="10" t="n"/>
@@ -9847,8 +9857,12 @@
       <c r="CQ3" s="10" t="n">
         <v>23.239</v>
       </c>
-      <c r="CR3" s="10" t="n"/>
-      <c r="CS3" s="10" t="n"/>
+      <c r="CR3" s="10" t="n">
+        <v>23.164</v>
+      </c>
+      <c r="CS3" s="10" t="n">
+        <v>23.815</v>
+      </c>
       <c r="CT3" s="10" t="n"/>
       <c r="CU3" s="10" t="n"/>
       <c r="CV3" s="10" t="n"/>
@@ -9898,8 +9912,12 @@
       <c r="DR3" s="10" t="n">
         <v>21.606</v>
       </c>
-      <c r="DS3" s="10" t="n"/>
-      <c r="DT3" s="10" t="n"/>
+      <c r="DS3" s="10" t="n">
+        <v>21.508</v>
+      </c>
+      <c r="DT3" s="10" t="n">
+        <v>23.056</v>
+      </c>
       <c r="DU3" s="10" t="n"/>
       <c r="DV3" s="10" t="n"/>
       <c r="DW3" s="10" t="n"/>
@@ -15654,8 +15672,12 @@
         </is>
       </c>
       <c r="B3" s="10" t="n"/>
-      <c r="C3" s="10" t="n"/>
-      <c r="D3" s="10" t="n"/>
+      <c r="C3" s="10" t="n">
+        <v>42.949</v>
+      </c>
+      <c r="D3" s="10" t="n">
+        <v>43.094</v>
+      </c>
       <c r="E3" s="10" t="n"/>
       <c r="F3" s="10" t="n"/>
       <c r="G3" s="10" t="n"/>
@@ -15724,8 +15746,12 @@
       <c r="AL3" s="10" t="n">
         <v>25.019</v>
       </c>
-      <c r="AM3" s="10" t="n"/>
-      <c r="AN3" s="10" t="n"/>
+      <c r="AM3" s="10" t="n">
+        <v>26.751</v>
+      </c>
+      <c r="AN3" s="10" t="n">
+        <v>26.478</v>
+      </c>
       <c r="AO3" s="10" t="n"/>
     </row>
     <row r="4">
@@ -17618,8 +17644,12 @@
       <c r="P3" s="10" t="n">
         <v>23.869</v>
       </c>
-      <c r="Q3" s="10" t="n"/>
-      <c r="R3" s="10" t="n"/>
+      <c r="Q3" s="10" t="n">
+        <v>23.105</v>
+      </c>
+      <c r="R3" s="10" t="n">
+        <v>22.863</v>
+      </c>
       <c r="S3" s="10" t="n"/>
       <c r="T3" s="10" t="n"/>
       <c r="U3" s="10" t="n"/>

</xml_diff>

<commit_message>
data: EEX curves full hub recovery (latest trade date 2026-04-29)
Re-scraped PSV (18 to 36 tenors), PEG (57 to 98 tenors), and PVB (17 to 31 tenors) to recover missing front-month tenors (May/Jun/Jul-26) from this morning's partial scrape. All 5 hubs now have complete M+1/M+2/M+3 coverage.
</commit_message>
<xml_diff>
--- a/data/EEX_Gas_Curves.xlsx
+++ b/data/EEX_Gas_Curves.xlsx
@@ -526,7 +526,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 30 Apr 2026 09:33  ·  Source: EEX Market Data Hub (public)  ·  EUR/MWh</t>
+          <t>Generated: 30 Apr 2026 13:36  ·  Source: EEX Market Data Hub (public)  ·  EUR/MWh</t>
         </is>
       </c>
     </row>
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="F6" s="6" t="n">
-        <v>509</v>
+        <v>537</v>
       </c>
     </row>
     <row r="7">
@@ -643,7 +643,7 @@
         </is>
       </c>
       <c r="F7" s="4" t="n">
-        <v>1852</v>
+        <v>1962</v>
       </c>
     </row>
     <row r="8">
@@ -671,7 +671,7 @@
         </is>
       </c>
       <c r="F8" s="6" t="n">
-        <v>515</v>
+        <v>553</v>
       </c>
     </row>
     <row r="9">
@@ -7582,20 +7582,42 @@
           <t>29 Apr 2026</t>
         </is>
       </c>
-      <c r="B3" s="10" t="n"/>
-      <c r="C3" s="10" t="n"/>
-      <c r="D3" s="10" t="n"/>
-      <c r="E3" s="10" t="n"/>
-      <c r="F3" s="10" t="n"/>
-      <c r="G3" s="10" t="n"/>
-      <c r="H3" s="10" t="n"/>
-      <c r="I3" s="10" t="n"/>
-      <c r="J3" s="10" t="n"/>
+      <c r="B3" s="10" t="n">
+        <v>47.125</v>
+      </c>
+      <c r="C3" s="10" t="n">
+        <v>47.477</v>
+      </c>
+      <c r="D3" s="10" t="n">
+        <v>48.493</v>
+      </c>
+      <c r="E3" s="10" t="n">
+        <v>49.691</v>
+      </c>
+      <c r="F3" s="10" t="n">
+        <v>48.477</v>
+      </c>
+      <c r="G3" s="10" t="n">
+        <v>50.36</v>
+      </c>
+      <c r="H3" s="10" t="n">
+        <v>48.093</v>
+      </c>
+      <c r="I3" s="10" t="n">
+        <v>47.898</v>
+      </c>
+      <c r="J3" s="10" t="n">
+        <v>47.502</v>
+      </c>
       <c r="K3" s="10" t="n">
         <v>39.725</v>
       </c>
-      <c r="L3" s="10" t="n"/>
-      <c r="M3" s="10" t="n"/>
+      <c r="L3" s="10" t="n">
+        <v>37.898</v>
+      </c>
+      <c r="M3" s="10" t="n">
+        <v>36.311</v>
+      </c>
       <c r="N3" s="10" t="n">
         <v>46.091</v>
       </c>
@@ -7611,8 +7633,12 @@
       <c r="R3" s="10" t="n">
         <v>30.23</v>
       </c>
-      <c r="S3" s="10" t="n"/>
-      <c r="T3" s="10" t="n"/>
+      <c r="S3" s="10" t="n">
+        <v>28.576</v>
+      </c>
+      <c r="T3" s="10" t="n">
+        <v>28.679</v>
+      </c>
       <c r="U3" s="10" t="n">
         <v>25.939</v>
       </c>
@@ -7653,11 +7679,21 @@
       <c r="AJ3" s="10" t="n">
         <v>36.825</v>
       </c>
-      <c r="AK3" s="10" t="n"/>
-      <c r="AL3" s="10" t="n"/>
-      <c r="AM3" s="10" t="n"/>
-      <c r="AN3" s="10" t="n"/>
-      <c r="AO3" s="10" t="n"/>
+      <c r="AK3" s="10" t="n">
+        <v>35.791</v>
+      </c>
+      <c r="AL3" s="10" t="n">
+        <v>29.509</v>
+      </c>
+      <c r="AM3" s="10" t="n">
+        <v>27.654</v>
+      </c>
+      <c r="AN3" s="10" t="n">
+        <v>28.028</v>
+      </c>
+      <c r="AO3" s="10" t="n">
+        <v>29.345</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
@@ -7665,7 +7701,9 @@
           <t>28 Apr 2026</t>
         </is>
       </c>
-      <c r="B4" s="12" t="n"/>
+      <c r="B4" s="12" t="n">
+        <v>44.213</v>
+      </c>
       <c r="C4" s="12" t="n">
         <v>44.29</v>
       </c>
@@ -7693,8 +7731,12 @@
       <c r="K4" s="12" t="n">
         <v>37.922</v>
       </c>
-      <c r="L4" s="12" t="n"/>
-      <c r="M4" s="12" t="n"/>
+      <c r="L4" s="12" t="n">
+        <v>36.324</v>
+      </c>
+      <c r="M4" s="12" t="n">
+        <v>34.949</v>
+      </c>
       <c r="N4" s="12" t="n">
         <v>43.356</v>
       </c>
@@ -7710,8 +7752,12 @@
       <c r="R4" s="12" t="n">
         <v>29.611</v>
       </c>
-      <c r="S4" s="12" t="n"/>
-      <c r="T4" s="12" t="n"/>
+      <c r="S4" s="12" t="n">
+        <v>28.164</v>
+      </c>
+      <c r="T4" s="12" t="n">
+        <v>28.29</v>
+      </c>
       <c r="U4" s="12" t="n">
         <v>25.685</v>
       </c>
@@ -7758,11 +7804,21 @@
       <c r="AJ4" s="12" t="n">
         <v>35.436</v>
       </c>
-      <c r="AK4" s="12" t="n"/>
-      <c r="AL4" s="12" t="n"/>
-      <c r="AM4" s="12" t="n"/>
-      <c r="AN4" s="12" t="n"/>
-      <c r="AO4" s="12" t="n"/>
+      <c r="AK4" s="12" t="n">
+        <v>34.456</v>
+      </c>
+      <c r="AL4" s="12" t="n">
+        <v>28.839</v>
+      </c>
+      <c r="AM4" s="12" t="n">
+        <v>27.496</v>
+      </c>
+      <c r="AN4" s="12" t="n">
+        <v>27.697</v>
+      </c>
+      <c r="AO4" s="12" t="n">
+        <v>28.896</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -10201,24 +10257,48 @@
           <t>29 Apr 2026</t>
         </is>
       </c>
-      <c r="B3" s="10" t="n"/>
+      <c r="B3" s="10" t="n">
+        <v>44.682</v>
+      </c>
       <c r="C3" s="10" t="n">
         <v>45.944</v>
       </c>
-      <c r="D3" s="10" t="n"/>
-      <c r="E3" s="10" t="n"/>
-      <c r="F3" s="10" t="n"/>
-      <c r="G3" s="10" t="n"/>
-      <c r="H3" s="10" t="n"/>
-      <c r="I3" s="10" t="n"/>
-      <c r="J3" s="10" t="n"/>
+      <c r="D3" s="10" t="n">
+        <v>46.148</v>
+      </c>
+      <c r="E3" s="10" t="n">
+        <v>46.229</v>
+      </c>
+      <c r="F3" s="10" t="n">
+        <v>46.142</v>
+      </c>
+      <c r="G3" s="10" t="n">
+        <v>46.09</v>
+      </c>
+      <c r="H3" s="10" t="n">
+        <v>45.574</v>
+      </c>
+      <c r="I3" s="10" t="n">
+        <v>45.115</v>
+      </c>
+      <c r="J3" s="10" t="n">
+        <v>44.82</v>
+      </c>
       <c r="K3" s="10" t="n">
         <v>37.342</v>
       </c>
-      <c r="L3" s="10" t="n"/>
-      <c r="M3" s="10" t="n"/>
-      <c r="N3" s="10" t="n"/>
-      <c r="O3" s="10" t="n"/>
+      <c r="L3" s="10" t="n">
+        <v>35.319</v>
+      </c>
+      <c r="M3" s="10" t="n">
+        <v>34.052</v>
+      </c>
+      <c r="N3" s="10" t="n">
+        <v>44.398</v>
+      </c>
+      <c r="O3" s="10" t="n">
+        <v>44.363</v>
+      </c>
       <c r="P3" s="10" t="n"/>
       <c r="Q3" s="10" t="n">
         <v>37.598</v>
@@ -10261,14 +10341,30 @@
       <c r="AE3" s="10" t="n">
         <v>32.756</v>
       </c>
-      <c r="AF3" s="10" t="n"/>
-      <c r="AG3" s="10" t="n"/>
-      <c r="AH3" s="10" t="n"/>
-      <c r="AI3" s="10" t="n"/>
-      <c r="AJ3" s="10" t="n"/>
-      <c r="AK3" s="10" t="n"/>
-      <c r="AL3" s="10" t="n"/>
-      <c r="AM3" s="10" t="n"/>
+      <c r="AF3" s="10" t="n">
+        <v>27.784</v>
+      </c>
+      <c r="AG3" s="10" t="n">
+        <v>27.317</v>
+      </c>
+      <c r="AH3" s="10" t="n">
+        <v>26.614</v>
+      </c>
+      <c r="AI3" s="10" t="n">
+        <v>25.226</v>
+      </c>
+      <c r="AJ3" s="10" t="n">
+        <v>25.309</v>
+      </c>
+      <c r="AK3" s="10" t="n">
+        <v>25.458</v>
+      </c>
+      <c r="AL3" s="10" t="n">
+        <v>25.791</v>
+      </c>
+      <c r="AM3" s="10" t="n">
+        <v>26.107</v>
+      </c>
       <c r="AN3" s="10" t="n"/>
       <c r="AO3" s="10" t="n">
         <v>23.39</v>
@@ -10323,11 +10419,21 @@
       <c r="BM3" s="10" t="n">
         <v>20.433</v>
       </c>
-      <c r="BN3" s="10" t="n"/>
-      <c r="BO3" s="10" t="n"/>
-      <c r="BP3" s="10" t="n"/>
-      <c r="BQ3" s="10" t="n"/>
-      <c r="BR3" s="10" t="n"/>
+      <c r="BN3" s="10" t="n">
+        <v>20.735</v>
+      </c>
+      <c r="BO3" s="10" t="n">
+        <v>21.002</v>
+      </c>
+      <c r="BP3" s="10" t="n">
+        <v>21.979</v>
+      </c>
+      <c r="BQ3" s="10" t="n">
+        <v>23.023</v>
+      </c>
+      <c r="BR3" s="10" t="n">
+        <v>23.131</v>
+      </c>
       <c r="BS3" s="10" t="n">
         <v>22.704</v>
       </c>
@@ -10335,11 +10441,21 @@
       <c r="BU3" s="10" t="n">
         <v>24.136</v>
       </c>
-      <c r="BV3" s="10" t="n"/>
-      <c r="BW3" s="10" t="n"/>
-      <c r="BX3" s="10" t="n"/>
-      <c r="BY3" s="10" t="n"/>
-      <c r="BZ3" s="10" t="n"/>
+      <c r="BV3" s="10" t="n">
+        <v>23.539</v>
+      </c>
+      <c r="BW3" s="10" t="n">
+        <v>22.951</v>
+      </c>
+      <c r="BX3" s="10" t="n">
+        <v>22.568</v>
+      </c>
+      <c r="BY3" s="10" t="n">
+        <v>22.632</v>
+      </c>
+      <c r="BZ3" s="10" t="n">
+        <v>22.495</v>
+      </c>
       <c r="CA3" s="10" t="n"/>
       <c r="CB3" s="10" t="n"/>
       <c r="CC3" s="10" t="n"/>
@@ -10389,12 +10505,24 @@
       <c r="CU3" s="10" t="n">
         <v>24.211</v>
       </c>
-      <c r="CV3" s="10" t="n"/>
-      <c r="CW3" s="10" t="n"/>
-      <c r="CX3" s="10" t="n"/>
-      <c r="CY3" s="10" t="n"/>
-      <c r="CZ3" s="10" t="n"/>
-      <c r="DA3" s="10" t="n"/>
+      <c r="CV3" s="10" t="n">
+        <v>25.779</v>
+      </c>
+      <c r="CW3" s="10" t="n">
+        <v>25.692</v>
+      </c>
+      <c r="CX3" s="10" t="n">
+        <v>24.818</v>
+      </c>
+      <c r="CY3" s="10" t="n">
+        <v>46.154</v>
+      </c>
+      <c r="CZ3" s="10" t="n">
+        <v>45.17</v>
+      </c>
+      <c r="DA3" s="10" t="n">
+        <v>44.183</v>
+      </c>
       <c r="DB3" s="10" t="n"/>
       <c r="DC3" s="10" t="n"/>
       <c r="DD3" s="10" t="n"/>
@@ -10438,11 +10566,21 @@
       <c r="DT3" s="10" t="n">
         <v>23.401</v>
       </c>
-      <c r="DU3" s="10" t="n"/>
-      <c r="DV3" s="10" t="n"/>
-      <c r="DW3" s="10" t="n"/>
-      <c r="DX3" s="10" t="n"/>
-      <c r="DY3" s="10" t="n"/>
+      <c r="DU3" s="10" t="n">
+        <v>24.88</v>
+      </c>
+      <c r="DV3" s="10" t="n">
+        <v>23.528</v>
+      </c>
+      <c r="DW3" s="10" t="n">
+        <v>23.27</v>
+      </c>
+      <c r="DX3" s="10" t="n">
+        <v>23.99</v>
+      </c>
+      <c r="DY3" s="10" t="n">
+        <v>25.421</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
@@ -10450,22 +10588,42 @@
           <t>28 Apr 2026</t>
         </is>
       </c>
-      <c r="B4" s="12" t="n"/>
+      <c r="B4" s="12" t="n">
+        <v>41.752</v>
+      </c>
       <c r="C4" s="12" t="n">
         <v>42.722</v>
       </c>
-      <c r="D4" s="12" t="n"/>
-      <c r="E4" s="12" t="n"/>
-      <c r="F4" s="12" t="n"/>
-      <c r="G4" s="12" t="n"/>
-      <c r="H4" s="12" t="n"/>
-      <c r="I4" s="12" t="n"/>
-      <c r="J4" s="12" t="n"/>
+      <c r="D4" s="12" t="n">
+        <v>43.007</v>
+      </c>
+      <c r="E4" s="12" t="n">
+        <v>43.004</v>
+      </c>
+      <c r="F4" s="12" t="n">
+        <v>43.018</v>
+      </c>
+      <c r="G4" s="12" t="n">
+        <v>42.888</v>
+      </c>
+      <c r="H4" s="12" t="n">
+        <v>42.387</v>
+      </c>
+      <c r="I4" s="12" t="n">
+        <v>41.941</v>
+      </c>
+      <c r="J4" s="12" t="n">
+        <v>41.971</v>
+      </c>
       <c r="K4" s="12" t="n">
         <v>35.51</v>
       </c>
-      <c r="L4" s="12" t="n"/>
-      <c r="M4" s="12" t="n"/>
+      <c r="L4" s="12" t="n">
+        <v>33.727</v>
+      </c>
+      <c r="M4" s="12" t="n">
+        <v>32.69</v>
+      </c>
       <c r="N4" s="12" t="n">
         <v>41.566</v>
       </c>
@@ -10516,14 +10674,30 @@
       <c r="AE4" s="12" t="n">
         <v>31.437</v>
       </c>
-      <c r="AF4" s="12" t="n"/>
-      <c r="AG4" s="12" t="n"/>
-      <c r="AH4" s="12" t="n"/>
-      <c r="AI4" s="12" t="n"/>
-      <c r="AJ4" s="12" t="n"/>
-      <c r="AK4" s="12" t="n"/>
-      <c r="AL4" s="12" t="n"/>
-      <c r="AM4" s="12" t="n"/>
+      <c r="AF4" s="12" t="n">
+        <v>27.168</v>
+      </c>
+      <c r="AG4" s="12" t="n">
+        <v>26.713</v>
+      </c>
+      <c r="AH4" s="12" t="n">
+        <v>26.028</v>
+      </c>
+      <c r="AI4" s="12" t="n">
+        <v>25.138</v>
+      </c>
+      <c r="AJ4" s="12" t="n">
+        <v>25.219</v>
+      </c>
+      <c r="AK4" s="12" t="n">
+        <v>25.366</v>
+      </c>
+      <c r="AL4" s="12" t="n">
+        <v>25.451</v>
+      </c>
+      <c r="AM4" s="12" t="n">
+        <v>25.76</v>
+      </c>
       <c r="AN4" s="12" t="n"/>
       <c r="AO4" s="12" t="n">
         <v>23.249</v>
@@ -10586,11 +10760,21 @@
       <c r="BM4" s="12" t="n">
         <v>20.303</v>
       </c>
-      <c r="BN4" s="12" t="n"/>
-      <c r="BO4" s="12" t="n"/>
-      <c r="BP4" s="12" t="n"/>
-      <c r="BQ4" s="12" t="n"/>
-      <c r="BR4" s="12" t="n"/>
+      <c r="BN4" s="12" t="n">
+        <v>20.601</v>
+      </c>
+      <c r="BO4" s="12" t="n">
+        <v>20.864</v>
+      </c>
+      <c r="BP4" s="12" t="n">
+        <v>21.68</v>
+      </c>
+      <c r="BQ4" s="12" t="n">
+        <v>22.703</v>
+      </c>
+      <c r="BR4" s="12" t="n">
+        <v>22.808</v>
+      </c>
       <c r="BS4" s="12" t="n">
         <v>22.166</v>
       </c>
@@ -10600,11 +10784,21 @@
       <c r="BU4" s="12" t="n">
         <v>23.844</v>
       </c>
-      <c r="BV4" s="12" t="n"/>
-      <c r="BW4" s="12" t="n"/>
-      <c r="BX4" s="12" t="n"/>
-      <c r="BY4" s="12" t="n"/>
-      <c r="BZ4" s="12" t="n"/>
+      <c r="BV4" s="12" t="n">
+        <v>23</v>
+      </c>
+      <c r="BW4" s="12" t="n">
+        <v>22.424</v>
+      </c>
+      <c r="BX4" s="12" t="n">
+        <v>22.049</v>
+      </c>
+      <c r="BY4" s="12" t="n">
+        <v>21.98</v>
+      </c>
+      <c r="BZ4" s="12" t="n">
+        <v>21.846</v>
+      </c>
       <c r="CA4" s="12" t="n"/>
       <c r="CB4" s="12" t="n"/>
       <c r="CC4" s="12" t="n"/>
@@ -10662,12 +10856,24 @@
       <c r="CU4" s="12" t="n">
         <v>24.284</v>
       </c>
-      <c r="CV4" s="12" t="n"/>
-      <c r="CW4" s="12" t="n"/>
-      <c r="CX4" s="12" t="n"/>
-      <c r="CY4" s="12" t="n"/>
-      <c r="CZ4" s="12" t="n"/>
-      <c r="DA4" s="12" t="n"/>
+      <c r="CV4" s="12" t="n">
+        <v>25.776</v>
+      </c>
+      <c r="CW4" s="12" t="n">
+        <v>25.691</v>
+      </c>
+      <c r="CX4" s="12" t="n">
+        <v>24.819</v>
+      </c>
+      <c r="CY4" s="12" t="n">
+        <v>42.971</v>
+      </c>
+      <c r="CZ4" s="12" t="n">
+        <v>42.101</v>
+      </c>
+      <c r="DA4" s="12" t="n">
+        <v>41.395</v>
+      </c>
       <c r="DB4" s="12" t="n"/>
       <c r="DC4" s="12" t="n"/>
       <c r="DD4" s="12" t="n"/>
@@ -10715,11 +10921,21 @@
       <c r="DT4" s="12" t="n">
         <v>23.056</v>
       </c>
-      <c r="DU4" s="12" t="n"/>
-      <c r="DV4" s="12" t="n"/>
-      <c r="DW4" s="12" t="n"/>
-      <c r="DX4" s="12" t="n"/>
-      <c r="DY4" s="12" t="n"/>
+      <c r="DU4" s="12" t="n">
+        <v>24.64</v>
+      </c>
+      <c r="DV4" s="12" t="n">
+        <v>23.612</v>
+      </c>
+      <c r="DW4" s="12" t="n">
+        <v>23.354</v>
+      </c>
+      <c r="DX4" s="12" t="n">
+        <v>24.062</v>
+      </c>
+      <c r="DY4" s="12" t="n">
+        <v>25.42</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -10727,7 +10943,9 @@
           <t>27 Apr 2026</t>
         </is>
       </c>
-      <c r="B5" s="10" t="n"/>
+      <c r="B5" s="10" t="n">
+        <v>42.856</v>
+      </c>
       <c r="C5" s="10" t="n">
         <v>43.993</v>
       </c>
@@ -10755,8 +10973,12 @@
       <c r="K5" s="10" t="n">
         <v>36.332</v>
       </c>
-      <c r="L5" s="10" t="n"/>
-      <c r="M5" s="10" t="n"/>
+      <c r="L5" s="10" t="n">
+        <v>34.481</v>
+      </c>
+      <c r="M5" s="10" t="n">
+        <v>33.396</v>
+      </c>
       <c r="N5" s="10" t="n">
         <v>42.699</v>
       </c>
@@ -10807,14 +11029,30 @@
       <c r="AE5" s="10" t="n">
         <v>32.167</v>
       </c>
-      <c r="AF5" s="10" t="n"/>
-      <c r="AG5" s="10" t="n"/>
-      <c r="AH5" s="10" t="n"/>
-      <c r="AI5" s="10" t="n"/>
-      <c r="AJ5" s="10" t="n"/>
-      <c r="AK5" s="10" t="n"/>
-      <c r="AL5" s="10" t="n"/>
-      <c r="AM5" s="10" t="n"/>
+      <c r="AF5" s="10" t="n">
+        <v>27.165</v>
+      </c>
+      <c r="AG5" s="10" t="n">
+        <v>26.709</v>
+      </c>
+      <c r="AH5" s="10" t="n">
+        <v>26.023</v>
+      </c>
+      <c r="AI5" s="10" t="n">
+        <v>25.134</v>
+      </c>
+      <c r="AJ5" s="10" t="n">
+        <v>25.215</v>
+      </c>
+      <c r="AK5" s="10" t="n">
+        <v>25.362</v>
+      </c>
+      <c r="AL5" s="10" t="n">
+        <v>25.701</v>
+      </c>
+      <c r="AM5" s="10" t="n">
+        <v>26.011</v>
+      </c>
       <c r="AN5" s="10" t="n"/>
       <c r="AO5" s="10" t="n">
         <v>23.7</v>
@@ -10879,11 +11117,21 @@
       <c r="BM5" s="10" t="n">
         <v>20.482</v>
       </c>
-      <c r="BN5" s="10" t="n"/>
-      <c r="BO5" s="10" t="n"/>
-      <c r="BP5" s="10" t="n"/>
-      <c r="BQ5" s="10" t="n"/>
-      <c r="BR5" s="10" t="n"/>
+      <c r="BN5" s="10" t="n">
+        <v>20.781</v>
+      </c>
+      <c r="BO5" s="10" t="n">
+        <v>21.045</v>
+      </c>
+      <c r="BP5" s="10" t="n">
+        <v>21.73</v>
+      </c>
+      <c r="BQ5" s="10" t="n">
+        <v>22.75</v>
+      </c>
+      <c r="BR5" s="10" t="n">
+        <v>22.855</v>
+      </c>
       <c r="BS5" s="10" t="n">
         <v>22.166</v>
       </c>
@@ -10893,11 +11141,21 @@
       <c r="BU5" s="10" t="n">
         <v>23.838</v>
       </c>
-      <c r="BV5" s="10" t="n"/>
-      <c r="BW5" s="10" t="n"/>
-      <c r="BX5" s="10" t="n"/>
-      <c r="BY5" s="10" t="n"/>
-      <c r="BZ5" s="10" t="n"/>
+      <c r="BV5" s="10" t="n">
+        <v>23.073</v>
+      </c>
+      <c r="BW5" s="10" t="n">
+        <v>22.498</v>
+      </c>
+      <c r="BX5" s="10" t="n">
+        <v>22.124</v>
+      </c>
+      <c r="BY5" s="10" t="n">
+        <v>21.905</v>
+      </c>
+      <c r="BZ5" s="10" t="n">
+        <v>21.773</v>
+      </c>
       <c r="CA5" s="10" t="n"/>
       <c r="CB5" s="10" t="n"/>
       <c r="CC5" s="10" t="n"/>
@@ -10955,12 +11213,24 @@
       <c r="CU5" s="10" t="n">
         <v>24.265</v>
       </c>
-      <c r="CV5" s="10" t="n"/>
-      <c r="CW5" s="10" t="n"/>
-      <c r="CX5" s="10" t="n"/>
-      <c r="CY5" s="10" t="n"/>
-      <c r="CZ5" s="10" t="n"/>
-      <c r="DA5" s="10" t="n"/>
+      <c r="CV5" s="10" t="n">
+        <v>25.784</v>
+      </c>
+      <c r="CW5" s="10" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="CX5" s="10" t="n">
+        <v>24.831</v>
+      </c>
+      <c r="CY5" s="10" t="n">
+        <v>44.081</v>
+      </c>
+      <c r="CZ5" s="10" t="n">
+        <v>43.195</v>
+      </c>
+      <c r="DA5" s="10" t="n">
+        <v>42.509</v>
+      </c>
       <c r="DB5" s="10" t="n"/>
       <c r="DC5" s="10" t="n"/>
       <c r="DD5" s="10" t="n"/>
@@ -11014,9 +11284,15 @@
       <c r="DV5" s="10" t="n">
         <v>23.659</v>
       </c>
-      <c r="DW5" s="10" t="n"/>
-      <c r="DX5" s="10" t="n"/>
-      <c r="DY5" s="10" t="n"/>
+      <c r="DW5" s="10" t="n">
+        <v>23.407</v>
+      </c>
+      <c r="DX5" s="10" t="n">
+        <v>24.044</v>
+      </c>
+      <c r="DY5" s="10" t="n">
+        <v>25.429</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
@@ -16474,23 +16750,43 @@
           <t>29 Apr 2026</t>
         </is>
       </c>
-      <c r="B3" s="10" t="n"/>
+      <c r="B3" s="10" t="n">
+        <v>44.964</v>
+      </c>
       <c r="C3" s="10" t="n">
         <v>46.213</v>
       </c>
       <c r="D3" s="10" t="n">
         <v>46.271</v>
       </c>
-      <c r="E3" s="10" t="n"/>
-      <c r="F3" s="10" t="n"/>
-      <c r="G3" s="10" t="n"/>
-      <c r="H3" s="10" t="n"/>
-      <c r="I3" s="10" t="n"/>
-      <c r="J3" s="10" t="n"/>
+      <c r="E3" s="10" t="n">
+        <v>46.774</v>
+      </c>
+      <c r="F3" s="10" t="n">
+        <v>46.565</v>
+      </c>
+      <c r="G3" s="10" t="n">
+        <v>46.313</v>
+      </c>
+      <c r="H3" s="10" t="n">
+        <v>45.325</v>
+      </c>
+      <c r="I3" s="10" t="n">
+        <v>45.134</v>
+      </c>
+      <c r="J3" s="10" t="n">
+        <v>46.304</v>
+      </c>
       <c r="K3" s="10" t="n"/>
-      <c r="L3" s="10" t="n"/>
-      <c r="M3" s="10" t="n"/>
-      <c r="N3" s="10" t="n"/>
+      <c r="L3" s="10" t="n">
+        <v>35.401</v>
+      </c>
+      <c r="M3" s="10" t="n">
+        <v>33.669</v>
+      </c>
+      <c r="N3" s="10" t="n">
+        <v>45.803</v>
+      </c>
       <c r="O3" s="10" t="n"/>
       <c r="P3" s="10" t="n"/>
       <c r="Q3" s="10" t="n">
@@ -16499,8 +16795,12 @@
       <c r="R3" s="10" t="n">
         <v>28.033</v>
       </c>
-      <c r="S3" s="10" t="n"/>
-      <c r="T3" s="10" t="n"/>
+      <c r="S3" s="10" t="n">
+        <v>26.297</v>
+      </c>
+      <c r="T3" s="10" t="n">
+        <v>26.357</v>
+      </c>
       <c r="U3" s="10" t="n">
         <v>23.586</v>
       </c>
@@ -16546,8 +16846,12 @@
       <c r="AM3" s="10" t="n">
         <v>26.904</v>
       </c>
-      <c r="AN3" s="10" t="n"/>
-      <c r="AO3" s="10" t="n"/>
+      <c r="AN3" s="10" t="n">
+        <v>26.808</v>
+      </c>
+      <c r="AO3" s="10" t="n">
+        <v>25.896</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
@@ -16555,25 +16859,45 @@
           <t>28 Apr 2026</t>
         </is>
       </c>
-      <c r="B4" s="12" t="n"/>
+      <c r="B4" s="12" t="n">
+        <v>42.093</v>
+      </c>
       <c r="C4" s="12" t="n">
         <v>42.949</v>
       </c>
       <c r="D4" s="12" t="n">
         <v>43.094</v>
       </c>
-      <c r="E4" s="12" t="n"/>
-      <c r="F4" s="12" t="n"/>
-      <c r="G4" s="12" t="n"/>
-      <c r="H4" s="12" t="n"/>
-      <c r="I4" s="12" t="n"/>
-      <c r="J4" s="12" t="n"/>
+      <c r="E4" s="12" t="n">
+        <v>43.564</v>
+      </c>
+      <c r="F4" s="12" t="n">
+        <v>43.355</v>
+      </c>
+      <c r="G4" s="12" t="n">
+        <v>43.177</v>
+      </c>
+      <c r="H4" s="12" t="n">
+        <v>42.343</v>
+      </c>
+      <c r="I4" s="12" t="n">
+        <v>42.165</v>
+      </c>
+      <c r="J4" s="12" t="n">
+        <v>43.66</v>
+      </c>
       <c r="K4" s="12" t="n">
         <v>35.598</v>
       </c>
-      <c r="L4" s="12" t="n"/>
-      <c r="M4" s="12" t="n"/>
-      <c r="N4" s="12" t="n"/>
+      <c r="L4" s="12" t="n">
+        <v>33.951</v>
+      </c>
+      <c r="M4" s="12" t="n">
+        <v>32.296</v>
+      </c>
+      <c r="N4" s="12" t="n">
+        <v>42.881</v>
+      </c>
       <c r="O4" s="12" t="n">
         <v>43.495</v>
       </c>
@@ -16586,8 +16910,12 @@
       <c r="R4" s="12" t="n">
         <v>27.414</v>
       </c>
-      <c r="S4" s="12" t="n"/>
-      <c r="T4" s="12" t="n"/>
+      <c r="S4" s="12" t="n">
+        <v>25.89</v>
+      </c>
+      <c r="T4" s="12" t="n">
+        <v>25.966</v>
+      </c>
       <c r="U4" s="12" t="n">
         <v>23.332</v>
       </c>
@@ -16636,7 +16964,9 @@
       <c r="AN4" s="12" t="n">
         <v>26.478</v>
       </c>
-      <c r="AO4" s="12" t="n"/>
+      <c r="AO4" s="12" t="n">
+        <v>25.443</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -16644,7 +16974,9 @@
           <t>27 Apr 2026</t>
         </is>
       </c>
-      <c r="B5" s="10" t="n"/>
+      <c r="B5" s="10" t="n">
+        <v>43.156</v>
+      </c>
       <c r="C5" s="10" t="n">
         <v>43.935</v>
       </c>
@@ -16654,17 +16986,33 @@
       <c r="E5" s="10" t="n">
         <v>44.634</v>
       </c>
-      <c r="F5" s="10" t="n"/>
-      <c r="G5" s="10" t="n"/>
-      <c r="H5" s="10" t="n"/>
-      <c r="I5" s="10" t="n"/>
-      <c r="J5" s="10" t="n"/>
+      <c r="F5" s="10" t="n">
+        <v>44.41</v>
+      </c>
+      <c r="G5" s="10" t="n">
+        <v>44.422</v>
+      </c>
+      <c r="H5" s="10" t="n">
+        <v>43.427</v>
+      </c>
+      <c r="I5" s="10" t="n">
+        <v>42.923</v>
+      </c>
+      <c r="J5" s="10" t="n">
+        <v>44.892</v>
+      </c>
       <c r="K5" s="10" t="n">
         <v>36.324</v>
       </c>
-      <c r="L5" s="10" t="n"/>
-      <c r="M5" s="10" t="n"/>
-      <c r="N5" s="10" t="n"/>
+      <c r="L5" s="10" t="n">
+        <v>34.555</v>
+      </c>
+      <c r="M5" s="10" t="n">
+        <v>33.008</v>
+      </c>
+      <c r="N5" s="10" t="n">
+        <v>44</v>
+      </c>
       <c r="O5" s="10" t="n">
         <v>44.596</v>
       </c>
@@ -16677,8 +17025,12 @@
       <c r="R5" s="10" t="n">
         <v>27.773</v>
       </c>
-      <c r="S5" s="10" t="n"/>
-      <c r="T5" s="10" t="n"/>
+      <c r="S5" s="10" t="n">
+        <v>26.031</v>
+      </c>
+      <c r="T5" s="10" t="n">
+        <v>26.272</v>
+      </c>
       <c r="U5" s="10" t="n">
         <v>23.487</v>
       </c>

</xml_diff>

<commit_message>
data: EEX curves refresh (latest trade date 2026-04-29)
</commit_message>
<xml_diff>
--- a/data/EEX_Gas_Curves.xlsx
+++ b/data/EEX_Gas_Curves.xlsx
@@ -526,7 +526,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 30 Apr 2026 13:36  ·  Source: EEX Market Data Hub (public)  ·  EUR/MWh</t>
+          <t>Generated: 30 Apr 2026 19:00  ·  Source: EEX Market Data Hub (public)  ·  EUR/MWh</t>
         </is>
       </c>
     </row>
@@ -587,7 +587,7 @@
         </is>
       </c>
       <c r="F5" s="4" t="n">
-        <v>1751</v>
+        <v>1814</v>
       </c>
     </row>
     <row r="6">
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="F6" s="6" t="n">
-        <v>537</v>
+        <v>542</v>
       </c>
     </row>
     <row r="7">
@@ -643,7 +643,7 @@
         </is>
       </c>
       <c r="F7" s="4" t="n">
-        <v>1962</v>
+        <v>2021</v>
       </c>
     </row>
     <row r="8">
@@ -671,7 +671,7 @@
         </is>
       </c>
       <c r="F8" s="6" t="n">
-        <v>553</v>
+        <v>574</v>
       </c>
     </row>
     <row r="9">
@@ -699,7 +699,7 @@
         </is>
       </c>
       <c r="F9" s="4" t="n">
-        <v>277</v>
+        <v>288</v>
       </c>
     </row>
   </sheetData>
@@ -1511,7 +1511,9 @@
           <t>29 Apr 2026</t>
         </is>
       </c>
-      <c r="B3" s="10" t="n"/>
+      <c r="B3" s="10" t="n">
+        <v>47.67</v>
+      </c>
       <c r="C3" s="10" t="n">
         <v>47.204</v>
       </c>
@@ -1539,8 +1541,12 @@
       <c r="K3" s="10" t="n">
         <v>40.018</v>
       </c>
-      <c r="L3" s="10" t="n"/>
-      <c r="M3" s="10" t="n"/>
+      <c r="L3" s="10" t="n">
+        <v>37.571</v>
+      </c>
+      <c r="M3" s="10" t="n">
+        <v>37.144</v>
+      </c>
       <c r="N3" s="10" t="n">
         <v>48.124</v>
       </c>
@@ -1574,22 +1580,46 @@
       <c r="X3" s="10" t="n">
         <v>37.577</v>
       </c>
-      <c r="Y3" s="10" t="n"/>
+      <c r="Y3" s="10" t="n">
+        <v>38.079</v>
+      </c>
       <c r="Z3" s="10" t="n">
         <v>30.52</v>
       </c>
-      <c r="AA3" s="10" t="n"/>
+      <c r="AA3" s="10" t="n">
+        <v>28.188</v>
+      </c>
       <c r="AB3" s="10" t="n"/>
-      <c r="AC3" s="10" t="n"/>
-      <c r="AD3" s="10" t="n"/>
-      <c r="AE3" s="10" t="n"/>
-      <c r="AF3" s="10" t="n"/>
-      <c r="AG3" s="10" t="n"/>
-      <c r="AH3" s="10" t="n"/>
-      <c r="AI3" s="10" t="n"/>
-      <c r="AJ3" s="10" t="n"/>
-      <c r="AK3" s="10" t="n"/>
-      <c r="AL3" s="10" t="n"/>
+      <c r="AC3" s="10" t="n">
+        <v>37.383</v>
+      </c>
+      <c r="AD3" s="10" t="n">
+        <v>36.457</v>
+      </c>
+      <c r="AE3" s="10" t="n">
+        <v>35.856</v>
+      </c>
+      <c r="AF3" s="10" t="n">
+        <v>29.599</v>
+      </c>
+      <c r="AG3" s="10" t="n">
+        <v>29.094</v>
+      </c>
+      <c r="AH3" s="10" t="n">
+        <v>28.334</v>
+      </c>
+      <c r="AI3" s="10" t="n">
+        <v>27.262</v>
+      </c>
+      <c r="AJ3" s="10" t="n">
+        <v>27.353</v>
+      </c>
+      <c r="AK3" s="10" t="n">
+        <v>27.516</v>
+      </c>
+      <c r="AL3" s="10" t="n">
+        <v>28.83</v>
+      </c>
       <c r="AM3" s="10" t="n">
         <v>29.208</v>
       </c>
@@ -1628,9 +1658,15 @@
       <c r="AZ3" s="10" t="n">
         <v>24.852</v>
       </c>
-      <c r="BA3" s="10" t="n"/>
-      <c r="BB3" s="10" t="n"/>
-      <c r="BC3" s="10" t="n"/>
+      <c r="BA3" s="10" t="n">
+        <v>24.375</v>
+      </c>
+      <c r="BB3" s="10" t="n">
+        <v>24.665</v>
+      </c>
+      <c r="BC3" s="10" t="n">
+        <v>24.89</v>
+      </c>
       <c r="BD3" s="10" t="n">
         <v>24.638</v>
       </c>
@@ -1638,7 +1674,9 @@
       <c r="BF3" s="10" t="n">
         <v>24.531</v>
       </c>
-      <c r="BG3" s="10" t="n"/>
+      <c r="BG3" s="10" t="n">
+        <v>25.961</v>
+      </c>
       <c r="BH3" s="10" t="n">
         <v>26.012</v>
       </c>
@@ -1684,17 +1722,39 @@
       <c r="BV3" s="10" t="n">
         <v>25.699</v>
       </c>
-      <c r="BW3" s="10" t="n"/>
-      <c r="BX3" s="10" t="n"/>
-      <c r="BY3" s="10" t="n"/>
-      <c r="BZ3" s="10" t="n"/>
-      <c r="CA3" s="10" t="n"/>
-      <c r="CB3" s="10" t="n"/>
-      <c r="CC3" s="10" t="n"/>
-      <c r="CD3" s="10" t="n"/>
-      <c r="CE3" s="10" t="n"/>
-      <c r="CF3" s="10" t="n"/>
-      <c r="CG3" s="10" t="n"/>
+      <c r="BW3" s="10" t="n">
+        <v>25.132</v>
+      </c>
+      <c r="BX3" s="10" t="n">
+        <v>24.923</v>
+      </c>
+      <c r="BY3" s="10" t="n">
+        <v>25.212</v>
+      </c>
+      <c r="BZ3" s="10" t="n">
+        <v>25.038</v>
+      </c>
+      <c r="CA3" s="10" t="n">
+        <v>24.098</v>
+      </c>
+      <c r="CB3" s="10" t="n">
+        <v>24.794</v>
+      </c>
+      <c r="CC3" s="10" t="n">
+        <v>24.872</v>
+      </c>
+      <c r="CD3" s="10" t="n">
+        <v>24.685</v>
+      </c>
+      <c r="CE3" s="10" t="n">
+        <v>24.444</v>
+      </c>
+      <c r="CF3" s="10" t="n">
+        <v>24.836</v>
+      </c>
+      <c r="CG3" s="10" t="n">
+        <v>25.098</v>
+      </c>
       <c r="CH3" s="10" t="n">
         <v>25.915</v>
       </c>
@@ -1739,16 +1799,36 @@
       </c>
       <c r="CV3" s="10" t="n"/>
       <c r="CW3" s="10" t="n"/>
-      <c r="CX3" s="10" t="n"/>
-      <c r="CY3" s="10" t="n"/>
-      <c r="CZ3" s="10" t="n"/>
-      <c r="DA3" s="10" t="n"/>
-      <c r="DB3" s="10" t="n"/>
-      <c r="DC3" s="10" t="n"/>
-      <c r="DD3" s="10" t="n"/>
-      <c r="DE3" s="10" t="n"/>
-      <c r="DF3" s="10" t="n"/>
-      <c r="DG3" s="10" t="n"/>
+      <c r="CX3" s="10" t="n">
+        <v>26.904</v>
+      </c>
+      <c r="CY3" s="10" t="n">
+        <v>47.722</v>
+      </c>
+      <c r="CZ3" s="10" t="n">
+        <v>47.979</v>
+      </c>
+      <c r="DA3" s="10" t="n">
+        <v>47.354</v>
+      </c>
+      <c r="DB3" s="10" t="n">
+        <v>38.506</v>
+      </c>
+      <c r="DC3" s="10" t="n">
+        <v>36.646</v>
+      </c>
+      <c r="DD3" s="10" t="n">
+        <v>37.714</v>
+      </c>
+      <c r="DE3" s="10" t="n">
+        <v>36.568</v>
+      </c>
+      <c r="DF3" s="10" t="n">
+        <v>29.01</v>
+      </c>
+      <c r="DG3" s="10" t="n">
+        <v>27.375</v>
+      </c>
       <c r="DH3" s="10" t="n"/>
       <c r="DI3" s="10" t="n"/>
       <c r="DJ3" s="10" t="n">
@@ -1790,9 +1870,15 @@
       <c r="DV3" s="10" t="n">
         <v>24.764</v>
       </c>
-      <c r="DW3" s="10" t="n"/>
-      <c r="DX3" s="10" t="n"/>
-      <c r="DY3" s="10" t="n"/>
+      <c r="DW3" s="10" t="n">
+        <v>24.846</v>
+      </c>
+      <c r="DX3" s="10" t="n">
+        <v>27.183</v>
+      </c>
+      <c r="DY3" s="10" t="n">
+        <v>27.556</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
@@ -1869,7 +1955,9 @@
       <c r="X4" s="12" t="n">
         <v>36.209</v>
       </c>
-      <c r="Y4" s="12" t="n"/>
+      <c r="Y4" s="12" t="n">
+        <v>36.707</v>
+      </c>
       <c r="Z4" s="12" t="n">
         <v>29.862</v>
       </c>
@@ -1947,9 +2035,15 @@
       <c r="AZ4" s="12" t="n">
         <v>24.808</v>
       </c>
-      <c r="BA4" s="12" t="n"/>
-      <c r="BB4" s="12" t="n"/>
-      <c r="BC4" s="12" t="n"/>
+      <c r="BA4" s="12" t="n">
+        <v>24.276</v>
+      </c>
+      <c r="BB4" s="12" t="n">
+        <v>24.562</v>
+      </c>
+      <c r="BC4" s="12" t="n">
+        <v>24.784</v>
+      </c>
       <c r="BD4" s="12" t="n">
         <v>24.438</v>
       </c>
@@ -1957,7 +2051,9 @@
       <c r="BF4" s="12" t="n">
         <v>24.112</v>
       </c>
-      <c r="BG4" s="12" t="n"/>
+      <c r="BG4" s="12" t="n">
+        <v>25.77</v>
+      </c>
       <c r="BH4" s="12" t="n">
         <v>25.82</v>
       </c>
@@ -2015,13 +2111,27 @@
       <c r="BZ4" s="12" t="n">
         <v>24.388</v>
       </c>
-      <c r="CA4" s="12" t="n"/>
-      <c r="CB4" s="12" t="n"/>
-      <c r="CC4" s="12" t="n"/>
-      <c r="CD4" s="12" t="n"/>
-      <c r="CE4" s="12" t="n"/>
-      <c r="CF4" s="12" t="n"/>
-      <c r="CG4" s="12" t="n"/>
+      <c r="CA4" s="12" t="n">
+        <v>23.472</v>
+      </c>
+      <c r="CB4" s="12" t="n">
+        <v>24.153</v>
+      </c>
+      <c r="CC4" s="12" t="n">
+        <v>24.229</v>
+      </c>
+      <c r="CD4" s="12" t="n">
+        <v>24.047</v>
+      </c>
+      <c r="CE4" s="12" t="n">
+        <v>24.106</v>
+      </c>
+      <c r="CF4" s="12" t="n">
+        <v>24.493</v>
+      </c>
+      <c r="CG4" s="12" t="n">
+        <v>24.752</v>
+      </c>
       <c r="CH4" s="12" t="n">
         <v>25.915</v>
       </c>
@@ -2088,10 +2198,18 @@
       <c r="DC4" s="12" t="n">
         <v>35.276</v>
       </c>
-      <c r="DD4" s="12" t="n"/>
-      <c r="DE4" s="12" t="n"/>
-      <c r="DF4" s="12" t="n"/>
-      <c r="DG4" s="12" t="n"/>
+      <c r="DD4" s="12" t="n">
+        <v>36.34</v>
+      </c>
+      <c r="DE4" s="12" t="n">
+        <v>35.446</v>
+      </c>
+      <c r="DF4" s="12" t="n">
+        <v>28.055</v>
+      </c>
+      <c r="DG4" s="12" t="n">
+        <v>26.932</v>
+      </c>
       <c r="DH4" s="12" t="n"/>
       <c r="DI4" s="12" t="n"/>
       <c r="DJ4" s="12" t="n">
@@ -2398,7 +2516,9 @@
       <c r="CF5" s="10" t="n">
         <v>24.556</v>
       </c>
-      <c r="CG5" s="10" t="n"/>
+      <c r="CG5" s="10" t="n">
+        <v>24.814</v>
+      </c>
       <c r="CH5" s="10" t="n">
         <v>25.915</v>
       </c>
@@ -2468,9 +2588,15 @@
       <c r="DD5" s="10" t="n">
         <v>37.102</v>
       </c>
-      <c r="DE5" s="10" t="n"/>
-      <c r="DF5" s="10" t="n"/>
-      <c r="DG5" s="10" t="n"/>
+      <c r="DE5" s="10" t="n">
+        <v>36.297</v>
+      </c>
+      <c r="DF5" s="10" t="n">
+        <v>28.118</v>
+      </c>
+      <c r="DG5" s="10" t="n">
+        <v>26.995</v>
+      </c>
       <c r="DH5" s="10" t="n"/>
       <c r="DI5" s="10" t="n"/>
       <c r="DJ5" s="10" t="n">
@@ -7642,13 +7768,21 @@
       <c r="U3" s="10" t="n">
         <v>25.939</v>
       </c>
-      <c r="V3" s="10" t="n"/>
-      <c r="W3" s="10" t="n"/>
+      <c r="V3" s="10" t="n">
+        <v>24.748</v>
+      </c>
+      <c r="W3" s="10" t="n">
+        <v>25.9</v>
+      </c>
       <c r="X3" s="10" t="n">
         <v>24.502</v>
       </c>
-      <c r="Y3" s="10" t="n"/>
-      <c r="Z3" s="10" t="n"/>
+      <c r="Y3" s="10" t="n">
+        <v>23.728</v>
+      </c>
+      <c r="Z3" s="10" t="n">
+        <v>25.074</v>
+      </c>
       <c r="AA3" s="10" t="n">
         <v>24.413</v>
       </c>
@@ -7761,7 +7895,9 @@
       <c r="U4" s="12" t="n">
         <v>25.685</v>
       </c>
-      <c r="V4" s="12" t="n"/>
+      <c r="V4" s="12" t="n">
+        <v>24.578</v>
+      </c>
       <c r="W4" s="12" t="n">
         <v>25.69</v>
       </c>
@@ -10299,7 +10435,9 @@
       <c r="O3" s="10" t="n">
         <v>44.363</v>
       </c>
-      <c r="P3" s="10" t="n"/>
+      <c r="P3" s="10" t="n">
+        <v>43.806</v>
+      </c>
       <c r="Q3" s="10" t="n">
         <v>37.598</v>
       </c>
@@ -10330,8 +10468,12 @@
       <c r="Z3" s="10" t="n">
         <v>28.006</v>
       </c>
-      <c r="AA3" s="10" t="n"/>
-      <c r="AB3" s="10" t="n"/>
+      <c r="AA3" s="10" t="n">
+        <v>26.279</v>
+      </c>
+      <c r="AB3" s="10" t="n">
+        <v>26.142</v>
+      </c>
       <c r="AC3" s="10" t="n">
         <v>34.188</v>
       </c>
@@ -10369,15 +10511,33 @@
       <c r="AO3" s="10" t="n">
         <v>23.39</v>
       </c>
-      <c r="AP3" s="10" t="n"/>
-      <c r="AQ3" s="10" t="n"/>
-      <c r="AR3" s="10" t="n"/>
-      <c r="AS3" s="10" t="n"/>
-      <c r="AT3" s="10" t="n"/>
-      <c r="AU3" s="10" t="n"/>
-      <c r="AV3" s="10" t="n"/>
-      <c r="AW3" s="10" t="n"/>
-      <c r="AX3" s="10" t="n"/>
+      <c r="AP3" s="10" t="n">
+        <v>22.187</v>
+      </c>
+      <c r="AQ3" s="10" t="n">
+        <v>23.666</v>
+      </c>
+      <c r="AR3" s="10" t="n">
+        <v>26.823</v>
+      </c>
+      <c r="AS3" s="10" t="n">
+        <v>26.118</v>
+      </c>
+      <c r="AT3" s="10" t="n">
+        <v>25.661</v>
+      </c>
+      <c r="AU3" s="10" t="n">
+        <v>22.78</v>
+      </c>
+      <c r="AV3" s="10" t="n">
+        <v>22.359</v>
+      </c>
+      <c r="AW3" s="10" t="n">
+        <v>21.729</v>
+      </c>
+      <c r="AX3" s="10" t="n">
+        <v>21.989</v>
+      </c>
       <c r="AY3" s="10" t="n">
         <v>22.065</v>
       </c>
@@ -10396,8 +10556,12 @@
       <c r="BD3" s="10" t="n">
         <v>22.629</v>
       </c>
-      <c r="BE3" s="10" t="n"/>
-      <c r="BF3" s="10" t="n"/>
+      <c r="BE3" s="10" t="n">
+        <v>21.759</v>
+      </c>
+      <c r="BF3" s="10" t="n">
+        <v>22.863</v>
+      </c>
       <c r="BG3" s="10" t="n">
         <v>24.433</v>
       </c>
@@ -10437,7 +10601,9 @@
       <c r="BS3" s="10" t="n">
         <v>22.704</v>
       </c>
-      <c r="BT3" s="10" t="n"/>
+      <c r="BT3" s="10" t="n">
+        <v>22.198</v>
+      </c>
       <c r="BU3" s="10" t="n">
         <v>24.136</v>
       </c>
@@ -10456,13 +10622,21 @@
       <c r="BZ3" s="10" t="n">
         <v>22.495</v>
       </c>
-      <c r="CA3" s="10" t="n"/>
-      <c r="CB3" s="10" t="n"/>
-      <c r="CC3" s="10" t="n"/>
+      <c r="CA3" s="10" t="n">
+        <v>21.609</v>
+      </c>
+      <c r="CB3" s="10" t="n">
+        <v>21.808</v>
+      </c>
+      <c r="CC3" s="10" t="n">
+        <v>21.88</v>
+      </c>
       <c r="CD3" s="10" t="n"/>
       <c r="CE3" s="10" t="n"/>
       <c r="CF3" s="10" t="n"/>
-      <c r="CG3" s="10" t="n"/>
+      <c r="CG3" s="10" t="n">
+        <v>23.547</v>
+      </c>
       <c r="CH3" s="10" t="n">
         <v>23.915</v>
       </c>
@@ -10523,13 +10697,27 @@
       <c r="DA3" s="10" t="n">
         <v>44.183</v>
       </c>
-      <c r="DB3" s="10" t="n"/>
-      <c r="DC3" s="10" t="n"/>
-      <c r="DD3" s="10" t="n"/>
-      <c r="DE3" s="10" t="n"/>
-      <c r="DF3" s="10" t="n"/>
-      <c r="DG3" s="10" t="n"/>
-      <c r="DH3" s="10" t="n"/>
+      <c r="DB3" s="10" t="n">
+        <v>36.226</v>
+      </c>
+      <c r="DC3" s="10" t="n">
+        <v>34.421</v>
+      </c>
+      <c r="DD3" s="10" t="n">
+        <v>34.674</v>
+      </c>
+      <c r="DE3" s="10" t="n">
+        <v>33.424</v>
+      </c>
+      <c r="DF3" s="10" t="n">
+        <v>27.239</v>
+      </c>
+      <c r="DG3" s="10" t="n">
+        <v>25.33</v>
+      </c>
+      <c r="DH3" s="10" t="n">
+        <v>26.083</v>
+      </c>
       <c r="DI3" s="10" t="n">
         <v>26.203</v>
       </c>
@@ -10663,8 +10851,12 @@
       <c r="Z4" s="12" t="n">
         <v>27.411</v>
       </c>
-      <c r="AA4" s="12" t="n"/>
-      <c r="AB4" s="12" t="n"/>
+      <c r="AA4" s="12" t="n">
+        <v>25.935</v>
+      </c>
+      <c r="AB4" s="12" t="n">
+        <v>25.799</v>
+      </c>
       <c r="AC4" s="12" t="n">
         <v>32.802</v>
       </c>
@@ -10702,12 +10894,24 @@
       <c r="AO4" s="12" t="n">
         <v>23.249</v>
       </c>
-      <c r="AP4" s="12" t="n"/>
-      <c r="AQ4" s="12" t="n"/>
-      <c r="AR4" s="12" t="n"/>
-      <c r="AS4" s="12" t="n"/>
-      <c r="AT4" s="12" t="n"/>
-      <c r="AU4" s="12" t="n"/>
+      <c r="AP4" s="12" t="n">
+        <v>22.13</v>
+      </c>
+      <c r="AQ4" s="12" t="n">
+        <v>23.513</v>
+      </c>
+      <c r="AR4" s="12" t="n">
+        <v>26.47</v>
+      </c>
+      <c r="AS4" s="12" t="n">
+        <v>25.78</v>
+      </c>
+      <c r="AT4" s="12" t="n">
+        <v>25.332</v>
+      </c>
+      <c r="AU4" s="12" t="n">
+        <v>22.716</v>
+      </c>
       <c r="AV4" s="12" t="n">
         <v>22.3</v>
       </c>
@@ -10735,7 +10939,9 @@
       <c r="BD4" s="12" t="n">
         <v>22.429</v>
       </c>
-      <c r="BE4" s="12" t="n"/>
+      <c r="BE4" s="12" t="n">
+        <v>21.611</v>
+      </c>
       <c r="BF4" s="12" t="n">
         <v>22.443</v>
       </c>
@@ -10799,9 +11005,15 @@
       <c r="BZ4" s="12" t="n">
         <v>21.846</v>
       </c>
-      <c r="CA4" s="12" t="n"/>
-      <c r="CB4" s="12" t="n"/>
-      <c r="CC4" s="12" t="n"/>
+      <c r="CA4" s="12" t="n">
+        <v>20.984</v>
+      </c>
+      <c r="CB4" s="12" t="n">
+        <v>21.168</v>
+      </c>
+      <c r="CC4" s="12" t="n">
+        <v>21.238</v>
+      </c>
       <c r="CD4" s="12" t="n">
         <v>22.136</v>
       </c>
@@ -10874,11 +11086,21 @@
       <c r="DA4" s="12" t="n">
         <v>41.395</v>
       </c>
-      <c r="DB4" s="12" t="n"/>
-      <c r="DC4" s="12" t="n"/>
-      <c r="DD4" s="12" t="n"/>
-      <c r="DE4" s="12" t="n"/>
-      <c r="DF4" s="12" t="n"/>
+      <c r="DB4" s="12" t="n">
+        <v>34.487</v>
+      </c>
+      <c r="DC4" s="12" t="n">
+        <v>32.976</v>
+      </c>
+      <c r="DD4" s="12" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="DE4" s="12" t="n">
+        <v>32.073</v>
+      </c>
+      <c r="DF4" s="12" t="n">
+        <v>26.637</v>
+      </c>
       <c r="DG4" s="12" t="n">
         <v>25.24</v>
       </c>
@@ -11018,8 +11240,12 @@
       <c r="Z5" s="10" t="n">
         <v>27.657</v>
       </c>
-      <c r="AA5" s="10" t="n"/>
-      <c r="AB5" s="10" t="n"/>
+      <c r="AA5" s="10" t="n">
+        <v>25.931</v>
+      </c>
+      <c r="AB5" s="10" t="n">
+        <v>26.211</v>
+      </c>
       <c r="AC5" s="10" t="n">
         <v>33.557</v>
       </c>
@@ -11057,11 +11283,21 @@
       <c r="AO5" s="10" t="n">
         <v>23.7</v>
       </c>
-      <c r="AP5" s="10" t="n"/>
-      <c r="AQ5" s="10" t="n"/>
-      <c r="AR5" s="10" t="n"/>
-      <c r="AS5" s="10" t="n"/>
-      <c r="AT5" s="10" t="n"/>
+      <c r="AP5" s="10" t="n">
+        <v>22.552</v>
+      </c>
+      <c r="AQ5" s="10" t="n">
+        <v>23.86</v>
+      </c>
+      <c r="AR5" s="10" t="n">
+        <v>27.048</v>
+      </c>
+      <c r="AS5" s="10" t="n">
+        <v>26.356</v>
+      </c>
+      <c r="AT5" s="10" t="n">
+        <v>25.906</v>
+      </c>
       <c r="AU5" s="10" t="n">
         <v>23.137</v>
       </c>
@@ -11092,7 +11328,9 @@
       <c r="BD5" s="10" t="n">
         <v>22.609</v>
       </c>
-      <c r="BE5" s="10" t="n"/>
+      <c r="BE5" s="10" t="n">
+        <v>21.795</v>
+      </c>
       <c r="BF5" s="10" t="n">
         <v>22.504</v>
       </c>
@@ -11156,9 +11394,15 @@
       <c r="BZ5" s="10" t="n">
         <v>21.773</v>
       </c>
-      <c r="CA5" s="10" t="n"/>
-      <c r="CB5" s="10" t="n"/>
-      <c r="CC5" s="10" t="n"/>
+      <c r="CA5" s="10" t="n">
+        <v>20.919</v>
+      </c>
+      <c r="CB5" s="10" t="n">
+        <v>21.097</v>
+      </c>
+      <c r="CC5" s="10" t="n">
+        <v>21.166</v>
+      </c>
       <c r="CD5" s="10" t="n">
         <v>22.066</v>
       </c>
@@ -11231,11 +11475,21 @@
       <c r="DA5" s="10" t="n">
         <v>42.509</v>
       </c>
-      <c r="DB5" s="10" t="n"/>
-      <c r="DC5" s="10" t="n"/>
-      <c r="DD5" s="10" t="n"/>
-      <c r="DE5" s="10" t="n"/>
-      <c r="DF5" s="10" t="n"/>
+      <c r="DB5" s="10" t="n">
+        <v>35.209</v>
+      </c>
+      <c r="DC5" s="10" t="n">
+        <v>33.76</v>
+      </c>
+      <c r="DD5" s="10" t="n">
+        <v>33.971</v>
+      </c>
+      <c r="DE5" s="10" t="n">
+        <v>32.815</v>
+      </c>
+      <c r="DF5" s="10" t="n">
+        <v>26.633</v>
+      </c>
       <c r="DG5" s="10" t="n">
         <v>25.236</v>
       </c>
@@ -16777,7 +17031,9 @@
       <c r="J3" s="10" t="n">
         <v>46.304</v>
       </c>
-      <c r="K3" s="10" t="n"/>
+      <c r="K3" s="10" t="n">
+        <v>37.39</v>
+      </c>
       <c r="L3" s="10" t="n">
         <v>35.401</v>
       </c>
@@ -16787,8 +17043,12 @@
       <c r="N3" s="10" t="n">
         <v>45.803</v>
       </c>
-      <c r="O3" s="10" t="n"/>
-      <c r="P3" s="10" t="n"/>
+      <c r="O3" s="10" t="n">
+        <v>46.375</v>
+      </c>
+      <c r="P3" s="10" t="n">
+        <v>40.984</v>
+      </c>
       <c r="Q3" s="10" t="n">
         <v>37.486</v>
       </c>
@@ -16804,18 +17064,30 @@
       <c r="U3" s="10" t="n">
         <v>23.586</v>
       </c>
-      <c r="V3" s="10" t="n"/>
-      <c r="W3" s="10" t="n"/>
+      <c r="V3" s="10" t="n">
+        <v>22.289</v>
+      </c>
+      <c r="W3" s="10" t="n">
+        <v>23.261</v>
+      </c>
       <c r="X3" s="10" t="n">
         <v>22.674</v>
       </c>
-      <c r="Y3" s="10" t="n"/>
-      <c r="Z3" s="10" t="n"/>
+      <c r="Y3" s="10" t="n">
+        <v>21.011</v>
+      </c>
+      <c r="Z3" s="10" t="n">
+        <v>22.17</v>
+      </c>
       <c r="AA3" s="10" t="n">
         <v>23.148</v>
       </c>
-      <c r="AB3" s="10" t="n"/>
-      <c r="AC3" s="10" t="n"/>
+      <c r="AB3" s="10" t="n">
+        <v>21.293</v>
+      </c>
+      <c r="AC3" s="10" t="n">
+        <v>24.22</v>
+      </c>
       <c r="AD3" s="10" t="n">
         <v>24.315</v>
       </c>
@@ -16919,18 +17191,30 @@
       <c r="U4" s="12" t="n">
         <v>23.332</v>
       </c>
-      <c r="V4" s="12" t="n"/>
-      <c r="W4" s="12" t="n"/>
+      <c r="V4" s="12" t="n">
+        <v>22.119</v>
+      </c>
+      <c r="W4" s="12" t="n">
+        <v>23.051</v>
+      </c>
       <c r="X4" s="12" t="n">
         <v>22.474</v>
       </c>
-      <c r="Y4" s="12" t="n"/>
-      <c r="Z4" s="12" t="n"/>
+      <c r="Y4" s="12" t="n">
+        <v>20.863</v>
+      </c>
+      <c r="Z4" s="12" t="n">
+        <v>21.75</v>
+      </c>
       <c r="AA4" s="12" t="n">
         <v>22.61</v>
       </c>
-      <c r="AB4" s="12" t="n"/>
-      <c r="AC4" s="12" t="n"/>
+      <c r="AB4" s="12" t="n">
+        <v>20.651</v>
+      </c>
+      <c r="AC4" s="12" t="n">
+        <v>23.929</v>
+      </c>
       <c r="AD4" s="12" t="n">
         <v>24.315</v>
       </c>
@@ -17034,18 +17318,30 @@
       <c r="U5" s="10" t="n">
         <v>23.487</v>
       </c>
-      <c r="V5" s="10" t="n"/>
-      <c r="W5" s="10" t="n"/>
+      <c r="V5" s="10" t="n">
+        <v>22.245</v>
+      </c>
+      <c r="W5" s="10" t="n">
+        <v>23.249</v>
+      </c>
       <c r="X5" s="10" t="n">
         <v>22.654</v>
       </c>
-      <c r="Y5" s="10" t="n"/>
-      <c r="Z5" s="10" t="n"/>
+      <c r="Y5" s="10" t="n">
+        <v>21.047</v>
+      </c>
+      <c r="Z5" s="10" t="n">
+        <v>21.812</v>
+      </c>
       <c r="AA5" s="10" t="n">
         <v>22.61</v>
       </c>
-      <c r="AB5" s="10" t="n"/>
-      <c r="AC5" s="10" t="n"/>
+      <c r="AB5" s="10" t="n">
+        <v>20.583</v>
+      </c>
+      <c r="AC5" s="10" t="n">
+        <v>23.918</v>
+      </c>
       <c r="AD5" s="10" t="n">
         <v>24.315</v>
       </c>
@@ -18857,7 +19153,9 @@
       <c r="G3" s="10" t="n">
         <v>46.29</v>
       </c>
-      <c r="H3" s="10" t="n"/>
+      <c r="H3" s="10" t="n">
+        <v>45.357</v>
+      </c>
       <c r="I3" s="10" t="n">
         <v>37.622</v>
       </c>
@@ -18882,11 +19180,21 @@
       <c r="P3" s="10" t="n">
         <v>24.039</v>
       </c>
-      <c r="Q3" s="10" t="n"/>
-      <c r="R3" s="10" t="n"/>
-      <c r="S3" s="10" t="n"/>
-      <c r="T3" s="10" t="n"/>
-      <c r="U3" s="10" t="n"/>
+      <c r="Q3" s="10" t="n">
+        <v>23.305</v>
+      </c>
+      <c r="R3" s="10" t="n">
+        <v>23.401</v>
+      </c>
+      <c r="S3" s="10" t="n">
+        <v>24.515</v>
+      </c>
+      <c r="T3" s="10" t="n">
+        <v>46.212</v>
+      </c>
+      <c r="U3" s="10" t="n">
+        <v>45.541</v>
+      </c>
       <c r="V3" s="10" t="n"/>
       <c r="W3" s="10" t="n"/>
       <c r="X3" s="10" t="n"/>
@@ -18921,7 +19229,9 @@
       <c r="G4" s="12" t="n">
         <v>42.856</v>
       </c>
-      <c r="H4" s="12" t="n"/>
+      <c r="H4" s="12" t="n">
+        <v>42.314</v>
+      </c>
       <c r="I4" s="12" t="n">
         <v>35.819</v>
       </c>
@@ -18952,9 +19262,15 @@
       <c r="R4" s="12" t="n">
         <v>22.863</v>
       </c>
-      <c r="S4" s="12" t="n"/>
-      <c r="T4" s="12" t="n"/>
-      <c r="U4" s="12" t="n"/>
+      <c r="S4" s="12" t="n">
+        <v>24.515</v>
+      </c>
+      <c r="T4" s="12" t="n">
+        <v>42.936</v>
+      </c>
+      <c r="U4" s="12" t="n">
+        <v>42.544</v>
+      </c>
       <c r="V4" s="12" t="n"/>
       <c r="W4" s="12" t="n"/>
       <c r="X4" s="12" t="n"/>
@@ -19028,7 +19344,9 @@
       <c r="T5" s="10" t="n">
         <v>44.209</v>
       </c>
-      <c r="U5" s="10" t="n"/>
+      <c r="U5" s="10" t="n">
+        <v>43.906</v>
+      </c>
       <c r="V5" s="10" t="n"/>
       <c r="W5" s="10" t="n"/>
       <c r="X5" s="10" t="n"/>

</xml_diff>

<commit_message>
data: EEX curves refresh (latest trade date 2026-04-30)
</commit_message>
<xml_diff>
--- a/data/EEX_Gas_Curves.xlsx
+++ b/data/EEX_Gas_Curves.xlsx
@@ -526,7 +526,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 01 May 2026 09:32  ·  Source: EEX Market Data Hub (public)  ·  EUR/MWh</t>
+          <t>Generated: 01 May 2026 10:06  ·  Source: EEX Market Data Hub (public)  ·  EUR/MWh</t>
         </is>
       </c>
     </row>
@@ -587,7 +587,7 @@
         </is>
       </c>
       <c r="F5" s="4" t="n">
-        <v>1928</v>
+        <v>1930</v>
       </c>
     </row>
     <row r="6">
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="F6" s="6" t="n">
-        <v>577</v>
+        <v>578</v>
       </c>
     </row>
     <row r="7">
@@ -643,7 +643,7 @@
         </is>
       </c>
       <c r="F7" s="4" t="n">
-        <v>2095</v>
+        <v>2102</v>
       </c>
     </row>
     <row r="8">
@@ -671,7 +671,7 @@
         </is>
       </c>
       <c r="F8" s="6" t="n">
-        <v>603</v>
+        <v>612</v>
       </c>
     </row>
     <row r="9">
@@ -699,7 +699,7 @@
         </is>
       </c>
       <c r="F9" s="4" t="n">
-        <v>319</v>
+        <v>321</v>
       </c>
     </row>
   </sheetData>
@@ -1589,7 +1589,9 @@
         <v>28.597</v>
       </c>
       <c r="AC3" s="10" t="n"/>
-      <c r="AD3" s="10" t="n"/>
+      <c r="AD3" s="10" t="n">
+        <v>36.018</v>
+      </c>
       <c r="AE3" s="10" t="n">
         <v>35.427</v>
       </c>
@@ -1828,7 +1830,9 @@
       <c r="DR3" s="10" t="n"/>
       <c r="DS3" s="10" t="n"/>
       <c r="DT3" s="10" t="n"/>
-      <c r="DU3" s="10" t="n"/>
+      <c r="DU3" s="10" t="n">
+        <v>24.712</v>
+      </c>
       <c r="DV3" s="10" t="n">
         <v>26.793</v>
       </c>
@@ -8157,7 +8161,9 @@
         <v>25.78</v>
       </c>
       <c r="W3" s="10" t="n"/>
-      <c r="X3" s="10" t="n"/>
+      <c r="X3" s="10" t="n">
+        <v>25.679</v>
+      </c>
       <c r="Y3" s="10" t="n">
         <v>24.233</v>
       </c>
@@ -10994,7 +11000,9 @@
         <v>33.561</v>
       </c>
       <c r="AD3" s="10" t="n"/>
-      <c r="AE3" s="10" t="n"/>
+      <c r="AE3" s="10" t="n">
+        <v>32.155</v>
+      </c>
       <c r="AF3" s="10" t="n"/>
       <c r="AG3" s="10" t="n"/>
       <c r="AH3" s="10" t="n"/>
@@ -11063,7 +11071,9 @@
       <c r="BK3" s="10" t="n">
         <v>22.413</v>
       </c>
-      <c r="BL3" s="10" t="n"/>
+      <c r="BL3" s="10" t="n">
+        <v>22.207</v>
+      </c>
       <c r="BM3" s="10" t="n"/>
       <c r="BN3" s="10" t="n"/>
       <c r="BO3" s="10" t="n"/>
@@ -11132,8 +11142,12 @@
       <c r="CR3" s="10" t="n">
         <v>23.129</v>
       </c>
-      <c r="CS3" s="10" t="n"/>
-      <c r="CT3" s="10" t="n"/>
+      <c r="CS3" s="10" t="n">
+        <v>23.718</v>
+      </c>
+      <c r="CT3" s="10" t="n">
+        <v>23.993</v>
+      </c>
       <c r="CU3" s="10" t="n"/>
       <c r="CV3" s="10" t="n"/>
       <c r="CW3" s="10" t="n"/>
@@ -11183,9 +11197,15 @@
       <c r="DQ3" s="10" t="n">
         <v>22.747</v>
       </c>
-      <c r="DR3" s="10" t="n"/>
-      <c r="DS3" s="10" t="n"/>
-      <c r="DT3" s="10" t="n"/>
+      <c r="DR3" s="10" t="n">
+        <v>22.048</v>
+      </c>
+      <c r="DS3" s="10" t="n">
+        <v>21.948</v>
+      </c>
+      <c r="DT3" s="10" t="n">
+        <v>23.322</v>
+      </c>
       <c r="DU3" s="10" t="n"/>
       <c r="DV3" s="10" t="n"/>
       <c r="DW3" s="10" t="n"/>
@@ -17549,7 +17569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AO20"/>
+  <dimension ref="A1:AP20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -17593,6 +17613,7 @@
     <col width="10" customWidth="1" min="39" max="39"/>
     <col width="10" customWidth="1" min="40" max="40"/>
     <col width="10" customWidth="1" min="41" max="41"/>
+    <col width="10" customWidth="1" min="42" max="42"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -17690,120 +17711,125 @@
       </c>
       <c r="R2" s="3" t="inlineStr">
         <is>
+          <t>May-27</t>
+        </is>
+      </c>
+      <c r="S2" s="3" t="inlineStr">
+        <is>
           <t>Cal-28</t>
         </is>
       </c>
-      <c r="S2" s="3" t="inlineStr">
+      <c r="T2" s="3" t="inlineStr">
         <is>
           <t>Sum-28</t>
         </is>
       </c>
-      <c r="T2" s="3" t="inlineStr">
+      <c r="U2" s="3" t="inlineStr">
         <is>
           <t>Win-28</t>
         </is>
       </c>
-      <c r="U2" s="3" t="inlineStr">
+      <c r="V2" s="3" t="inlineStr">
         <is>
           <t>Cal-29</t>
         </is>
       </c>
-      <c r="V2" s="3" t="inlineStr">
+      <c r="W2" s="3" t="inlineStr">
         <is>
           <t>Sum-29</t>
         </is>
       </c>
-      <c r="W2" s="3" t="inlineStr">
+      <c r="X2" s="3" t="inlineStr">
         <is>
           <t>Win-29</t>
         </is>
       </c>
-      <c r="X2" s="3" t="inlineStr">
+      <c r="Y2" s="3" t="inlineStr">
         <is>
           <t>Cal-30</t>
         </is>
       </c>
-      <c r="Y2" s="3" t="inlineStr">
+      <c r="Z2" s="3" t="inlineStr">
         <is>
           <t>Sum-30</t>
         </is>
       </c>
-      <c r="Z2" s="3" t="inlineStr">
+      <c r="AA2" s="3" t="inlineStr">
         <is>
           <t>Win-30</t>
         </is>
       </c>
-      <c r="AA2" s="3" t="inlineStr">
+      <c r="AB2" s="3" t="inlineStr">
         <is>
           <t>Cal-31</t>
         </is>
       </c>
-      <c r="AB2" s="3" t="inlineStr">
+      <c r="AC2" s="3" t="inlineStr">
         <is>
           <t>Sum-31</t>
         </is>
       </c>
-      <c r="AC2" s="3" t="inlineStr">
+      <c r="AD2" s="3" t="inlineStr">
         <is>
           <t>Win-31</t>
         </is>
       </c>
-      <c r="AD2" s="3" t="inlineStr">
+      <c r="AE2" s="3" t="inlineStr">
         <is>
           <t>Cal-32</t>
         </is>
       </c>
-      <c r="AE2" s="3" t="inlineStr">
+      <c r="AF2" s="3" t="inlineStr">
         <is>
           <t>2026-03</t>
         </is>
       </c>
-      <c r="AF2" s="3" t="inlineStr">
+      <c r="AG2" s="3" t="inlineStr">
         <is>
           <t>2026-04</t>
         </is>
       </c>
-      <c r="AG2" s="3" t="inlineStr">
+      <c r="AH2" s="3" t="inlineStr">
         <is>
           <t>2027-01</t>
         </is>
       </c>
-      <c r="AH2" s="3" t="inlineStr">
+      <c r="AI2" s="3" t="inlineStr">
         <is>
           <t>2027-02</t>
         </is>
       </c>
-      <c r="AI2" s="3" t="inlineStr">
+      <c r="AJ2" s="3" t="inlineStr">
         <is>
           <t>2027-03</t>
         </is>
       </c>
-      <c r="AJ2" s="3" t="inlineStr">
+      <c r="AK2" s="3" t="inlineStr">
         <is>
           <t>2027-04</t>
         </is>
       </c>
-      <c r="AK2" s="3" t="inlineStr">
+      <c r="AL2" s="3" t="inlineStr">
         <is>
           <t>2028-01</t>
         </is>
       </c>
-      <c r="AL2" s="3" t="inlineStr">
+      <c r="AM2" s="3" t="inlineStr">
         <is>
           <t>2028-02</t>
         </is>
       </c>
-      <c r="AM2" s="3" t="inlineStr">
+      <c r="AN2" s="3" t="inlineStr">
         <is>
           <t>2028-03</t>
         </is>
       </c>
-      <c r="AN2" s="3" t="inlineStr">
+      <c r="AO2" s="3" t="inlineStr">
         <is>
           <t>2028-04</t>
         </is>
       </c>
-      <c r="AO2" s="3" t="inlineStr">
+      <c r="AP2" s="3" t="inlineStr">
         <is>
           <t>2029-01</t>
         </is>
@@ -17857,60 +17883,79 @@
         <v>40.171</v>
       </c>
       <c r="Q3" s="10" t="n"/>
-      <c r="R3" s="10" t="n"/>
+      <c r="R3" s="10" t="n">
+        <v>34.701</v>
+      </c>
       <c r="S3" s="10" t="n">
+        <v>27.467</v>
+      </c>
+      <c r="T3" s="10" t="n">
         <v>25.71</v>
       </c>
-      <c r="T3" s="10" t="n">
+      <c r="U3" s="10" t="n">
         <v>25.922</v>
       </c>
-      <c r="U3" s="10" t="n"/>
       <c r="V3" s="10" t="n">
+        <v>23.359</v>
+      </c>
+      <c r="W3" s="10" t="n">
         <v>22.205</v>
       </c>
-      <c r="W3" s="10" t="n">
+      <c r="X3" s="10" t="n">
         <v>23.04</v>
       </c>
-      <c r="X3" s="10" t="n"/>
       <c r="Y3" s="10" t="n">
+        <v>22.405</v>
+      </c>
+      <c r="Z3" s="10" t="n">
         <v>20.691</v>
       </c>
-      <c r="Z3" s="10" t="n">
+      <c r="AA3" s="10" t="n">
         <v>21.897</v>
       </c>
-      <c r="AA3" s="10" t="n"/>
       <c r="AB3" s="10" t="n">
+        <v>22.96</v>
+      </c>
+      <c r="AC3" s="10" t="n">
         <v>21.093</v>
       </c>
-      <c r="AC3" s="10" t="n">
+      <c r="AD3" s="10" t="n">
         <v>24.144</v>
       </c>
-      <c r="AD3" s="10" t="n"/>
-      <c r="AE3" s="10" t="n"/>
-      <c r="AF3" s="10" t="n"/>
-      <c r="AG3" s="10" t="n"/>
+      <c r="AE3" s="10" t="n">
+        <v>24.315</v>
+      </c>
+      <c r="AF3" s="10" t="n">
+        <v>45.923</v>
+      </c>
+      <c r="AG3" s="10" t="n">
+        <v>45.087</v>
+      </c>
       <c r="AH3" s="10" t="n">
+        <v>43.496</v>
+      </c>
+      <c r="AI3" s="10" t="n">
         <v>34.714</v>
       </c>
-      <c r="AI3" s="10" t="n">
+      <c r="AJ3" s="10" t="n">
         <v>34.434</v>
       </c>
-      <c r="AJ3" s="10" t="n">
+      <c r="AK3" s="10" t="n">
         <v>33.837</v>
       </c>
-      <c r="AK3" s="10" t="n">
+      <c r="AL3" s="10" t="n">
         <v>32.075</v>
       </c>
-      <c r="AL3" s="10" t="n">
+      <c r="AM3" s="10" t="n">
         <v>25.086</v>
       </c>
-      <c r="AM3" s="10" t="n">
+      <c r="AN3" s="10" t="n">
         <v>26.328</v>
       </c>
-      <c r="AN3" s="10" t="n">
+      <c r="AO3" s="10" t="n">
         <v>26.404</v>
       </c>
-      <c r="AO3" s="10" t="n">
+      <c r="AP3" s="10" t="n">
         <v>25.429</v>
       </c>
     </row>
@@ -17968,76 +18013,77 @@
       <c r="Q4" s="12" t="n">
         <v>37.486</v>
       </c>
-      <c r="R4" s="12" t="n">
+      <c r="R4" s="12" t="n"/>
+      <c r="S4" s="12" t="n">
         <v>28.033</v>
       </c>
-      <c r="S4" s="12" t="n">
+      <c r="T4" s="12" t="n">
         <v>26.297</v>
       </c>
-      <c r="T4" s="12" t="n">
+      <c r="U4" s="12" t="n">
         <v>26.357</v>
       </c>
-      <c r="U4" s="12" t="n">
+      <c r="V4" s="12" t="n">
         <v>23.586</v>
       </c>
-      <c r="V4" s="12" t="n">
+      <c r="W4" s="12" t="n">
         <v>22.289</v>
       </c>
-      <c r="W4" s="12" t="n">
+      <c r="X4" s="12" t="n">
         <v>23.261</v>
       </c>
-      <c r="X4" s="12" t="n">
+      <c r="Y4" s="12" t="n">
         <v>22.674</v>
       </c>
-      <c r="Y4" s="12" t="n">
+      <c r="Z4" s="12" t="n">
         <v>21.011</v>
       </c>
-      <c r="Z4" s="12" t="n">
+      <c r="AA4" s="12" t="n">
         <v>22.17</v>
       </c>
-      <c r="AA4" s="12" t="n">
+      <c r="AB4" s="12" t="n">
         <v>23.148</v>
       </c>
-      <c r="AB4" s="12" t="n">
+      <c r="AC4" s="12" t="n">
         <v>21.293</v>
       </c>
-      <c r="AC4" s="12" t="n">
+      <c r="AD4" s="12" t="n">
         <v>24.22</v>
       </c>
-      <c r="AD4" s="12" t="n">
+      <c r="AE4" s="12" t="n">
         <v>24.315</v>
       </c>
-      <c r="AE4" s="12" t="n">
+      <c r="AF4" s="12" t="n">
         <v>46.553</v>
       </c>
-      <c r="AF4" s="12" t="n">
+      <c r="AG4" s="12" t="n">
         <v>45.593</v>
       </c>
-      <c r="AG4" s="12" t="n">
+      <c r="AH4" s="12" t="n">
         <v>44.321</v>
       </c>
-      <c r="AH4" s="12" t="n">
+      <c r="AI4" s="12" t="n">
         <v>35.617</v>
       </c>
-      <c r="AI4" s="12" t="n">
+      <c r="AJ4" s="12" t="n">
         <v>35.188</v>
       </c>
-      <c r="AJ4" s="12" t="n">
+      <c r="AK4" s="12" t="n">
         <v>34.567</v>
       </c>
-      <c r="AK4" s="12" t="n">
+      <c r="AL4" s="12" t="n">
         <v>32.761</v>
       </c>
-      <c r="AL4" s="12" t="n">
+      <c r="AM4" s="12" t="n">
         <v>25.684</v>
       </c>
-      <c r="AM4" s="12" t="n">
+      <c r="AN4" s="12" t="n">
         <v>26.904</v>
       </c>
-      <c r="AN4" s="12" t="n">
+      <c r="AO4" s="12" t="n">
         <v>26.808</v>
       </c>
-      <c r="AO4" s="12" t="n">
+      <c r="AP4" s="12" t="n">
         <v>25.896</v>
       </c>
     </row>
@@ -18095,76 +18141,77 @@
       <c r="Q5" s="10" t="n">
         <v>35.797</v>
       </c>
-      <c r="R5" s="10" t="n">
+      <c r="R5" s="10" t="n"/>
+      <c r="S5" s="10" t="n">
         <v>27.414</v>
       </c>
-      <c r="S5" s="10" t="n">
+      <c r="T5" s="10" t="n">
         <v>25.89</v>
       </c>
-      <c r="T5" s="10" t="n">
+      <c r="U5" s="10" t="n">
         <v>25.966</v>
       </c>
-      <c r="U5" s="10" t="n">
+      <c r="V5" s="10" t="n">
         <v>23.332</v>
       </c>
-      <c r="V5" s="10" t="n">
+      <c r="W5" s="10" t="n">
         <v>22.119</v>
       </c>
-      <c r="W5" s="10" t="n">
+      <c r="X5" s="10" t="n">
         <v>23.051</v>
       </c>
-      <c r="X5" s="10" t="n">
+      <c r="Y5" s="10" t="n">
         <v>22.474</v>
       </c>
-      <c r="Y5" s="10" t="n">
+      <c r="Z5" s="10" t="n">
         <v>20.863</v>
       </c>
-      <c r="Z5" s="10" t="n">
+      <c r="AA5" s="10" t="n">
         <v>21.75</v>
       </c>
-      <c r="AA5" s="10" t="n">
+      <c r="AB5" s="10" t="n">
         <v>22.61</v>
       </c>
-      <c r="AB5" s="10" t="n">
+      <c r="AC5" s="10" t="n">
         <v>20.651</v>
       </c>
-      <c r="AC5" s="10" t="n">
+      <c r="AD5" s="10" t="n">
         <v>23.929</v>
       </c>
-      <c r="AD5" s="10" t="n">
+      <c r="AE5" s="10" t="n">
         <v>24.315</v>
       </c>
-      <c r="AE5" s="10" t="n">
+      <c r="AF5" s="10" t="n">
         <v>43.367</v>
       </c>
-      <c r="AF5" s="10" t="n">
+      <c r="AG5" s="10" t="n">
         <v>42.729</v>
       </c>
-      <c r="AG5" s="10" t="n">
+      <c r="AH5" s="10" t="n">
         <v>41.443</v>
       </c>
-      <c r="AH5" s="10" t="n">
+      <c r="AI5" s="10" t="n">
         <v>34.054</v>
       </c>
-      <c r="AI5" s="10" t="n">
+      <c r="AJ5" s="10" t="n">
         <v>33.849</v>
       </c>
-      <c r="AJ5" s="10" t="n">
+      <c r="AK5" s="10" t="n">
         <v>33.156</v>
       </c>
-      <c r="AK5" s="10" t="n">
+      <c r="AL5" s="10" t="n">
         <v>31.427</v>
       </c>
-      <c r="AL5" s="10" t="n">
+      <c r="AM5" s="10" t="n">
         <v>25.019</v>
       </c>
-      <c r="AM5" s="10" t="n">
+      <c r="AN5" s="10" t="n">
         <v>26.751</v>
       </c>
-      <c r="AN5" s="10" t="n">
+      <c r="AO5" s="10" t="n">
         <v>26.478</v>
       </c>
-      <c r="AO5" s="10" t="n">
+      <c r="AP5" s="10" t="n">
         <v>25.443</v>
       </c>
     </row>
@@ -18222,76 +18269,77 @@
       <c r="Q6" s="12" t="n">
         <v>36.548</v>
       </c>
-      <c r="R6" s="12" t="n">
+      <c r="R6" s="12" t="n"/>
+      <c r="S6" s="12" t="n">
         <v>27.773</v>
       </c>
-      <c r="S6" s="12" t="n">
+      <c r="T6" s="12" t="n">
         <v>26.031</v>
       </c>
-      <c r="T6" s="12" t="n">
+      <c r="U6" s="12" t="n">
         <v>26.272</v>
       </c>
-      <c r="U6" s="12" t="n">
+      <c r="V6" s="12" t="n">
         <v>23.487</v>
       </c>
-      <c r="V6" s="12" t="n">
+      <c r="W6" s="12" t="n">
         <v>22.245</v>
       </c>
-      <c r="W6" s="12" t="n">
+      <c r="X6" s="12" t="n">
         <v>23.249</v>
       </c>
-      <c r="X6" s="12" t="n">
+      <c r="Y6" s="12" t="n">
         <v>22.654</v>
       </c>
-      <c r="Y6" s="12" t="n">
+      <c r="Z6" s="12" t="n">
         <v>21.047</v>
       </c>
-      <c r="Z6" s="12" t="n">
+      <c r="AA6" s="12" t="n">
         <v>21.812</v>
       </c>
-      <c r="AA6" s="12" t="n">
+      <c r="AB6" s="12" t="n">
         <v>22.61</v>
       </c>
-      <c r="AB6" s="12" t="n">
+      <c r="AC6" s="12" t="n">
         <v>20.583</v>
       </c>
-      <c r="AC6" s="12" t="n">
+      <c r="AD6" s="12" t="n">
         <v>23.918</v>
       </c>
-      <c r="AD6" s="12" t="n">
+      <c r="AE6" s="12" t="n">
         <v>24.315</v>
       </c>
-      <c r="AE6" s="12" t="n">
+      <c r="AF6" s="12" t="n">
         <v>44.489</v>
       </c>
-      <c r="AF6" s="12" t="n">
+      <c r="AG6" s="12" t="n">
         <v>43.756</v>
       </c>
-      <c r="AG6" s="12" t="n">
+      <c r="AH6" s="12" t="n">
         <v>42.543</v>
       </c>
-      <c r="AH6" s="12" t="n">
+      <c r="AI6" s="12" t="n">
         <v>34.629</v>
       </c>
-      <c r="AI6" s="12" t="n">
+      <c r="AJ6" s="12" t="n">
         <v>34.482</v>
       </c>
-      <c r="AJ6" s="12" t="n">
+      <c r="AK6" s="12" t="n">
         <v>33.758</v>
       </c>
-      <c r="AK6" s="12" t="n">
+      <c r="AL6" s="12" t="n">
         <v>32.25</v>
       </c>
-      <c r="AL6" s="12" t="n">
+      <c r="AM6" s="12" t="n">
         <v>25.16</v>
       </c>
-      <c r="AM6" s="12" t="n">
+      <c r="AN6" s="12" t="n">
         <v>26.892</v>
       </c>
-      <c r="AN6" s="12" t="n">
+      <c r="AO6" s="12" t="n">
         <v>26.81</v>
       </c>
-      <c r="AO6" s="12" t="n">
+      <c r="AP6" s="12" t="n">
         <v>25.723</v>
       </c>
     </row>
@@ -18344,10 +18392,10 @@
       <c r="P7" s="10" t="n"/>
       <c r="Q7" s="10" t="n"/>
       <c r="R7" s="10" t="n"/>
-      <c r="S7" s="10" t="n">
+      <c r="S7" s="10" t="n"/>
+      <c r="T7" s="10" t="n">
         <v>26.545</v>
       </c>
-      <c r="T7" s="10" t="n"/>
       <c r="U7" s="10" t="n"/>
       <c r="V7" s="10" t="n"/>
       <c r="W7" s="10" t="n"/>
@@ -18361,28 +18409,29 @@
       <c r="AE7" s="10" t="n"/>
       <c r="AF7" s="10" t="n"/>
       <c r="AG7" s="10" t="n"/>
-      <c r="AH7" s="10" t="n">
+      <c r="AH7" s="10" t="n"/>
+      <c r="AI7" s="10" t="n">
         <v>35.099</v>
       </c>
-      <c r="AI7" s="10" t="n">
+      <c r="AJ7" s="10" t="n">
         <v>34.846</v>
       </c>
-      <c r="AJ7" s="10" t="n">
+      <c r="AK7" s="10" t="n">
         <v>34.118</v>
       </c>
-      <c r="AK7" s="10" t="n">
+      <c r="AL7" s="10" t="n">
         <v>32.595</v>
       </c>
-      <c r="AL7" s="10" t="n">
+      <c r="AM7" s="10" t="n">
         <v>25.679</v>
       </c>
-      <c r="AM7" s="10" t="n">
+      <c r="AN7" s="10" t="n">
         <v>27.401</v>
       </c>
-      <c r="AN7" s="10" t="n">
+      <c r="AO7" s="10" t="n">
         <v>27.255</v>
       </c>
-      <c r="AO7" s="10" t="n">
+      <c r="AP7" s="10" t="n">
         <v>26.145</v>
       </c>
     </row>
@@ -18438,62 +18487,63 @@
       <c r="Q8" s="12" t="n">
         <v>35.942</v>
       </c>
-      <c r="R8" s="12" t="n">
+      <c r="R8" s="12" t="n"/>
+      <c r="S8" s="12" t="n">
         <v>27.303</v>
       </c>
-      <c r="S8" s="12" t="n">
+      <c r="T8" s="12" t="n">
         <v>25.636</v>
       </c>
-      <c r="T8" s="12" t="n"/>
-      <c r="U8" s="12" t="n">
+      <c r="U8" s="12" t="n"/>
+      <c r="V8" s="12" t="n">
         <v>23.187</v>
       </c>
-      <c r="V8" s="12" t="n"/>
       <c r="W8" s="12" t="n"/>
-      <c r="X8" s="12" t="n">
+      <c r="X8" s="12" t="n"/>
+      <c r="Y8" s="12" t="n">
         <v>22.524</v>
       </c>
-      <c r="Y8" s="12" t="n"/>
       <c r="Z8" s="12" t="n"/>
-      <c r="AA8" s="12" t="n">
+      <c r="AA8" s="12" t="n"/>
+      <c r="AB8" s="12" t="n">
         <v>23.248</v>
       </c>
-      <c r="AB8" s="12" t="n"/>
       <c r="AC8" s="12" t="n"/>
-      <c r="AD8" s="12" t="n">
+      <c r="AD8" s="12" t="n"/>
+      <c r="AE8" s="12" t="n">
         <v>24.315</v>
       </c>
-      <c r="AE8" s="12" t="n">
+      <c r="AF8" s="12" t="n">
         <v>44.069</v>
       </c>
-      <c r="AF8" s="12" t="n">
+      <c r="AG8" s="12" t="n">
         <v>43.179</v>
       </c>
-      <c r="AG8" s="12" t="n">
+      <c r="AH8" s="12" t="n">
         <v>41.846</v>
       </c>
-      <c r="AH8" s="12" t="n">
+      <c r="AI8" s="12" t="n">
         <v>34.119</v>
       </c>
-      <c r="AI8" s="12" t="n">
+      <c r="AJ8" s="12" t="n">
         <v>33.956</v>
       </c>
-      <c r="AJ8" s="12" t="n">
+      <c r="AK8" s="12" t="n">
         <v>33.107</v>
       </c>
-      <c r="AK8" s="12" t="n">
+      <c r="AL8" s="12" t="n">
         <v>31.568</v>
       </c>
-      <c r="AL8" s="12" t="n">
+      <c r="AM8" s="12" t="n">
         <v>24.76</v>
       </c>
-      <c r="AM8" s="12" t="n">
+      <c r="AN8" s="12" t="n">
         <v>26.502</v>
       </c>
-      <c r="AN8" s="12" t="n">
+      <c r="AO8" s="12" t="n">
         <v>26.402</v>
       </c>
-      <c r="AO8" s="12" t="n">
+      <c r="AP8" s="12" t="n">
         <v>25.515</v>
       </c>
     </row>
@@ -18549,62 +18599,63 @@
       <c r="Q9" s="10" t="n">
         <v>35.691</v>
       </c>
-      <c r="R9" s="10" t="n">
+      <c r="R9" s="10" t="n"/>
+      <c r="S9" s="10" t="n">
         <v>27.265</v>
       </c>
-      <c r="S9" s="10" t="n">
+      <c r="T9" s="10" t="n">
         <v>25.6</v>
       </c>
-      <c r="T9" s="10" t="n"/>
-      <c r="U9" s="10" t="n">
+      <c r="U9" s="10" t="n"/>
+      <c r="V9" s="10" t="n">
         <v>23.265</v>
       </c>
-      <c r="V9" s="10" t="n"/>
       <c r="W9" s="10" t="n"/>
-      <c r="X9" s="10" t="n">
+      <c r="X9" s="10" t="n"/>
+      <c r="Y9" s="10" t="n">
         <v>22.364</v>
       </c>
-      <c r="Y9" s="10" t="n"/>
       <c r="Z9" s="10" t="n"/>
-      <c r="AA9" s="10" t="n">
+      <c r="AA9" s="10" t="n"/>
+      <c r="AB9" s="10" t="n">
         <v>23.248</v>
       </c>
-      <c r="AB9" s="10" t="n"/>
       <c r="AC9" s="10" t="n"/>
-      <c r="AD9" s="10" t="n">
+      <c r="AD9" s="10" t="n"/>
+      <c r="AE9" s="10" t="n">
         <v>24.315</v>
       </c>
-      <c r="AE9" s="10" t="n">
+      <c r="AF9" s="10" t="n">
         <v>43.259</v>
       </c>
-      <c r="AF9" s="10" t="n">
+      <c r="AG9" s="10" t="n">
         <v>42.384</v>
       </c>
-      <c r="AG9" s="10" t="n">
+      <c r="AH9" s="10" t="n">
         <v>40.958</v>
       </c>
-      <c r="AH9" s="10" t="n">
+      <c r="AI9" s="10" t="n">
         <v>33.876</v>
       </c>
-      <c r="AI9" s="10" t="n">
+      <c r="AJ9" s="10" t="n">
         <v>33.707</v>
       </c>
-      <c r="AJ9" s="10" t="n">
+      <c r="AK9" s="10" t="n">
         <v>32.812</v>
       </c>
-      <c r="AK9" s="10" t="n">
+      <c r="AL9" s="10" t="n">
         <v>31.513</v>
       </c>
-      <c r="AL9" s="10" t="n">
+      <c r="AM9" s="10" t="n">
         <v>24.722</v>
       </c>
-      <c r="AM9" s="10" t="n">
+      <c r="AN9" s="10" t="n">
         <v>26.468</v>
       </c>
-      <c r="AN9" s="10" t="n">
+      <c r="AO9" s="10" t="n">
         <v>26.376</v>
       </c>
-      <c r="AO9" s="10" t="n">
+      <c r="AP9" s="10" t="n">
         <v>25.494</v>
       </c>
     </row>
@@ -18662,68 +18713,69 @@
       <c r="Q10" s="12" t="n">
         <v>34.251</v>
       </c>
-      <c r="R10" s="12" t="n">
+      <c r="R10" s="12" t="n"/>
+      <c r="S10" s="12" t="n">
         <v>26.527</v>
       </c>
-      <c r="S10" s="12" t="n">
+      <c r="T10" s="12" t="n">
         <v>25.024</v>
       </c>
-      <c r="T10" s="12" t="n">
+      <c r="U10" s="12" t="n">
         <v>25.322</v>
       </c>
-      <c r="U10" s="12" t="n">
+      <c r="V10" s="12" t="n">
         <v>22.996</v>
       </c>
-      <c r="V10" s="12" t="n">
+      <c r="W10" s="12" t="n">
         <v>21.825</v>
       </c>
-      <c r="W10" s="12" t="n">
+      <c r="X10" s="12" t="n">
         <v>23.013</v>
       </c>
-      <c r="X10" s="12" t="n">
+      <c r="Y10" s="12" t="n">
         <v>22.762</v>
       </c>
-      <c r="Y10" s="12" t="n"/>
       <c r="Z10" s="12" t="n"/>
-      <c r="AA10" s="12" t="n">
+      <c r="AA10" s="12" t="n"/>
+      <c r="AB10" s="12" t="n">
         <v>23.248</v>
       </c>
-      <c r="AB10" s="12" t="n"/>
       <c r="AC10" s="12" t="n"/>
-      <c r="AD10" s="12" t="n">
+      <c r="AD10" s="12" t="n"/>
+      <c r="AE10" s="12" t="n">
         <v>24.315</v>
       </c>
-      <c r="AE10" s="12" t="n">
+      <c r="AF10" s="12" t="n">
         <v>41.517</v>
       </c>
-      <c r="AF10" s="12" t="n">
+      <c r="AG10" s="12" t="n">
         <v>40.519</v>
       </c>
-      <c r="AG10" s="12" t="n">
+      <c r="AH10" s="12" t="n">
         <v>39.5</v>
       </c>
-      <c r="AH10" s="12" t="n">
+      <c r="AI10" s="12" t="n">
         <v>32.551</v>
       </c>
-      <c r="AI10" s="12" t="n">
+      <c r="AJ10" s="12" t="n">
         <v>32.487</v>
       </c>
-      <c r="AJ10" s="12" t="n">
+      <c r="AK10" s="12" t="n">
         <v>31.559</v>
       </c>
-      <c r="AK10" s="12" t="n">
+      <c r="AL10" s="12" t="n">
         <v>30.329</v>
       </c>
-      <c r="AL10" s="12" t="n">
+      <c r="AM10" s="12" t="n">
         <v>24.14</v>
       </c>
-      <c r="AM10" s="12" t="n">
+      <c r="AN10" s="12" t="n">
         <v>25.898</v>
       </c>
-      <c r="AN10" s="12" t="n">
+      <c r="AO10" s="12" t="n">
         <v>25.757</v>
       </c>
-      <c r="AO10" s="12" t="n">
+      <c r="AP10" s="12" t="n">
         <v>24.877</v>
       </c>
     </row>
@@ -18781,76 +18833,77 @@
       <c r="Q11" s="10" t="n">
         <v>33.425</v>
       </c>
-      <c r="R11" s="10" t="n">
+      <c r="R11" s="10" t="n"/>
+      <c r="S11" s="10" t="n">
         <v>26.31</v>
       </c>
-      <c r="S11" s="10" t="n">
+      <c r="T11" s="10" t="n">
         <v>24.936</v>
       </c>
-      <c r="T11" s="10" t="n">
+      <c r="U11" s="10" t="n">
         <v>25.362</v>
       </c>
-      <c r="U11" s="10" t="n">
+      <c r="V11" s="10" t="n">
         <v>22.913</v>
       </c>
-      <c r="V11" s="10" t="n">
+      <c r="W11" s="10" t="n">
         <v>21.599</v>
       </c>
-      <c r="W11" s="10" t="n">
+      <c r="X11" s="10" t="n">
         <v>22.934</v>
       </c>
-      <c r="X11" s="10" t="n">
+      <c r="Y11" s="10" t="n">
         <v>22.549</v>
       </c>
-      <c r="Y11" s="10" t="n">
+      <c r="Z11" s="10" t="n">
         <v>20.723</v>
       </c>
-      <c r="Z11" s="10" t="n">
+      <c r="AA11" s="10" t="n">
         <v>22.309</v>
       </c>
-      <c r="AA11" s="10" t="n">
+      <c r="AB11" s="10" t="n">
         <v>23.235</v>
       </c>
-      <c r="AB11" s="10" t="n">
+      <c r="AC11" s="10" t="n">
         <v>21.331</v>
       </c>
-      <c r="AC11" s="10" t="n">
+      <c r="AD11" s="10" t="n">
         <v>24.349</v>
       </c>
-      <c r="AD11" s="10" t="n">
+      <c r="AE11" s="10" t="n">
         <v>24.315</v>
       </c>
-      <c r="AE11" s="10" t="n">
+      <c r="AF11" s="10" t="n">
         <v>39.832</v>
       </c>
-      <c r="AF11" s="10" t="n">
+      <c r="AG11" s="10" t="n">
         <v>39.3</v>
       </c>
-      <c r="AG11" s="10" t="n">
+      <c r="AH11" s="10" t="n">
         <v>38.103</v>
       </c>
-      <c r="AH11" s="10" t="n">
+      <c r="AI11" s="10" t="n">
         <v>31.665</v>
       </c>
-      <c r="AI11" s="10" t="n">
+      <c r="AJ11" s="10" t="n">
         <v>31.929</v>
       </c>
-      <c r="AJ11" s="10" t="n">
+      <c r="AK11" s="10" t="n">
         <v>31.035</v>
       </c>
-      <c r="AK11" s="10" t="n">
+      <c r="AL11" s="10" t="n">
         <v>29.613</v>
       </c>
-      <c r="AL11" s="10" t="n">
+      <c r="AM11" s="10" t="n">
         <v>24.05</v>
       </c>
-      <c r="AM11" s="10" t="n">
+      <c r="AN11" s="10" t="n">
         <v>25.812</v>
       </c>
-      <c r="AN11" s="10" t="n">
+      <c r="AO11" s="10" t="n">
         <v>25.777</v>
       </c>
-      <c r="AO11" s="10" t="n">
+      <c r="AP11" s="10" t="n">
         <v>24.937</v>
       </c>
     </row>
@@ -18907,55 +18960,56 @@
       <c r="R12" s="12" t="n"/>
       <c r="S12" s="12" t="n"/>
       <c r="T12" s="12" t="n"/>
-      <c r="U12" s="12" t="n">
+      <c r="U12" s="12" t="n"/>
+      <c r="V12" s="12" t="n">
         <v>22.863</v>
       </c>
-      <c r="V12" s="12" t="n"/>
       <c r="W12" s="12" t="n"/>
-      <c r="X12" s="12" t="n">
+      <c r="X12" s="12" t="n"/>
+      <c r="Y12" s="12" t="n">
         <v>22.474</v>
       </c>
-      <c r="Y12" s="12" t="n"/>
       <c r="Z12" s="12" t="n"/>
-      <c r="AA12" s="12" t="n">
+      <c r="AA12" s="12" t="n"/>
+      <c r="AB12" s="12" t="n">
         <v>23.36</v>
       </c>
-      <c r="AB12" s="12" t="n"/>
       <c r="AC12" s="12" t="n"/>
-      <c r="AD12" s="12" t="n">
+      <c r="AD12" s="12" t="n"/>
+      <c r="AE12" s="12" t="n">
         <v>24.4</v>
       </c>
-      <c r="AE12" s="12" t="n">
+      <c r="AF12" s="12" t="n">
         <v>38.24</v>
       </c>
-      <c r="AF12" s="12" t="n">
+      <c r="AG12" s="12" t="n">
         <v>38.055</v>
       </c>
-      <c r="AG12" s="12" t="n">
+      <c r="AH12" s="12" t="n">
         <v>37.163</v>
       </c>
-      <c r="AH12" s="12" t="n">
+      <c r="AI12" s="12" t="n">
         <v>30.898</v>
       </c>
-      <c r="AI12" s="12" t="n">
+      <c r="AJ12" s="12" t="n">
         <v>31.457</v>
       </c>
-      <c r="AJ12" s="12" t="n">
+      <c r="AK12" s="12" t="n">
         <v>30.429</v>
       </c>
-      <c r="AK12" s="12" t="n">
+      <c r="AL12" s="12" t="n">
         <v>28.948</v>
       </c>
-      <c r="AL12" s="12" t="n">
+      <c r="AM12" s="12" t="n">
         <v>23.615</v>
       </c>
-      <c r="AM12" s="12" t="n">
+      <c r="AN12" s="12" t="n">
         <v>25.387</v>
       </c>
-      <c r="AN12" s="12" t="n">
+      <c r="AO12" s="12" t="n">
         <v>25.341</v>
       </c>
-      <c r="AO12" s="12" t="n">
+      <c r="AP12" s="12" t="n">
         <v>24.425</v>
       </c>
     </row>
@@ -19010,61 +19064,62 @@
         <v>34.162</v>
       </c>
       <c r="R13" s="10" t="n"/>
-      <c r="S13" s="10" t="n">
+      <c r="S13" s="10" t="n"/>
+      <c r="T13" s="10" t="n">
         <v>25.137</v>
       </c>
-      <c r="T13" s="10" t="n">
+      <c r="U13" s="10" t="n">
         <v>25.76</v>
       </c>
-      <c r="U13" s="10" t="n">
+      <c r="V13" s="10" t="n">
         <v>23.483</v>
       </c>
-      <c r="V13" s="10" t="n"/>
       <c r="W13" s="10" t="n"/>
-      <c r="X13" s="10" t="n">
+      <c r="X13" s="10" t="n"/>
+      <c r="Y13" s="10" t="n">
         <v>22.974</v>
       </c>
-      <c r="Y13" s="10" t="n"/>
       <c r="Z13" s="10" t="n"/>
-      <c r="AA13" s="10" t="n">
+      <c r="AA13" s="10" t="n"/>
+      <c r="AB13" s="10" t="n">
         <v>23.36</v>
       </c>
-      <c r="AB13" s="10" t="n"/>
       <c r="AC13" s="10" t="n"/>
-      <c r="AD13" s="10" t="n">
+      <c r="AD13" s="10" t="n"/>
+      <c r="AE13" s="10" t="n">
         <v>24.4</v>
       </c>
-      <c r="AE13" s="10" t="n">
+      <c r="AF13" s="10" t="n">
         <v>41.975</v>
       </c>
-      <c r="AF13" s="10" t="n">
+      <c r="AG13" s="10" t="n">
         <v>41.17</v>
       </c>
-      <c r="AG13" s="10" t="n">
+      <c r="AH13" s="10" t="n">
         <v>39.953</v>
       </c>
-      <c r="AH13" s="10" t="n">
+      <c r="AI13" s="10" t="n">
         <v>32.857</v>
       </c>
-      <c r="AI13" s="10" t="n">
+      <c r="AJ13" s="10" t="n">
         <v>32.849</v>
       </c>
-      <c r="AJ13" s="10" t="n">
+      <c r="AK13" s="10" t="n">
         <v>31.81</v>
       </c>
-      <c r="AK13" s="10" t="n">
+      <c r="AL13" s="10" t="n">
         <v>30.228</v>
       </c>
-      <c r="AL13" s="10" t="n">
+      <c r="AM13" s="10" t="n">
         <v>24.093</v>
       </c>
-      <c r="AM13" s="10" t="n">
+      <c r="AN13" s="10" t="n">
         <v>26.169</v>
       </c>
-      <c r="AN13" s="10" t="n">
+      <c r="AO13" s="10" t="n">
         <v>26.105</v>
       </c>
-      <c r="AO13" s="10" t="n">
+      <c r="AP13" s="10" t="n">
         <v>25.407</v>
       </c>
     </row>
@@ -19120,70 +19175,71 @@
       <c r="Q14" s="12" t="n">
         <v>32.927</v>
       </c>
-      <c r="R14" s="12" t="n">
+      <c r="R14" s="12" t="n"/>
+      <c r="S14" s="12" t="n">
         <v>26.163</v>
       </c>
-      <c r="S14" s="12" t="n">
+      <c r="T14" s="12" t="n">
         <v>24.89</v>
       </c>
-      <c r="T14" s="12" t="n">
+      <c r="U14" s="12" t="n">
         <v>25.33</v>
       </c>
-      <c r="U14" s="12" t="n">
+      <c r="V14" s="12" t="n">
         <v>23.191</v>
       </c>
-      <c r="V14" s="12" t="n"/>
       <c r="W14" s="12" t="n"/>
-      <c r="X14" s="12" t="n">
+      <c r="X14" s="12" t="n"/>
+      <c r="Y14" s="12" t="n">
         <v>22.724</v>
       </c>
-      <c r="Y14" s="12" t="n"/>
-      <c r="Z14" s="12" t="n">
+      <c r="Z14" s="12" t="n"/>
+      <c r="AA14" s="12" t="n">
         <v>22.467</v>
       </c>
-      <c r="AA14" s="12" t="n">
+      <c r="AB14" s="12" t="n">
         <v>23.61</v>
       </c>
-      <c r="AB14" s="12" t="n">
+      <c r="AC14" s="12" t="n">
         <v>21.797</v>
       </c>
-      <c r="AC14" s="12" t="n">
+      <c r="AD14" s="12" t="n">
         <v>24.609</v>
       </c>
-      <c r="AD14" s="12" t="n">
+      <c r="AE14" s="12" t="n">
         <v>24.4</v>
       </c>
-      <c r="AE14" s="12" t="n">
+      <c r="AF14" s="12" t="n">
         <v>40.793</v>
       </c>
-      <c r="AF14" s="12" t="n">
+      <c r="AG14" s="12" t="n">
         <v>40.037</v>
       </c>
-      <c r="AG14" s="12" t="n">
+      <c r="AH14" s="12" t="n">
         <v>38.896</v>
       </c>
-      <c r="AH14" s="12" t="n">
+      <c r="AI14" s="12" t="n">
         <v>31.781</v>
       </c>
-      <c r="AI14" s="12" t="n">
+      <c r="AJ14" s="12" t="n">
         <v>31.873</v>
       </c>
-      <c r="AJ14" s="12" t="n">
+      <c r="AK14" s="12" t="n">
         <v>30.578</v>
       </c>
-      <c r="AK14" s="12" t="n">
+      <c r="AL14" s="12" t="n">
         <v>28.997</v>
       </c>
-      <c r="AL14" s="12" t="n">
+      <c r="AM14" s="12" t="n">
         <v>23.844</v>
       </c>
-      <c r="AM14" s="12" t="n">
+      <c r="AN14" s="12" t="n">
         <v>25.924</v>
       </c>
-      <c r="AN14" s="12" t="n">
+      <c r="AO14" s="12" t="n">
         <v>25.894</v>
       </c>
-      <c r="AO14" s="12" t="n">
+      <c r="AP14" s="12" t="n">
         <v>24.754</v>
       </c>
     </row>
@@ -19241,70 +19297,71 @@
       <c r="Q15" s="10" t="n">
         <v>33.391</v>
       </c>
-      <c r="R15" s="10" t="n">
+      <c r="R15" s="10" t="n"/>
+      <c r="S15" s="10" t="n">
         <v>26.199</v>
       </c>
-      <c r="S15" s="10" t="n">
+      <c r="T15" s="10" t="n">
         <v>24.744</v>
       </c>
-      <c r="T15" s="10" t="n">
+      <c r="U15" s="10" t="n">
         <v>25.245</v>
       </c>
-      <c r="U15" s="10" t="n">
+      <c r="V15" s="10" t="n">
         <v>23.238</v>
       </c>
-      <c r="V15" s="10" t="n"/>
       <c r="W15" s="10" t="n"/>
-      <c r="X15" s="10" t="n">
+      <c r="X15" s="10" t="n"/>
+      <c r="Y15" s="10" t="n">
         <v>22.724</v>
       </c>
-      <c r="Y15" s="10" t="n"/>
-      <c r="Z15" s="10" t="n">
+      <c r="Z15" s="10" t="n"/>
+      <c r="AA15" s="10" t="n">
         <v>22.286</v>
       </c>
-      <c r="AA15" s="10" t="n">
+      <c r="AB15" s="10" t="n">
         <v>23.36</v>
       </c>
-      <c r="AB15" s="10" t="n">
+      <c r="AC15" s="10" t="n">
         <v>21.467</v>
       </c>
-      <c r="AC15" s="10" t="n">
+      <c r="AD15" s="10" t="n">
         <v>24.513</v>
       </c>
-      <c r="AD15" s="10" t="n">
+      <c r="AE15" s="10" t="n">
         <v>24.4</v>
       </c>
-      <c r="AE15" s="10" t="n">
+      <c r="AF15" s="10" t="n">
         <v>42.542</v>
       </c>
-      <c r="AF15" s="10" t="n">
+      <c r="AG15" s="10" t="n">
         <v>41.813</v>
       </c>
-      <c r="AG15" s="10" t="n">
+      <c r="AH15" s="10" t="n">
         <v>39.948</v>
       </c>
-      <c r="AH15" s="10" t="n">
+      <c r="AI15" s="10" t="n">
         <v>32.22</v>
       </c>
-      <c r="AI15" s="10" t="n">
+      <c r="AJ15" s="10" t="n">
         <v>32.237</v>
       </c>
-      <c r="AJ15" s="10" t="n">
+      <c r="AK15" s="10" t="n">
         <v>31.455</v>
       </c>
-      <c r="AK15" s="10" t="n">
+      <c r="AL15" s="10" t="n">
         <v>29.474</v>
       </c>
-      <c r="AL15" s="10" t="n">
+      <c r="AM15" s="10" t="n">
         <v>23.697</v>
       </c>
-      <c r="AM15" s="10" t="n">
+      <c r="AN15" s="10" t="n">
         <v>25.779</v>
       </c>
-      <c r="AN15" s="10" t="n">
+      <c r="AO15" s="10" t="n">
         <v>25.861</v>
       </c>
-      <c r="AO15" s="10" t="n">
+      <c r="AP15" s="10" t="n">
         <v>24.615</v>
       </c>
     </row>
@@ -19362,74 +19419,75 @@
       <c r="Q16" s="12" t="n">
         <v>35.007</v>
       </c>
-      <c r="R16" s="12" t="n">
+      <c r="R16" s="12" t="n"/>
+      <c r="S16" s="12" t="n">
         <v>26.85</v>
       </c>
-      <c r="S16" s="12" t="n">
+      <c r="T16" s="12" t="n">
         <v>25.226</v>
       </c>
-      <c r="T16" s="12" t="n">
+      <c r="U16" s="12" t="n">
         <v>25.609</v>
       </c>
-      <c r="U16" s="12" t="n">
+      <c r="V16" s="12" t="n">
         <v>23.495</v>
       </c>
-      <c r="V16" s="12" t="n">
+      <c r="W16" s="12" t="n">
         <v>22.419</v>
       </c>
-      <c r="W16" s="12" t="n">
+      <c r="X16" s="12" t="n">
         <v>23.435</v>
       </c>
-      <c r="X16" s="12" t="n">
+      <c r="Y16" s="12" t="n">
         <v>22.974</v>
       </c>
-      <c r="Y16" s="12" t="n"/>
-      <c r="Z16" s="12" t="n">
+      <c r="Z16" s="12" t="n"/>
+      <c r="AA16" s="12" t="n">
         <v>22.928</v>
       </c>
-      <c r="AA16" s="12" t="n">
+      <c r="AB16" s="12" t="n">
         <v>23.11</v>
       </c>
-      <c r="AB16" s="12" t="n">
+      <c r="AC16" s="12" t="n">
         <v>21.131</v>
       </c>
-      <c r="AC16" s="12" t="n">
+      <c r="AD16" s="12" t="n">
         <v>24.232</v>
       </c>
-      <c r="AD16" s="12" t="n">
+      <c r="AE16" s="12" t="n">
         <v>24.3</v>
       </c>
-      <c r="AE16" s="12" t="n">
+      <c r="AF16" s="12" t="n">
         <v>45.351</v>
       </c>
-      <c r="AF16" s="12" t="n">
+      <c r="AG16" s="12" t="n">
         <v>44.898</v>
       </c>
-      <c r="AG16" s="12" t="n">
+      <c r="AH16" s="12" t="n">
         <v>42.498</v>
       </c>
-      <c r="AH16" s="12" t="n">
+      <c r="AI16" s="12" t="n">
         <v>33.856</v>
       </c>
-      <c r="AI16" s="12" t="n">
+      <c r="AJ16" s="12" t="n">
         <v>33.89</v>
       </c>
-      <c r="AJ16" s="12" t="n">
+      <c r="AK16" s="12" t="n">
         <v>33.025</v>
       </c>
-      <c r="AK16" s="12" t="n">
+      <c r="AL16" s="12" t="n">
         <v>30.71</v>
       </c>
-      <c r="AL16" s="12" t="n">
+      <c r="AM16" s="12" t="n">
         <v>24.181</v>
       </c>
-      <c r="AM16" s="12" t="n">
+      <c r="AN16" s="12" t="n">
         <v>26.259</v>
       </c>
-      <c r="AN16" s="12" t="n">
+      <c r="AO16" s="12" t="n">
         <v>26.264</v>
       </c>
-      <c r="AO16" s="12" t="n">
+      <c r="AP16" s="12" t="n">
         <v>24.94</v>
       </c>
     </row>
@@ -19480,63 +19538,64 @@
       <c r="P17" s="10" t="n"/>
       <c r="Q17" s="10" t="n"/>
       <c r="R17" s="10" t="n"/>
-      <c r="S17" s="10" t="n">
+      <c r="S17" s="10" t="n"/>
+      <c r="T17" s="10" t="n">
         <v>24.893</v>
       </c>
-      <c r="T17" s="10" t="n">
+      <c r="U17" s="10" t="n">
         <v>25.366</v>
       </c>
-      <c r="U17" s="10" t="n"/>
-      <c r="V17" s="10" t="n">
+      <c r="V17" s="10" t="n"/>
+      <c r="W17" s="10" t="n">
         <v>22.282</v>
       </c>
-      <c r="W17" s="10" t="n">
+      <c r="X17" s="10" t="n">
         <v>23.402</v>
       </c>
-      <c r="X17" s="10" t="n">
+      <c r="Y17" s="10" t="n">
         <v>22.819</v>
       </c>
-      <c r="Y17" s="10" t="n"/>
       <c r="Z17" s="10" t="n"/>
-      <c r="AA17" s="10" t="n">
+      <c r="AA17" s="10" t="n"/>
+      <c r="AB17" s="10" t="n">
         <v>23.11</v>
       </c>
-      <c r="AB17" s="10" t="n"/>
       <c r="AC17" s="10" t="n"/>
-      <c r="AD17" s="10" t="n">
+      <c r="AD17" s="10" t="n"/>
+      <c r="AE17" s="10" t="n">
         <v>24.3</v>
       </c>
-      <c r="AE17" s="10" t="n">
+      <c r="AF17" s="10" t="n">
         <v>43.051</v>
       </c>
-      <c r="AF17" s="10" t="n">
+      <c r="AG17" s="10" t="n">
         <v>42.82</v>
       </c>
-      <c r="AG17" s="10" t="n">
+      <c r="AH17" s="10" t="n">
         <v>40.705</v>
       </c>
-      <c r="AH17" s="10" t="n">
+      <c r="AI17" s="10" t="n">
         <v>32.478</v>
       </c>
-      <c r="AI17" s="10" t="n">
+      <c r="AJ17" s="10" t="n">
         <v>33.379</v>
       </c>
-      <c r="AJ17" s="10" t="n">
+      <c r="AK17" s="10" t="n">
         <v>31.434</v>
       </c>
-      <c r="AK17" s="10" t="n">
+      <c r="AL17" s="10" t="n">
         <v>30.32</v>
       </c>
-      <c r="AL17" s="10" t="n">
+      <c r="AM17" s="10" t="n">
         <v>23.847</v>
       </c>
-      <c r="AM17" s="10" t="n">
+      <c r="AN17" s="10" t="n">
         <v>25.928</v>
       </c>
-      <c r="AN17" s="10" t="n">
+      <c r="AO17" s="10" t="n">
         <v>25.259</v>
       </c>
-      <c r="AO17" s="10" t="n">
+      <c r="AP17" s="10" t="n">
         <v>25.475</v>
       </c>
     </row>
@@ -19587,63 +19646,64 @@
       <c r="P18" s="12" t="n"/>
       <c r="Q18" s="12" t="n"/>
       <c r="R18" s="12" t="n"/>
-      <c r="S18" s="12" t="n">
+      <c r="S18" s="12" t="n"/>
+      <c r="T18" s="12" t="n">
         <v>25.392</v>
       </c>
-      <c r="T18" s="12" t="n">
+      <c r="U18" s="12" t="n">
         <v>25.621</v>
       </c>
-      <c r="U18" s="12" t="n"/>
-      <c r="V18" s="12" t="n">
+      <c r="V18" s="12" t="n"/>
+      <c r="W18" s="12" t="n">
         <v>22.563</v>
       </c>
-      <c r="W18" s="12" t="n">
+      <c r="X18" s="12" t="n">
         <v>22.513</v>
       </c>
-      <c r="X18" s="12" t="n">
+      <c r="Y18" s="12" t="n">
         <v>22.724</v>
       </c>
-      <c r="Y18" s="12" t="n"/>
       <c r="Z18" s="12" t="n"/>
-      <c r="AA18" s="12" t="n">
+      <c r="AA18" s="12" t="n"/>
+      <c r="AB18" s="12" t="n">
         <v>23.431</v>
       </c>
-      <c r="AB18" s="12" t="n"/>
       <c r="AC18" s="12" t="n"/>
-      <c r="AD18" s="12" t="n">
+      <c r="AD18" s="12" t="n"/>
+      <c r="AE18" s="12" t="n">
         <v>23.834</v>
       </c>
-      <c r="AE18" s="12" t="n">
+      <c r="AF18" s="12" t="n">
         <v>45.853</v>
       </c>
-      <c r="AF18" s="12" t="n">
+      <c r="AG18" s="12" t="n">
         <v>45.695</v>
       </c>
-      <c r="AG18" s="12" t="n">
+      <c r="AH18" s="12" t="n">
         <v>43.503</v>
       </c>
-      <c r="AH18" s="12" t="n">
+      <c r="AI18" s="12" t="n">
         <v>35.124</v>
       </c>
-      <c r="AI18" s="12" t="n">
+      <c r="AJ18" s="12" t="n">
         <v>34.599</v>
       </c>
-      <c r="AJ18" s="12" t="n">
+      <c r="AK18" s="12" t="n">
         <v>32.926</v>
       </c>
-      <c r="AK18" s="12" t="n">
+      <c r="AL18" s="12" t="n">
         <v>32.212</v>
       </c>
-      <c r="AL18" s="12" t="n">
+      <c r="AM18" s="12" t="n">
         <v>24.348</v>
       </c>
-      <c r="AM18" s="12" t="n">
+      <c r="AN18" s="12" t="n">
         <v>26.424</v>
       </c>
-      <c r="AN18" s="12" t="n">
+      <c r="AO18" s="12" t="n">
         <v>25.046</v>
       </c>
-      <c r="AO18" s="12" t="n">
+      <c r="AP18" s="12" t="n">
         <v>26.209</v>
       </c>
     </row>
@@ -19694,63 +19754,64 @@
       <c r="P19" s="10" t="n"/>
       <c r="Q19" s="10" t="n"/>
       <c r="R19" s="10" t="n"/>
-      <c r="S19" s="10" t="n">
+      <c r="S19" s="10" t="n"/>
+      <c r="T19" s="10" t="n">
         <v>25.539</v>
       </c>
-      <c r="T19" s="10" t="n">
+      <c r="U19" s="10" t="n">
         <v>26.064</v>
       </c>
-      <c r="U19" s="10" t="n"/>
-      <c r="V19" s="10" t="n">
+      <c r="V19" s="10" t="n"/>
+      <c r="W19" s="10" t="n">
         <v>22.835</v>
       </c>
-      <c r="W19" s="10" t="n">
+      <c r="X19" s="10" t="n">
         <v>23.027</v>
       </c>
-      <c r="X19" s="10" t="n">
+      <c r="Y19" s="10" t="n">
         <v>22.819</v>
       </c>
-      <c r="Y19" s="10" t="n"/>
       <c r="Z19" s="10" t="n"/>
-      <c r="AA19" s="10" t="n">
+      <c r="AA19" s="10" t="n"/>
+      <c r="AB19" s="10" t="n">
         <v>23.256</v>
       </c>
-      <c r="AB19" s="10" t="n"/>
       <c r="AC19" s="10" t="n"/>
-      <c r="AD19" s="10" t="n">
+      <c r="AD19" s="10" t="n"/>
+      <c r="AE19" s="10" t="n">
         <v>24.012</v>
       </c>
-      <c r="AE19" s="10" t="n">
+      <c r="AF19" s="10" t="n">
         <v>45.048</v>
       </c>
-      <c r="AF19" s="10" t="n">
+      <c r="AG19" s="10" t="n">
         <v>44.939</v>
       </c>
-      <c r="AG19" s="10" t="n">
+      <c r="AH19" s="10" t="n">
         <v>42.925</v>
       </c>
-      <c r="AH19" s="10" t="n">
+      <c r="AI19" s="10" t="n">
         <v>34.361</v>
       </c>
-      <c r="AI19" s="10" t="n">
+      <c r="AJ19" s="10" t="n">
         <v>35.246</v>
       </c>
-      <c r="AJ19" s="10" t="n">
+      <c r="AK19" s="10" t="n">
         <v>33.424</v>
       </c>
-      <c r="AK19" s="10" t="n">
+      <c r="AL19" s="10" t="n">
         <v>31.277</v>
       </c>
-      <c r="AL19" s="10" t="n">
+      <c r="AM19" s="10" t="n">
         <v>24.496</v>
       </c>
-      <c r="AM19" s="10" t="n">
+      <c r="AN19" s="10" t="n">
         <v>26.571</v>
       </c>
-      <c r="AN19" s="10" t="n">
+      <c r="AO19" s="10" t="n">
         <v>26.186</v>
       </c>
-      <c r="AO19" s="10" t="n">
+      <c r="AP19" s="10" t="n">
         <v>25.94</v>
       </c>
     </row>
@@ -19801,63 +19862,64 @@
       <c r="P20" s="12" t="n"/>
       <c r="Q20" s="12" t="n"/>
       <c r="R20" s="12" t="n"/>
-      <c r="S20" s="12" t="n">
+      <c r="S20" s="12" t="n"/>
+      <c r="T20" s="12" t="n">
         <v>26.837</v>
       </c>
-      <c r="T20" s="12" t="n">
+      <c r="U20" s="12" t="n">
         <v>26.96</v>
       </c>
-      <c r="U20" s="12" t="n"/>
-      <c r="V20" s="12" t="n">
+      <c r="V20" s="12" t="n"/>
+      <c r="W20" s="12" t="n">
         <v>22.93</v>
       </c>
-      <c r="W20" s="12" t="n">
+      <c r="X20" s="12" t="n">
         <v>23.995</v>
       </c>
-      <c r="X20" s="12" t="n">
+      <c r="Y20" s="12" t="n">
         <v>23.324</v>
       </c>
-      <c r="Y20" s="12" t="n"/>
       <c r="Z20" s="12" t="n"/>
-      <c r="AA20" s="12" t="n">
+      <c r="AA20" s="12" t="n"/>
+      <c r="AB20" s="12" t="n">
         <v>23.65</v>
       </c>
-      <c r="AB20" s="12" t="n"/>
       <c r="AC20" s="12" t="n"/>
-      <c r="AD20" s="12" t="n">
+      <c r="AD20" s="12" t="n"/>
+      <c r="AE20" s="12" t="n">
         <v>20.587</v>
       </c>
-      <c r="AE20" s="12" t="n">
+      <c r="AF20" s="12" t="n">
         <v>52.736</v>
       </c>
-      <c r="AF20" s="12" t="n">
+      <c r="AG20" s="12" t="n">
         <v>52.189</v>
       </c>
-      <c r="AG20" s="12" t="n">
+      <c r="AH20" s="12" t="n">
         <v>49.898</v>
       </c>
-      <c r="AH20" s="12" t="n">
+      <c r="AI20" s="12" t="n">
         <v>38.256</v>
       </c>
-      <c r="AI20" s="12" t="n">
+      <c r="AJ20" s="12" t="n">
         <v>39.103</v>
       </c>
-      <c r="AJ20" s="12" t="n">
+      <c r="AK20" s="12" t="n">
         <v>36.84</v>
       </c>
-      <c r="AK20" s="12" t="n">
+      <c r="AL20" s="12" t="n">
         <v>35.122</v>
       </c>
-      <c r="AL20" s="12" t="n">
+      <c r="AM20" s="12" t="n">
         <v>25.801</v>
       </c>
-      <c r="AM20" s="12" t="n">
+      <c r="AN20" s="12" t="n">
         <v>27.861</v>
       </c>
-      <c r="AN20" s="12" t="n">
+      <c r="AO20" s="12" t="n">
         <v>27.222</v>
       </c>
-      <c r="AO20" s="12" t="n">
+      <c r="AP20" s="12" t="n">
         <v>26.693</v>
       </c>
     </row>
@@ -20103,8 +20165,12 @@
       <c r="Q3" s="10" t="n">
         <v>23.955</v>
       </c>
-      <c r="R3" s="10" t="n"/>
-      <c r="S3" s="10" t="n"/>
+      <c r="R3" s="10" t="n">
+        <v>23.036</v>
+      </c>
+      <c r="S3" s="10" t="n">
+        <v>23.213</v>
+      </c>
       <c r="T3" s="10" t="n"/>
       <c r="U3" s="10" t="n">
         <v>45.561</v>

</xml_diff>